<commit_message>
Publish July Monetary Rules Report release
</commit_message>
<xml_diff>
--- a/data/monetary-rules-dashboard-data.xlsx
+++ b/data/monetary-rules-dashboard-data.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5987cab6cf37472a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Rules" sheetId="2" r:id="Ra884aaba367a4e19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Series" sheetId="3" r:id="Re5c1b52cbe204c8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Data Vintages" sheetId="4" r:id="Rcb617721bdba4e6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="5" r:id="Re1fb800def8c427b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="6" r:id="R67e2903f15614e30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rfbef0e35c79c4ba0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Rules" sheetId="2" r:id="Rf38328b45aa44f3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Series" sheetId="3" r:id="R7f726cef30db4791"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Data Vintages" sheetId="4" r:id="R059152960d494bc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="5" r:id="Rf1d57b0027d34aca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="6" r:id="R5823b686d4cd4e9a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -731,7 +731,7 @@
         <x:v>Dashboard generated at</x:v>
       </x:c>
       <x:c r="B17" s="30" t="n">
-        <x:v>46221.09476467592</x:v>
+        <x:v>46232.01116609954</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5966,13 +5966,13 @@
         <x:v>Latest Monetary Rules Report</x:v>
       </x:c>
       <x:c r="B2" s="99" t="n">
-        <x:v>46189.5</x:v>
+        <x:v>46231.5</x:v>
       </x:c>
       <x:c r="C2" s="99" t="n">
-        <x:v>46220.5</x:v>
+        <x:v>46231.5</x:v>
       </x:c>
       <x:c r="D2" s="54" t="str">
-        <x:v>https://fedagenda.substack.com/p/monetary-rules-report-b79</x:v>
+        <x:v>https://fedagenda.substack.com/p/monetary-rules-report-31f</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -5983,7 +5983,7 @@
         <x:v>46143.5</x:v>
       </x:c>
       <x:c r="C3" s="100" t="n">
-        <x:v>46220.5</x:v>
+        <x:v>46231.5</x:v>
       </x:c>
       <x:c r="D3" s="64" t="str">
         <x:v>https://fedagenda.substack.com/p/monetary-neutrality-report-d5a</x:v>

</xml_diff>

<commit_message>
Publish July post-FOMC dashboard release
</commit_message>
<xml_diff>
--- a/data/monetary-rules-dashboard-data.xlsx
+++ b/data/monetary-rules-dashboard-data.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rfbef0e35c79c4ba0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Rules" sheetId="2" r:id="Rf38328b45aa44f3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Series" sheetId="3" r:id="R7f726cef30db4791"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Data Vintages" sheetId="4" r:id="R059152960d494bc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="5" r:id="Rf1d57b0027d34aca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="6" r:id="R5823b686d4cd4e9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rac0494b4c1fd46a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Rules" sheetId="2" r:id="R005d9a8fe7cc41a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Series" sheetId="3" r:id="R7647299f7dc24e95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Data Vintages" sheetId="4" r:id="R9583aa62df874095"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="5" r:id="R344cd74e8ea84ab4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="6" r:id="Rd13ad4e8266d4b2e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -655,7 +655,7 @@
       </x:c>
       <x:c r="B8" s="26" t="n">
         <x:f>MIN('Current Rules'!D2:D13)</x:f>
-        <x:v>3.7586733078965597</x:v>
+        <x:v>3.7304804422764946</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -664,7 +664,7 @@
       </x:c>
       <x:c r="B9" s="26" t="n">
         <x:f>MEDIAN('Current Rules'!D2:D13)</x:f>
-        <x:v>4.537288202256551</x:v>
+        <x:v>4.422751070492143</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -673,7 +673,7 @@
       </x:c>
       <x:c r="B10" s="26" t="n">
         <x:f>MAX('Current Rules'!D2:D13)</x:f>
-        <x:v>6.011806193233088</x:v>
+        <x:v>5.916990999508785</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -691,7 +691,7 @@
       </x:c>
       <x:c r="B12" s="27" t="n">
         <x:f>COUNTIF('Current Rules'!H2:H13,"Above range")</x:f>
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -699,7 +699,7 @@
         <x:v>Last Monetary Rules Report</x:v>
       </x:c>
       <x:c r="B13" s="28" t="n">
-        <x:v>46189.5</x:v>
+        <x:v>46231.5</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -715,7 +715,7 @@
         <x:v>Taylor data vintage</x:v>
       </x:c>
       <x:c r="B15" s="28" t="n">
-        <x:v>46157.5</x:v>
+        <x:v>46249.5</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -723,7 +723,7 @@
         <x:v>NGDP data vintage</x:v>
       </x:c>
       <x:c r="B16" s="28" t="n">
-        <x:v>46157.5</x:v>
+        <x:v>46249.5</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -731,7 +731,7 @@
         <x:v>Dashboard generated at</x:v>
       </x:c>
       <x:c r="B17" s="30" t="n">
-        <x:v>46232.01116609954</x:v>
+        <x:v>46236.69091612269</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -794,18 +794,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D2" s="52" t="n">
-        <x:v>6.011806193233088</x:v>
+        <x:v>5.916990999508785</x:v>
       </x:c>
       <x:c r="E2" s="52" t="n">
-        <x:v>5.91</x:v>
+        <x:v>6.011806193233087</x:v>
       </x:c>
       <x:c r="F2" s="53" t="n">
         <x:f>IF(E2="","",D2-E2)</x:f>
-        <x:v>0.10180619323308804</x:v>
+        <x:v>-0.09481519372430203</x:v>
       </x:c>
       <x:c r="G2" s="53" t="n">
         <x:f>D2-'Summary'!$B$5</x:f>
-        <x:v>2.3818061932330883</x:v>
+        <x:v>2.2869909995087854</x:v>
       </x:c>
       <x:c r="H2" s="54" t="str">
         <x:f>IF(D2&gt;'Summary'!$B$7,"Above range",IF(D2&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -823,18 +823,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D3" s="57" t="n">
-        <x:v>5.944152809026208</x:v>
+        <x:v>5.849337615301906</x:v>
       </x:c>
       <x:c r="E3" s="57" t="n">
-        <x:v>5.71</x:v>
+        <x:v>5.944152809026209</x:v>
       </x:c>
       <x:c r="F3" s="58" t="n">
         <x:f>IF(E3="","",D3-E3)</x:f>
-        <x:v>0.23415280902620772</x:v>
+        <x:v>-0.09481519372430292</x:v>
       </x:c>
       <x:c r="G3" s="58" t="n">
         <x:f>D3-'Summary'!$B$5</x:f>
-        <x:v>2.314152809026208</x:v>
+        <x:v>2.2193376153019058</x:v>
       </x:c>
       <x:c r="H3" s="59" t="str">
         <x:f>IF(D3&gt;'Summary'!$B$7,"Above range",IF(D3&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -852,18 +852,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D4" s="57" t="n">
+        <x:v>3.8952809354265363</x:v>
+      </x:c>
+      <x:c r="E4" s="57" t="n">
         <x:v>4.898230227602368</x:v>
-      </x:c>
-      <x:c r="E4" s="57" t="n">
-        <x:v>4.78</x:v>
       </x:c>
       <x:c r="F4" s="58" t="n">
         <x:f>IF(E4="","",D4-E4)</x:f>
-        <x:v>0.11823022760236768</x:v>
+        <x:v>-1.0029492921758316</x:v>
       </x:c>
       <x:c r="G4" s="58" t="n">
         <x:f>D4-'Summary'!$B$5</x:f>
-        <x:v>1.268230227602368</x:v>
+        <x:v>0.2652809354265364</x:v>
       </x:c>
       <x:c r="H4" s="59" t="str">
         <x:f>IF(D4&gt;'Summary'!$B$7,"Above range",IF(D4&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -881,18 +881,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D5" s="57" t="n">
-        <x:v>4.830576843395488</x:v>
+        <x:v>3.8276275512196563</x:v>
       </x:c>
       <x:c r="E5" s="57" t="n">
-        <x:v>4.58</x:v>
+        <x:v>4.830576843395487</x:v>
       </x:c>
       <x:c r="F5" s="58" t="n">
         <x:f>IF(E5="","",D5-E5)</x:f>
-        <x:v>0.25057684339548825</x:v>
+        <x:v>-1.0029492921758312</x:v>
       </x:c>
       <x:c r="G5" s="58" t="n">
         <x:f>D5-'Summary'!$B$5</x:f>
-        <x:v>1.2005768433954884</x:v>
+        <x:v>0.19762755121965636</x:v>
       </x:c>
       <x:c r="H5" s="59" t="str">
         <x:f>IF(D5&gt;'Summary'!$B$7,"Above range",IF(D5&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -910,18 +910,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D6" s="57" t="n">
-        <x:v>4.825903096616544</x:v>
+        <x:v>4.775162166421059</x:v>
       </x:c>
       <x:c r="E6" s="57" t="n">
-        <x:v>4.77</x:v>
+        <x:v>4.825903096616543</x:v>
       </x:c>
       <x:c r="F6" s="58" t="n">
         <x:f>IF(E6="","",D6-E6)</x:f>
-        <x:v>0.0559030966165448</x:v>
+        <x:v>-0.050740930195483536</x:v>
       </x:c>
       <x:c r="G6" s="58" t="n">
         <x:f>D6-'Summary'!$B$5</x:f>
-        <x:v>1.1959030966165445</x:v>
+        <x:v>1.1451621664210592</x:v>
       </x:c>
       <x:c r="H6" s="59" t="str">
         <x:f>IF(D6&gt;'Summary'!$B$7,"Above range",IF(D6&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -939,18 +939,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D7" s="57" t="n">
-        <x:v>4.792076404513104</x:v>
+        <x:v>4.741335474317619</x:v>
       </x:c>
       <x:c r="E7" s="57" t="n">
-        <x:v>4.67</x:v>
+        <x:v>4.792076404513105</x:v>
       </x:c>
       <x:c r="F7" s="58" t="n">
         <x:f>IF(E7="","",D7-E7)</x:f>
-        <x:v>0.12207640451310375</x:v>
+        <x:v>-0.05074093019548531</x:v>
       </x:c>
       <x:c r="G7" s="58" t="n">
         <x:f>D7-'Summary'!$B$5</x:f>
-        <x:v>1.1620764045131038</x:v>
+        <x:v>1.1113354743176194</x:v>
       </x:c>
       <x:c r="H7" s="59" t="str">
         <x:f>IF(D7&gt;'Summary'!$B$7,"Above range",IF(D7&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -968,18 +968,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D8" s="57" t="n">
-        <x:v>4.269115113801184</x:v>
+        <x:v>3.7643071343799344</x:v>
       </x:c>
       <x:c r="E8" s="57" t="n">
-        <x:v>4.21</x:v>
+        <x:v>4.269115113801183</x:v>
       </x:c>
       <x:c r="F8" s="58" t="n">
         <x:f>IF(E8="","",D8-E8)</x:f>
-        <x:v>0.05911511380118384</x:v>
+        <x:v>-0.5048079794212486</x:v>
       </x:c>
       <x:c r="G8" s="58" t="n">
         <x:f>D8-'Summary'!$B$5</x:f>
-        <x:v>0.6391151138011839</x:v>
+        <x:v>0.13430713437993447</x:v>
       </x:c>
       <x:c r="H8" s="59" t="str">
         <x:f>IF(D8&gt;'Summary'!$B$7,"Above range",IF(D8&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -997,22 +997,22 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D9" s="57" t="n">
+        <x:v>3.7304804422764946</x:v>
+      </x:c>
+      <x:c r="E9" s="57" t="n">
         <x:v>4.235288421697744</x:v>
-      </x:c>
-      <x:c r="E9" s="57" t="n">
-        <x:v>4.109999999999999</x:v>
       </x:c>
       <x:c r="F9" s="58" t="n">
         <x:f>IF(E9="","",D9-E9)</x:f>
-        <x:v>0.12528842169774457</x:v>
+        <x:v>-0.5048079794212494</x:v>
       </x:c>
       <x:c r="G9" s="58" t="n">
         <x:f>D9-'Summary'!$B$5</x:f>
-        <x:v>0.6052884216977441</x:v>
+        <x:v>0.10048044227649466</x:v>
       </x:c>
       <x:c r="H9" s="59" t="str">
         <x:f>IF(D9&gt;'Summary'!$B$7,"Above range",IF(D9&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
-        <x:v>Above range</x:v>
+        <x:v>Within range</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1026,18 +1026,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D10" s="57" t="n">
-        <x:v>4.2825</x:v>
+        <x:v>5.329166666666667</x:v>
       </x:c>
       <x:c r="E10" s="57" t="n">
-        <x:v>3.9600000000000004</x:v>
+        <x:v>4.282500000000001</x:v>
       </x:c>
       <x:c r="F10" s="58" t="n">
         <x:f>IF(E10="","",D10-E10)</x:f>
-        <x:v>0.32249999999999934</x:v>
+        <x:v>1.046666666666666</x:v>
       </x:c>
       <x:c r="G10" s="58" t="n">
         <x:f>D10-'Summary'!$B$5</x:f>
-        <x:v>0.6524999999999999</x:v>
+        <x:v>1.6991666666666667</x:v>
       </x:c>
       <x:c r="H10" s="59" t="str">
         <x:f>IF(D10&gt;'Summary'!$B$7,"Above range",IF(D10&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -1055,18 +1055,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D11" s="57" t="n">
+        <x:v>5.295339974563227</x:v>
+      </x:c>
+      <x:c r="E11" s="57" t="n">
         <x:v>4.24867330789656</x:v>
-      </x:c>
-      <x:c r="E11" s="57" t="n">
-        <x:v>3.8600000000000003</x:v>
       </x:c>
       <x:c r="F11" s="58" t="n">
         <x:f>IF(E11="","",D11-E11)</x:f>
-        <x:v>0.3886733078965596</x:v>
+        <x:v>1.0466666666666669</x:v>
       </x:c>
       <x:c r="G11" s="58" t="n">
         <x:f>D11-'Summary'!$B$5</x:f>
-        <x:v>0.61867330789656</x:v>
+        <x:v>1.665339974563227</x:v>
       </x:c>
       <x:c r="H11" s="59" t="str">
         <x:f>IF(D11&gt;'Summary'!$B$7,"Above range",IF(D11&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -1084,18 +1084,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D12" s="57" t="n">
+        <x:v>4.104166666666666</x:v>
+      </x:c>
+      <x:c r="E12" s="57" t="n">
         <x:v>3.7925</x:v>
-      </x:c>
-      <x:c r="E12" s="57" t="n">
-        <x:v>3.7900000000000005</x:v>
       </x:c>
       <x:c r="F12" s="58" t="n">
         <x:f>IF(E12="","",D12-E12)</x:f>
-        <x:v>0.0024999999999995026</x:v>
+        <x:v>0.3116666666666661</x:v>
       </x:c>
       <x:c r="G12" s="58" t="n">
         <x:f>D12-'Summary'!$B$5</x:f>
-        <x:v>0.1625000000000001</x:v>
+        <x:v>0.4741666666666662</x:v>
       </x:c>
       <x:c r="H12" s="59" t="str">
         <x:f>IF(D12&gt;'Summary'!$B$7,"Above range",IF(D12&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -1113,18 +1113,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D13" s="62" t="n">
-        <x:v>3.7586733078965597</x:v>
+        <x:v>4.070339974563226</x:v>
       </x:c>
       <x:c r="E13" s="62" t="n">
-        <x:v>3.6900000000000004</x:v>
+        <x:v>3.75867330789656</x:v>
       </x:c>
       <x:c r="F13" s="63" t="n">
         <x:f>IF(E13="","",D13-E13)</x:f>
-        <x:v>0.06867330789655934</x:v>
+        <x:v>0.3116666666666661</x:v>
       </x:c>
       <x:c r="G13" s="63" t="n">
         <x:f>D13-'Summary'!$B$5</x:f>
-        <x:v>0.12867330789655984</x:v>
+        <x:v>0.4403399745632264</x:v>
       </x:c>
       <x:c r="H13" s="64" t="str">
         <x:f>IF(D13&gt;'Summary'!$B$7,"Above range",IF(D13&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -2659,29 +2659,55 @@
       </x:c>
     </x:row>
     <x:row r="59">
-      <x:c r="A59" s="69" t="n">
+      <x:c r="A59" s="28" t="n">
         <x:v>46157.5</x:v>
       </x:c>
-      <x:c r="B59" s="70" t="n">
+      <x:c r="B59" s="26" t="n">
         <x:v>3.63</x:v>
       </x:c>
-      <x:c r="C59" s="70" t="n">
+      <x:c r="C59" s="26" t="n">
         <x:v>3.5</x:v>
       </x:c>
-      <x:c r="D59" s="70" t="n">
+      <x:c r="D59" s="26" t="n">
         <x:v>3.75</x:v>
       </x:c>
-      <x:c r="E59" s="70" t="n">
-        <x:v>5.944152809026208</x:v>
-      </x:c>
-      <x:c r="F59" s="70" t="n">
+      <x:c r="E59" s="26" t="n">
+        <x:v>5.9543631105515</x:v>
+      </x:c>
+      <x:c r="F59" s="26" t="n">
         <x:v>4.235288421697744</x:v>
       </x:c>
-      <x:c r="G59" s="70" t="n">
+      <x:c r="G59" s="26" t="n">
         <x:v>4.24867330789656</x:v>
       </x:c>
-      <x:c r="H59" s="70" t="n">
+      <x:c r="H59" s="26" t="n">
         <x:v>3.7586733078965597</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="69" t="n">
+        <x:v>46249.5</x:v>
+      </x:c>
+      <x:c r="B60" s="70" t="n">
+        <x:v>3.63</x:v>
+      </x:c>
+      <x:c r="C60" s="70" t="n">
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="D60" s="70" t="n">
+        <x:v>3.75</x:v>
+      </x:c>
+      <x:c r="E60" s="70" t="n">
+        <x:v>5.849337615301906</x:v>
+      </x:c>
+      <x:c r="F60" s="70" t="n">
+        <x:v>3.7304804422764946</x:v>
+      </x:c>
+      <x:c r="G60" s="70" t="n">
+        <x:v>5.295339974563227</x:v>
+      </x:c>
+      <x:c r="H60" s="70" t="n">
+        <x:v>4.070339974563226</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5612,53 +5638,103 @@
       </x:c>
     </x:row>
     <x:row r="59">
-      <x:c r="A59" s="81" t="n">
+      <x:c r="A59" s="79" t="n">
         <x:v>46157.5</x:v>
       </x:c>
-      <x:c r="B59" s="62" t="n">
+      <x:c r="B59" s="57" t="n">
         <x:v>3.63</x:v>
       </x:c>
-      <x:c r="C59" s="62" t="n">
+      <x:c r="C59" s="57" t="n">
         <x:v>3.5</x:v>
       </x:c>
-      <x:c r="D59" s="62" t="n">
+      <x:c r="D59" s="57" t="n">
         <x:v>3.75</x:v>
       </x:c>
-      <x:c r="E59" s="62" t="n">
-        <x:v>6.011806193233088</x:v>
-      </x:c>
-      <x:c r="F59" s="62" t="n">
-        <x:v>5.944152809026208</x:v>
-      </x:c>
-      <x:c r="G59" s="62" t="n">
+      <x:c r="E59" s="57" t="n">
+        <x:v>6.022016494758381</x:v>
+      </x:c>
+      <x:c r="F59" s="57" t="n">
+        <x:v>5.9543631105515</x:v>
+      </x:c>
+      <x:c r="G59" s="57" t="n">
         <x:v>4.898230227602368</x:v>
       </x:c>
-      <x:c r="H59" s="62" t="n">
+      <x:c r="H59" s="57" t="n">
         <x:v>4.830576843395488</x:v>
       </x:c>
-      <x:c r="I59" s="62" t="n">
-        <x:v>4.825903096616544</x:v>
-      </x:c>
-      <x:c r="J59" s="62" t="n">
-        <x:v>4.792076404513104</x:v>
-      </x:c>
-      <x:c r="K59" s="62" t="n">
+      <x:c r="I59" s="57" t="n">
+        <x:v>4.831008247379191</x:v>
+      </x:c>
+      <x:c r="J59" s="57" t="n">
+        <x:v>4.79718155527575</x:v>
+      </x:c>
+      <x:c r="K59" s="57" t="n">
         <x:v>4.269115113801184</x:v>
       </x:c>
-      <x:c r="L59" s="62" t="n">
+      <x:c r="L59" s="57" t="n">
         <x:v>4.235288421697744</x:v>
       </x:c>
-      <x:c r="M59" s="62" t="n">
+      <x:c r="M59" s="57" t="n">
         <x:v>4.2825</x:v>
       </x:c>
-      <x:c r="N59" s="62" t="n">
+      <x:c r="N59" s="57" t="n">
         <x:v>4.24867330789656</x:v>
       </x:c>
-      <x:c r="O59" s="62" t="n">
+      <x:c r="O59" s="57" t="n">
         <x:v>3.7925</x:v>
       </x:c>
-      <x:c r="P59" s="82" t="n">
+      <x:c r="P59" s="80" t="n">
         <x:v>3.7586733078965597</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="81" t="n">
+        <x:v>46249.5</x:v>
+      </x:c>
+      <x:c r="B60" s="62" t="n">
+        <x:v>3.63</x:v>
+      </x:c>
+      <x:c r="C60" s="62" t="n">
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="D60" s="62" t="n">
+        <x:v>3.75</x:v>
+      </x:c>
+      <x:c r="E60" s="62" t="n">
+        <x:v>5.916990999508785</x:v>
+      </x:c>
+      <x:c r="F60" s="62" t="n">
+        <x:v>5.849337615301906</x:v>
+      </x:c>
+      <x:c r="G60" s="62" t="n">
+        <x:v>3.8952809354265363</x:v>
+      </x:c>
+      <x:c r="H60" s="62" t="n">
+        <x:v>3.8276275512196563</x:v>
+      </x:c>
+      <x:c r="I60" s="62" t="n">
+        <x:v>4.775162166421059</x:v>
+      </x:c>
+      <x:c r="J60" s="62" t="n">
+        <x:v>4.741335474317619</x:v>
+      </x:c>
+      <x:c r="K60" s="62" t="n">
+        <x:v>3.7643071343799344</x:v>
+      </x:c>
+      <x:c r="L60" s="62" t="n">
+        <x:v>3.7304804422764946</x:v>
+      </x:c>
+      <x:c r="M60" s="62" t="n">
+        <x:v>5.329166666666667</x:v>
+      </x:c>
+      <x:c r="N60" s="62" t="n">
+        <x:v>5.295339974563227</x:v>
+      </x:c>
+      <x:c r="O60" s="62" t="n">
+        <x:v>4.104166666666666</x:v>
+      </x:c>
+      <x:c r="P60" s="82" t="n">
+        <x:v>4.070339974563226</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5722,7 +5798,7 @@
         <x:v>lagged_ffr</x:v>
       </x:c>
       <x:c r="D3" s="93" t="n">
-        <x:v>3.64</x:v>
+        <x:v>3.633333333333333</x:v>
       </x:c>
       <x:c r="E3" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -5790,7 +5866,7 @@
         <x:v>pce</x:v>
       </x:c>
       <x:c r="D7" s="93" t="n">
-        <x:v>3.838981906599837</x:v>
+        <x:v>3.757784004422304</x:v>
       </x:c>
       <x:c r="E7" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -5807,7 +5883,7 @@
         <x:v>pce_spf</x:v>
       </x:c>
       <x:c r="D8" s="93" t="n">
-        <x:v>3.09659792951269</x:v>
+        <x:v>2.409977295034138</x:v>
       </x:c>
       <x:c r="E8" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -5824,7 +5900,7 @@
         <x:v>unemp_gap</x:v>
       </x:c>
       <x:c r="D9" s="93" t="n">
-        <x:v>0.2566666666666659</x:v>
+        <x:v>0.3106299857506585</x:v>
       </x:c>
       <x:c r="E9" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -5841,7 +5917,7 @@
         <x:v>lagged_ffr</x:v>
       </x:c>
       <x:c r="D10" s="93" t="n">
-        <x:v>3.64</x:v>
+        <x:v>3.633333333333333</x:v>
       </x:c>
       <x:c r="E10" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -5875,7 +5951,7 @@
         <x:v>ngdp</x:v>
       </x:c>
       <x:c r="D12" s="93" t="n">
-        <x:v>5.8</x:v>
+        <x:v>7.9</x:v>
       </x:c>
       <x:c r="E12" s="94" t="str">
         <x:v>Bureau of Economic Analysis Nominal GDP — https://www.bea.gov/data/gdp/gross-domestic-product</x:v>
@@ -5892,10 +5968,10 @@
         <x:v>nominal_gap</x:v>
       </x:c>
       <x:c r="D13" s="93" t="n">
-        <x:v>0.82</x:v>
+        <x:v>1.45</x:v>
       </x:c>
       <x:c r="E13" s="94" t="str">
-        <x:v>Monetary Neutrality Report Nominal-spending gap — https://fedagenda.substack.com/p/monetary-neutrality-report-d5a</x:v>
+        <x:v>Monetary Neutrality Report Nominal-spending gap — https://fedagenda.substack.com/p/monetary-neutrality-report-9d2</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -5969,7 +6045,7 @@
         <x:v>46231.5</x:v>
       </x:c>
       <x:c r="C2" s="99" t="n">
-        <x:v>46231.5</x:v>
+        <x:v>46236.5</x:v>
       </x:c>
       <x:c r="D2" s="54" t="str">
         <x:v>https://fedagenda.substack.com/p/monetary-rules-report-31f</x:v>
@@ -5980,13 +6056,13 @@
         <x:v>Latest Monetary Neutrality Report</x:v>
       </x:c>
       <x:c r="B3" s="100" t="n">
-        <x:v>46143.5</x:v>
+        <x:v>46234.5</x:v>
       </x:c>
       <x:c r="C3" s="100" t="n">
-        <x:v>46231.5</x:v>
+        <x:v>46236.5</x:v>
       </x:c>
       <x:c r="D3" s="64" t="str">
-        <x:v>https://fedagenda.substack.com/p/monetary-neutrality-report-d5a</x:v>
+        <x:v>https://fedagenda.substack.com/p/monetary-neutrality-report-9d2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Publish August dashboard update
</commit_message>
<xml_diff>
--- a/data/monetary-rules-dashboard-data.xlsx
+++ b/data/monetary-rules-dashboard-data.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rac0494b4c1fd46a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Rules" sheetId="2" r:id="R005d9a8fe7cc41a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Series" sheetId="3" r:id="R7647299f7dc24e95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Data Vintages" sheetId="4" r:id="R9583aa62df874095"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="5" r:id="R344cd74e8ea84ab4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="6" r:id="Rd13ad4e8266d4b2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re608004f407a4eb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Rules" sheetId="2" r:id="R50f1966e2347443c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Series" sheetId="3" r:id="Rec1dc02f49a4406e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Data Vintages" sheetId="4" r:id="R26f0b938e1884efd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="5" r:id="R6f08276680214ebc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="6" r:id="R9d59b04eaf7547f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -655,7 +655,7 @@
       </x:c>
       <x:c r="B8" s="26" t="n">
         <x:f>MIN('Current Rules'!D2:D13)</x:f>
-        <x:v>3.7304804422764946</x:v>
+        <x:v>3.7695344057616342</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -664,7 +664,7 @@
       </x:c>
       <x:c r="B9" s="26" t="n">
         <x:f>MEDIAN('Current Rules'!D2:D13)</x:f>
-        <x:v>4.422751070492143</x:v>
+        <x:v>4.4421423023799385</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -673,7 +673,7 @@
       </x:c>
       <x:c r="B10" s="26" t="n">
         <x:f>MAX('Current Rules'!D2:D13)</x:f>
-        <x:v>5.916990999508785</x:v>
+        <x:v>5.994555927059969</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -691,7 +691,7 @@
       </x:c>
       <x:c r="B12" s="27" t="n">
         <x:f>COUNTIF('Current Rules'!H2:H13,"Above range")</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -731,7 +731,7 @@
         <x:v>Dashboard generated at</x:v>
       </x:c>
       <x:c r="B17" s="30" t="n">
-        <x:v>46236.69091612269</x:v>
+        <x:v>46246.84373957176</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -794,18 +794,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D2" s="52" t="n">
-        <x:v>5.916990999508785</x:v>
+        <x:v>5.994555927059969</x:v>
       </x:c>
       <x:c r="E2" s="52" t="n">
         <x:v>6.011806193233087</x:v>
       </x:c>
       <x:c r="F2" s="53" t="n">
         <x:f>IF(E2="","",D2-E2)</x:f>
-        <x:v>-0.09481519372430203</x:v>
+        <x:v>-0.01725026617311798</x:v>
       </x:c>
       <x:c r="G2" s="53" t="n">
         <x:f>D2-'Summary'!$B$5</x:f>
-        <x:v>2.2869909995087854</x:v>
+        <x:v>2.3645559270599694</x:v>
       </x:c>
       <x:c r="H2" s="54" t="str">
         <x:f>IF(D2&gt;'Summary'!$B$7,"Above range",IF(D2&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -823,18 +823,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D3" s="57" t="n">
-        <x:v>5.849337615301906</x:v>
+        <x:v>5.926902542853089</x:v>
       </x:c>
       <x:c r="E3" s="57" t="n">
         <x:v>5.944152809026209</x:v>
       </x:c>
       <x:c r="F3" s="58" t="n">
         <x:f>IF(E3="","",D3-E3)</x:f>
-        <x:v>-0.09481519372430292</x:v>
+        <x:v>-0.017250266173119755</x:v>
       </x:c>
       <x:c r="G3" s="58" t="n">
         <x:f>D3-'Summary'!$B$5</x:f>
-        <x:v>2.2193376153019058</x:v>
+        <x:v>2.296902542853089</x:v>
       </x:c>
       <x:c r="H3" s="59" t="str">
         <x:f>IF(D3&gt;'Summary'!$B$7,"Above range",IF(D3&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -852,18 +852,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D4" s="57" t="n">
-        <x:v>3.8952809354265363</x:v>
+        <x:v>3.973388862396815</x:v>
       </x:c>
       <x:c r="E4" s="57" t="n">
         <x:v>4.898230227602368</x:v>
       </x:c>
       <x:c r="F4" s="58" t="n">
         <x:f>IF(E4="","",D4-E4)</x:f>
-        <x:v>-1.0029492921758316</x:v>
+        <x:v>-0.9248413652055527</x:v>
       </x:c>
       <x:c r="G4" s="58" t="n">
         <x:f>D4-'Summary'!$B$5</x:f>
-        <x:v>0.2652809354265364</x:v>
+        <x:v>0.3433888623968153</x:v>
       </x:c>
       <x:c r="H4" s="59" t="str">
         <x:f>IF(D4&gt;'Summary'!$B$7,"Above range",IF(D4&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -881,18 +881,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D5" s="57" t="n">
-        <x:v>3.8276275512196563</x:v>
+        <x:v>3.9057354781899356</x:v>
       </x:c>
       <x:c r="E5" s="57" t="n">
         <x:v>4.830576843395487</x:v>
       </x:c>
       <x:c r="F5" s="58" t="n">
         <x:f>IF(E5="","",D5-E5)</x:f>
-        <x:v>-1.0029492921758312</x:v>
+        <x:v>-0.9248413652055518</x:v>
       </x:c>
       <x:c r="G5" s="58" t="n">
         <x:f>D5-'Summary'!$B$5</x:f>
-        <x:v>0.19762755121965636</x:v>
+        <x:v>0.2757354781899357</x:v>
       </x:c>
       <x:c r="H5" s="59" t="str">
         <x:f>IF(D5&gt;'Summary'!$B$7,"Above range",IF(D5&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -910,18 +910,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D6" s="57" t="n">
-        <x:v>4.775162166421059</x:v>
+        <x:v>4.8139446301966515</x:v>
       </x:c>
       <x:c r="E6" s="57" t="n">
         <x:v>4.825903096616543</x:v>
       </x:c>
       <x:c r="F6" s="58" t="n">
         <x:f>IF(E6="","",D6-E6)</x:f>
-        <x:v>-0.050740930195483536</x:v>
+        <x:v>-0.011958466419891067</x:v>
       </x:c>
       <x:c r="G6" s="58" t="n">
         <x:f>D6-'Summary'!$B$5</x:f>
-        <x:v>1.1451621664210592</x:v>
+        <x:v>1.1839446301966516</x:v>
       </x:c>
       <x:c r="H6" s="59" t="str">
         <x:f>IF(D6&gt;'Summary'!$B$7,"Above range",IF(D6&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -939,18 +939,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D7" s="57" t="n">
-        <x:v>4.741335474317619</x:v>
+        <x:v>4.780117938093211</x:v>
       </x:c>
       <x:c r="E7" s="57" t="n">
         <x:v>4.792076404513105</x:v>
       </x:c>
       <x:c r="F7" s="58" t="n">
         <x:f>IF(E7="","",D7-E7)</x:f>
-        <x:v>-0.05074093019548531</x:v>
+        <x:v>-0.011958466419893732</x:v>
       </x:c>
       <x:c r="G7" s="58" t="n">
         <x:f>D7-'Summary'!$B$5</x:f>
-        <x:v>1.1113354743176194</x:v>
+        <x:v>1.150117938093211</x:v>
       </x:c>
       <x:c r="H7" s="59" t="str">
         <x:f>IF(D7&gt;'Summary'!$B$7,"Above range",IF(D7&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -968,18 +968,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D8" s="57" t="n">
-        <x:v>3.7643071343799344</x:v>
+        <x:v>3.803361097865074</x:v>
       </x:c>
       <x:c r="E8" s="57" t="n">
         <x:v>4.269115113801183</x:v>
       </x:c>
       <x:c r="F8" s="58" t="n">
         <x:f>IF(E8="","",D8-E8)</x:f>
-        <x:v>-0.5048079794212486</x:v>
+        <x:v>-0.4657540159361089</x:v>
       </x:c>
       <x:c r="G8" s="58" t="n">
         <x:f>D8-'Summary'!$B$5</x:f>
-        <x:v>0.13430713437993447</x:v>
+        <x:v>0.17336109786507414</x:v>
       </x:c>
       <x:c r="H8" s="59" t="str">
         <x:f>IF(D8&gt;'Summary'!$B$7,"Above range",IF(D8&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -997,22 +997,22 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D9" s="57" t="n">
-        <x:v>3.7304804422764946</x:v>
+        <x:v>3.7695344057616342</x:v>
       </x:c>
       <x:c r="E9" s="57" t="n">
         <x:v>4.235288421697744</x:v>
       </x:c>
       <x:c r="F9" s="58" t="n">
         <x:f>IF(E9="","",D9-E9)</x:f>
-        <x:v>-0.5048079794212494</x:v>
+        <x:v>-0.46575401593610977</x:v>
       </x:c>
       <x:c r="G9" s="58" t="n">
         <x:f>D9-'Summary'!$B$5</x:f>
-        <x:v>0.10048044227649466</x:v>
+        <x:v>0.13953440576163434</x:v>
       </x:c>
       <x:c r="H9" s="59" t="str">
         <x:f>IF(D9&gt;'Summary'!$B$7,"Above range",IF(D9&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
-        <x:v>Within range</x:v>
+        <x:v>Above range</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2698,10 +2698,10 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="E60" s="70" t="n">
-        <x:v>5.849337615301906</x:v>
+        <x:v>5.926902542853089</x:v>
       </x:c>
       <x:c r="F60" s="70" t="n">
-        <x:v>3.7304804422764946</x:v>
+        <x:v>3.7695344057616342</x:v>
       </x:c>
       <x:c r="G60" s="70" t="n">
         <x:v>5.295339974563227</x:v>
@@ -5701,28 +5701,28 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="E60" s="62" t="n">
-        <x:v>5.916990999508785</x:v>
+        <x:v>5.994555927059969</x:v>
       </x:c>
       <x:c r="F60" s="62" t="n">
-        <x:v>5.849337615301906</x:v>
+        <x:v>5.926902542853089</x:v>
       </x:c>
       <x:c r="G60" s="62" t="n">
-        <x:v>3.8952809354265363</x:v>
+        <x:v>3.973388862396815</x:v>
       </x:c>
       <x:c r="H60" s="62" t="n">
-        <x:v>3.8276275512196563</x:v>
+        <x:v>3.9057354781899356</x:v>
       </x:c>
       <x:c r="I60" s="62" t="n">
-        <x:v>4.775162166421059</x:v>
+        <x:v>4.8139446301966515</x:v>
       </x:c>
       <x:c r="J60" s="62" t="n">
-        <x:v>4.741335474317619</x:v>
+        <x:v>4.780117938093211</x:v>
       </x:c>
       <x:c r="K60" s="62" t="n">
-        <x:v>3.7643071343799344</x:v>
+        <x:v>3.803361097865074</x:v>
       </x:c>
       <x:c r="L60" s="62" t="n">
-        <x:v>3.7304804422764946</x:v>
+        <x:v>3.7695344057616342</x:v>
       </x:c>
       <x:c r="M60" s="62" t="n">
         <x:v>5.329166666666667</x:v>
@@ -5866,7 +5866,7 @@
         <x:v>pce</x:v>
       </x:c>
       <x:c r="D7" s="93" t="n">
-        <x:v>3.757784004422304</x:v>
+        <x:v>3.729916301013048</x:v>
       </x:c>
       <x:c r="E7" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -5883,7 +5883,7 @@
         <x:v>pce_spf</x:v>
       </x:c>
       <x:c r="D8" s="93" t="n">
-        <x:v>2.409977295034138</x:v>
+        <x:v>2.382471591237612</x:v>
       </x:c>
       <x:c r="E8" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -5900,7 +5900,7 @@
         <x:v>unemp_gap</x:v>
       </x:c>
       <x:c r="D9" s="93" t="n">
-        <x:v>0.3106299857506585</x:v>
+        <x:v>0.5493629510807949</x:v>
       </x:c>
       <x:c r="E9" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -6045,7 +6045,7 @@
         <x:v>46231.5</x:v>
       </x:c>
       <x:c r="C2" s="99" t="n">
-        <x:v>46236.5</x:v>
+        <x:v>46246.5</x:v>
       </x:c>
       <x:c r="D2" s="54" t="str">
         <x:v>https://fedagenda.substack.com/p/monetary-rules-report-31f</x:v>
@@ -6059,7 +6059,7 @@
         <x:v>46234.5</x:v>
       </x:c>
       <x:c r="C3" s="100" t="n">
-        <x:v>46236.5</x:v>
+        <x:v>46246.5</x:v>
       </x:c>
       <x:c r="D3" s="64" t="str">
         <x:v>https://fedagenda.substack.com/p/monetary-neutrality-report-9d2</x:v>

</xml_diff>

<commit_message>
Publish dashboard release 2026-08-issue-7
</commit_message>
<xml_diff>
--- a/data/monetary-rules-dashboard-data.xlsx
+++ b/data/monetary-rules-dashboard-data.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re608004f407a4eb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Rules" sheetId="2" r:id="R50f1966e2347443c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Series" sheetId="3" r:id="Rec1dc02f49a4406e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Data Vintages" sheetId="4" r:id="R26f0b938e1884efd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="5" r:id="R6f08276680214ebc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="6" r:id="R9d59b04eaf7547f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R580cb2f0dadf4630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Rules" sheetId="2" r:id="R0bcc2abe82a64b6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Series" sheetId="3" r:id="Rb69cd8f98cfb4002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Data Vintages" sheetId="4" r:id="R3e1d638f896647c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="5" r:id="Re0c80360d31a420c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="6" r:id="Re6590c021ec44d62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -655,7 +655,7 @@
       </x:c>
       <x:c r="B8" s="26" t="n">
         <x:f>MIN('Current Rules'!D2:D13)</x:f>
-        <x:v>3.7695344057616342</x:v>
+        <x:v>3.7871275818753105</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -664,7 +664,7 @@
       </x:c>
       <x:c r="B9" s="26" t="n">
         <x:f>MEDIAN('Current Rules'!D2:D13)</x:f>
-        <x:v>4.4421423023799385</x:v>
+        <x:v>4.449417282547672</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -673,7 +673,7 @@
       </x:c>
       <x:c r="B10" s="26" t="n">
         <x:f>MAX('Current Rules'!D2:D13)</x:f>
-        <x:v>5.994555927059969</x:v>
+        <x:v>6.023655847730904</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -731,7 +731,7 @@
         <x:v>Dashboard generated at</x:v>
       </x:c>
       <x:c r="B17" s="30" t="n">
-        <x:v>46246.84373957176</x:v>
+        <x:v>46261.11469394676</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -794,18 +794,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D2" s="52" t="n">
-        <x:v>5.994555927059969</x:v>
+        <x:v>6.023655847730904</x:v>
       </x:c>
       <x:c r="E2" s="52" t="n">
         <x:v>6.011806193233087</x:v>
       </x:c>
       <x:c r="F2" s="53" t="n">
         <x:f>IF(E2="","",D2-E2)</x:f>
-        <x:v>-0.01725026617311798</x:v>
+        <x:v>0.011849654497816609</x:v>
       </x:c>
       <x:c r="G2" s="53" t="n">
         <x:f>D2-'Summary'!$B$5</x:f>
-        <x:v>2.3645559270599694</x:v>
+        <x:v>2.393655847730904</x:v>
       </x:c>
       <x:c r="H2" s="54" t="str">
         <x:f>IF(D2&gt;'Summary'!$B$7,"Above range",IF(D2&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -823,18 +823,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D3" s="57" t="n">
-        <x:v>5.926902542853089</x:v>
+        <x:v>5.956002463524023</x:v>
       </x:c>
       <x:c r="E3" s="57" t="n">
         <x:v>5.944152809026209</x:v>
       </x:c>
       <x:c r="F3" s="58" t="n">
         <x:f>IF(E3="","",D3-E3)</x:f>
-        <x:v>-0.017250266173119755</x:v>
+        <x:v>0.011849654497814832</x:v>
       </x:c>
       <x:c r="G3" s="58" t="n">
         <x:f>D3-'Summary'!$B$5</x:f>
-        <x:v>2.296902542853089</x:v>
+        <x:v>2.3260024635240235</x:v>
       </x:c>
       <x:c r="H3" s="59" t="str">
         <x:f>IF(D3&gt;'Summary'!$B$7,"Above range",IF(D3&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -852,18 +852,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D4" s="57" t="n">
-        <x:v>3.973388862396815</x:v>
+        <x:v>4.008575214624168</x:v>
       </x:c>
       <x:c r="E4" s="57" t="n">
         <x:v>4.898230227602368</x:v>
       </x:c>
       <x:c r="F4" s="58" t="n">
         <x:f>IF(E4="","",D4-E4)</x:f>
-        <x:v>-0.9248413652055527</x:v>
+        <x:v>-0.8896550129782002</x:v>
       </x:c>
       <x:c r="G4" s="58" t="n">
         <x:f>D4-'Summary'!$B$5</x:f>
-        <x:v>0.3433888623968153</x:v>
+        <x:v>0.3785752146241679</x:v>
       </x:c>
       <x:c r="H4" s="59" t="str">
         <x:f>IF(D4&gt;'Summary'!$B$7,"Above range",IF(D4&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -881,18 +881,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D5" s="57" t="n">
-        <x:v>3.9057354781899356</x:v>
+        <x:v>3.9409218304172877</x:v>
       </x:c>
       <x:c r="E5" s="57" t="n">
         <x:v>4.830576843395487</x:v>
       </x:c>
       <x:c r="F5" s="58" t="n">
         <x:f>IF(E5="","",D5-E5)</x:f>
-        <x:v>-0.9248413652055518</x:v>
+        <x:v>-0.8896550129781997</x:v>
       </x:c>
       <x:c r="G5" s="58" t="n">
         <x:f>D5-'Summary'!$B$5</x:f>
-        <x:v>0.2757354781899357</x:v>
+        <x:v>0.3109218304172878</x:v>
       </x:c>
       <x:c r="H5" s="59" t="str">
         <x:f>IF(D5&gt;'Summary'!$B$7,"Above range",IF(D5&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -910,18 +910,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D6" s="57" t="n">
-        <x:v>4.8139446301966515</x:v>
+        <x:v>4.828494590532118</x:v>
       </x:c>
       <x:c r="E6" s="57" t="n">
         <x:v>4.825903096616543</x:v>
       </x:c>
       <x:c r="F6" s="58" t="n">
         <x:f>IF(E6="","",D6-E6)</x:f>
-        <x:v>-0.011958466419891067</x:v>
+        <x:v>0.002591493915575782</x:v>
       </x:c>
       <x:c r="G6" s="58" t="n">
         <x:f>D6-'Summary'!$B$5</x:f>
-        <x:v>1.1839446301966516</x:v>
+        <x:v>1.1984945905321185</x:v>
       </x:c>
       <x:c r="H6" s="59" t="str">
         <x:f>IF(D6&gt;'Summary'!$B$7,"Above range",IF(D6&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -939,18 +939,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D7" s="57" t="n">
-        <x:v>4.780117938093211</x:v>
+        <x:v>4.794667898428678</x:v>
       </x:c>
       <x:c r="E7" s="57" t="n">
         <x:v>4.792076404513105</x:v>
       </x:c>
       <x:c r="F7" s="58" t="n">
         <x:f>IF(E7="","",D7-E7)</x:f>
-        <x:v>-0.011958466419893732</x:v>
+        <x:v>0.0025914939155731176</x:v>
       </x:c>
       <x:c r="G7" s="58" t="n">
         <x:f>D7-'Summary'!$B$5</x:f>
-        <x:v>1.150117938093211</x:v>
+        <x:v>1.1646678984286778</x:v>
       </x:c>
       <x:c r="H7" s="59" t="str">
         <x:f>IF(D7&gt;'Summary'!$B$7,"Above range",IF(D7&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -968,18 +968,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D8" s="57" t="n">
-        <x:v>3.803361097865074</x:v>
+        <x:v>3.8209542739787503</x:v>
       </x:c>
       <x:c r="E8" s="57" t="n">
         <x:v>4.269115113801183</x:v>
       </x:c>
       <x:c r="F8" s="58" t="n">
         <x:f>IF(E8="","",D8-E8)</x:f>
-        <x:v>-0.4657540159361089</x:v>
+        <x:v>-0.4481608398224326</x:v>
       </x:c>
       <x:c r="G8" s="58" t="n">
         <x:f>D8-'Summary'!$B$5</x:f>
-        <x:v>0.17336109786507414</x:v>
+        <x:v>0.19095427397875042</x:v>
       </x:c>
       <x:c r="H8" s="59" t="str">
         <x:f>IF(D8&gt;'Summary'!$B$7,"Above range",IF(D8&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -997,18 +997,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D9" s="57" t="n">
-        <x:v>3.7695344057616342</x:v>
+        <x:v>3.7871275818753105</x:v>
       </x:c>
       <x:c r="E9" s="57" t="n">
         <x:v>4.235288421697744</x:v>
       </x:c>
       <x:c r="F9" s="58" t="n">
         <x:f>IF(E9="","",D9-E9)</x:f>
-        <x:v>-0.46575401593610977</x:v>
+        <x:v>-0.4481608398224335</x:v>
       </x:c>
       <x:c r="G9" s="58" t="n">
         <x:f>D9-'Summary'!$B$5</x:f>
-        <x:v>0.13953440576163434</x:v>
+        <x:v>0.15712758187531062</x:v>
       </x:c>
       <x:c r="H9" s="59" t="str">
         <x:f>IF(D9&gt;'Summary'!$B$7,"Above range",IF(D9&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -1026,18 +1026,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D10" s="57" t="n">
-        <x:v>5.329166666666667</x:v>
+        <x:v>5.379166666666666</x:v>
       </x:c>
       <x:c r="E10" s="57" t="n">
         <x:v>4.282500000000001</x:v>
       </x:c>
       <x:c r="F10" s="58" t="n">
         <x:f>IF(E10="","",D10-E10)</x:f>
-        <x:v>1.046666666666666</x:v>
+        <x:v>1.0966666666666658</x:v>
       </x:c>
       <x:c r="G10" s="58" t="n">
         <x:f>D10-'Summary'!$B$5</x:f>
-        <x:v>1.6991666666666667</x:v>
+        <x:v>1.7491666666666665</x:v>
       </x:c>
       <x:c r="H10" s="59" t="str">
         <x:f>IF(D10&gt;'Summary'!$B$7,"Above range",IF(D10&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -1055,18 +1055,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D11" s="57" t="n">
-        <x:v>5.295339974563227</x:v>
+        <x:v>5.345339974563227</x:v>
       </x:c>
       <x:c r="E11" s="57" t="n">
         <x:v>4.24867330789656</x:v>
       </x:c>
       <x:c r="F11" s="58" t="n">
         <x:f>IF(E11="","",D11-E11)</x:f>
-        <x:v>1.0466666666666669</x:v>
+        <x:v>1.0966666666666667</x:v>
       </x:c>
       <x:c r="G11" s="58" t="n">
         <x:f>D11-'Summary'!$B$5</x:f>
-        <x:v>1.665339974563227</x:v>
+        <x:v>1.7153399745632267</x:v>
       </x:c>
       <x:c r="H11" s="59" t="str">
         <x:f>IF(D11&gt;'Summary'!$B$7,"Above range",IF(D11&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -2672,7 +2672,7 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="E59" s="26" t="n">
-        <x:v>5.9543631105515</x:v>
+        <x:v>6.000635970135097</x:v>
       </x:c>
       <x:c r="F59" s="26" t="n">
         <x:v>4.235288421697744</x:v>
@@ -2698,13 +2698,13 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="E60" s="70" t="n">
-        <x:v>5.926902542853089</x:v>
+        <x:v>5.956002463524023</x:v>
       </x:c>
       <x:c r="F60" s="70" t="n">
-        <x:v>3.7695344057616342</x:v>
+        <x:v>3.7871275818753105</x:v>
       </x:c>
       <x:c r="G60" s="70" t="n">
-        <x:v>5.295339974563227</x:v>
+        <x:v>5.345339974563227</x:v>
       </x:c>
       <x:c r="H60" s="70" t="n">
         <x:v>4.070339974563226</x:v>
@@ -5651,10 +5651,10 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="E59" s="57" t="n">
-        <x:v>6.022016494758381</x:v>
+        <x:v>6.068289354341977</x:v>
       </x:c>
       <x:c r="F59" s="57" t="n">
-        <x:v>5.9543631105515</x:v>
+        <x:v>6.000635970135097</x:v>
       </x:c>
       <x:c r="G59" s="57" t="n">
         <x:v>4.898230227602368</x:v>
@@ -5663,10 +5663,10 @@
         <x:v>4.830576843395488</x:v>
       </x:c>
       <x:c r="I59" s="57" t="n">
-        <x:v>4.831008247379191</x:v>
+        <x:v>4.854144677170988</x:v>
       </x:c>
       <x:c r="J59" s="57" t="n">
-        <x:v>4.79718155527575</x:v>
+        <x:v>4.820317985067549</x:v>
       </x:c>
       <x:c r="K59" s="57" t="n">
         <x:v>4.269115113801184</x:v>
@@ -5701,34 +5701,34 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="E60" s="62" t="n">
-        <x:v>5.994555927059969</x:v>
+        <x:v>6.023655847730904</x:v>
       </x:c>
       <x:c r="F60" s="62" t="n">
-        <x:v>5.926902542853089</x:v>
+        <x:v>5.956002463524023</x:v>
       </x:c>
       <x:c r="G60" s="62" t="n">
-        <x:v>3.973388862396815</x:v>
+        <x:v>4.008575214624168</x:v>
       </x:c>
       <x:c r="H60" s="62" t="n">
-        <x:v>3.9057354781899356</x:v>
+        <x:v>3.9409218304172877</x:v>
       </x:c>
       <x:c r="I60" s="62" t="n">
-        <x:v>4.8139446301966515</x:v>
+        <x:v>4.828494590532118</x:v>
       </x:c>
       <x:c r="J60" s="62" t="n">
-        <x:v>4.780117938093211</x:v>
+        <x:v>4.794667898428678</x:v>
       </x:c>
       <x:c r="K60" s="62" t="n">
-        <x:v>3.803361097865074</x:v>
+        <x:v>3.8209542739787503</x:v>
       </x:c>
       <x:c r="L60" s="62" t="n">
-        <x:v>3.7695344057616342</x:v>
+        <x:v>3.7871275818753105</x:v>
       </x:c>
       <x:c r="M60" s="62" t="n">
-        <x:v>5.329166666666667</x:v>
+        <x:v>5.379166666666666</x:v>
       </x:c>
       <x:c r="N60" s="62" t="n">
-        <x:v>5.295339974563227</x:v>
+        <x:v>5.345339974563227</x:v>
       </x:c>
       <x:c r="O60" s="62" t="n">
         <x:v>4.104166666666666</x:v>
@@ -5866,7 +5866,7 @@
         <x:v>pce</x:v>
       </x:c>
       <x:c r="D7" s="93" t="n">
-        <x:v>3.729916301013048</x:v>
+        <x:v>3.768335221498953</x:v>
       </x:c>
       <x:c r="E7" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -5883,7 +5883,7 @@
         <x:v>pce_spf</x:v>
       </x:c>
       <x:c r="D8" s="93" t="n">
-        <x:v>2.382471591237612</x:v>
+        <x:v>2.424948132761129</x:v>
       </x:c>
       <x:c r="E8" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -5900,7 +5900,7 @@
         <x:v>unemp_gap</x:v>
       </x:c>
       <x:c r="D9" s="93" t="n">
-        <x:v>0.5493629510807949</x:v>
+        <x:v>0.492306030964949</x:v>
       </x:c>
       <x:c r="E9" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -5951,7 +5951,7 @@
         <x:v>ngdp</x:v>
       </x:c>
       <x:c r="D12" s="93" t="n">
-        <x:v>7.9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E12" s="94" t="str">
         <x:v>Bureau of Economic Analysis Nominal GDP — https://www.bea.gov/data/gdp/gross-domestic-product</x:v>
@@ -6045,7 +6045,7 @@
         <x:v>46231.5</x:v>
       </x:c>
       <x:c r="C2" s="99" t="n">
-        <x:v>46246.5</x:v>
+        <x:v>46260.5</x:v>
       </x:c>
       <x:c r="D2" s="54" t="str">
         <x:v>https://fedagenda.substack.com/p/monetary-rules-report-31f</x:v>
@@ -6059,7 +6059,7 @@
         <x:v>46234.5</x:v>
       </x:c>
       <x:c r="C3" s="100" t="n">
-        <x:v>46246.5</x:v>
+        <x:v>46260.5</x:v>
       </x:c>
       <x:c r="D3" s="64" t="str">
         <x:v>https://fedagenda.substack.com/p/monetary-neutrality-report-9d2</x:v>

</xml_diff>

<commit_message>
Publish dashboard release 2026-09-issue-12
</commit_message>
<xml_diff>
--- a/data/monetary-rules-dashboard-data.xlsx
+++ b/data/monetary-rules-dashboard-data.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R580cb2f0dadf4630"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Rules" sheetId="2" r:id="R0bcc2abe82a64b6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Series" sheetId="3" r:id="Rb69cd8f98cfb4002"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Data Vintages" sheetId="4" r:id="R3e1d638f896647c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="5" r:id="Re0c80360d31a420c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="6" r:id="Re6590c021ec44d62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rac880583f4c84640"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Rules" sheetId="2" r:id="R4733a24713e3453f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Series" sheetId="3" r:id="R39fb2bba594e494b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Data Vintages" sheetId="4" r:id="R08ff6aacfaf04e18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="5" r:id="Radee14c6b0da4541"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="6" r:id="Rc509c566859f4ccb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -638,7 +638,7 @@
         <x:v>Target range lower bound</x:v>
       </x:c>
       <x:c r="B6" s="26" t="n">
-        <x:v>3.5</x:v>
+        <x:v>3.75</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -646,7 +646,7 @@
         <x:v>Target range upper bound</x:v>
       </x:c>
       <x:c r="B7" s="26" t="n">
-        <x:v>3.75</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -655,7 +655,7 @@
       </x:c>
       <x:c r="B8" s="26" t="n">
         <x:f>MIN('Current Rules'!D2:D13)</x:f>
-        <x:v>3.7871275818753105</x:v>
+        <x:v>3.7700675133562607</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -664,7 +664,7 @@
       </x:c>
       <x:c r="B9" s="26" t="n">
         <x:f>MEDIAN('Current Rules'!D2:D13)</x:f>
-        <x:v>4.449417282547672</x:v>
+        <x:v>4.470761793199724</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -673,7 +673,7 @@
       </x:c>
       <x:c r="B10" s="26" t="n">
         <x:f>MAX('Current Rules'!D2:D13)</x:f>
-        <x:v>6.023655847730904</x:v>
+        <x:v>6.157732147628201</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -691,7 +691,7 @@
       </x:c>
       <x:c r="B12" s="27" t="n">
         <x:f>COUNTIF('Current Rules'!H2:H13,"Above range")</x:f>
-        <x:v>12</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -731,7 +731,7 @@
         <x:v>Dashboard generated at</x:v>
       </x:c>
       <x:c r="B17" s="30" t="n">
-        <x:v>46261.11469394676</x:v>
+        <x:v>46282.10877106481</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -794,18 +794,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D2" s="52" t="n">
-        <x:v>6.023655847730904</x:v>
+        <x:v>6.157732147628201</x:v>
       </x:c>
       <x:c r="E2" s="52" t="n">
         <x:v>6.011806193233087</x:v>
       </x:c>
       <x:c r="F2" s="53" t="n">
         <x:f>IF(E2="","",D2-E2)</x:f>
-        <x:v>0.011849654497816609</x:v>
+        <x:v>0.14592595439511413</x:v>
       </x:c>
       <x:c r="G2" s="53" t="n">
         <x:f>D2-'Summary'!$B$5</x:f>
-        <x:v>2.393655847730904</x:v>
+        <x:v>2.5277321476282015</x:v>
       </x:c>
       <x:c r="H2" s="54" t="str">
         <x:f>IF(D2&gt;'Summary'!$B$7,"Above range",IF(D2&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -823,18 +823,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D3" s="57" t="n">
-        <x:v>5.956002463524023</x:v>
+        <x:v>5.978880506132231</x:v>
       </x:c>
       <x:c r="E3" s="57" t="n">
         <x:v>5.944152809026209</x:v>
       </x:c>
       <x:c r="F3" s="58" t="n">
         <x:f>IF(E3="","",D3-E3)</x:f>
-        <x:v>0.011849654497814832</x:v>
+        <x:v>0.03472769710602286</x:v>
       </x:c>
       <x:c r="G3" s="58" t="n">
         <x:f>D3-'Summary'!$B$5</x:f>
-        <x:v>2.3260024635240235</x:v>
+        <x:v>2.3488805061322315</x:v>
       </x:c>
       <x:c r="H3" s="59" t="str">
         <x:f>IF(D3&gt;'Summary'!$B$7,"Above range",IF(D3&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -852,18 +852,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D4" s="57" t="n">
-        <x:v>4.008575214624168</x:v>
+        <x:v>4.0856533348751585</x:v>
       </x:c>
       <x:c r="E4" s="57" t="n">
         <x:v>4.898230227602368</x:v>
       </x:c>
       <x:c r="F4" s="58" t="n">
         <x:f>IF(E4="","",D4-E4)</x:f>
-        <x:v>-0.8896550129782002</x:v>
+        <x:v>-0.8125768927272095</x:v>
       </x:c>
       <x:c r="G4" s="58" t="n">
         <x:f>D4-'Summary'!$B$5</x:f>
-        <x:v>0.3785752146241679</x:v>
+        <x:v>0.4556533348751586</x:v>
       </x:c>
       <x:c r="H4" s="59" t="str">
         <x:f>IF(D4&gt;'Summary'!$B$7,"Above range",IF(D4&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -881,22 +881,22 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D5" s="57" t="n">
-        <x:v>3.9409218304172877</x:v>
+        <x:v>3.9068016933791885</x:v>
       </x:c>
       <x:c r="E5" s="57" t="n">
         <x:v>4.830576843395487</x:v>
       </x:c>
       <x:c r="F5" s="58" t="n">
         <x:f>IF(E5="","",D5-E5)</x:f>
-        <x:v>-0.8896550129781997</x:v>
+        <x:v>-0.923775150016299</x:v>
       </x:c>
       <x:c r="G5" s="58" t="n">
         <x:f>D5-'Summary'!$B$5</x:f>
-        <x:v>0.3109218304172878</x:v>
+        <x:v>0.2768016933791886</x:v>
       </x:c>
       <x:c r="H5" s="59" t="str">
         <x:f>IF(D5&gt;'Summary'!$B$7,"Above range",IF(D5&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
-        <x:v>Above range</x:v>
+        <x:v>Within range</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -910,18 +910,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D6" s="57" t="n">
-        <x:v>4.828494590532118</x:v>
+        <x:v>4.895532740480768</x:v>
       </x:c>
       <x:c r="E6" s="57" t="n">
         <x:v>4.825903096616543</x:v>
       </x:c>
       <x:c r="F6" s="58" t="n">
         <x:f>IF(E6="","",D6-E6)</x:f>
-        <x:v>0.002591493915575782</x:v>
+        <x:v>0.06962964386422499</x:v>
       </x:c>
       <x:c r="G6" s="58" t="n">
         <x:f>D6-'Summary'!$B$5</x:f>
-        <x:v>1.1984945905321185</x:v>
+        <x:v>1.2655327404807677</x:v>
       </x:c>
       <x:c r="H6" s="59" t="str">
         <x:f>IF(D6&gt;'Summary'!$B$7,"Above range",IF(D6&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -939,18 +939,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D7" s="57" t="n">
-        <x:v>4.794667898428678</x:v>
+        <x:v>4.806106919732782</x:v>
       </x:c>
       <x:c r="E7" s="57" t="n">
         <x:v>4.792076404513105</x:v>
       </x:c>
       <x:c r="F7" s="58" t="n">
         <x:f>IF(E7="","",D7-E7)</x:f>
-        <x:v>0.0025914939155731176</x:v>
+        <x:v>0.014030515219677575</x:v>
       </x:c>
       <x:c r="G7" s="58" t="n">
         <x:f>D7-'Summary'!$B$5</x:f>
-        <x:v>1.1646678984286778</x:v>
+        <x:v>1.1761069197327823</x:v>
       </x:c>
       <x:c r="H7" s="59" t="str">
         <x:f>IF(D7&gt;'Summary'!$B$7,"Above range",IF(D7&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -968,22 +968,22 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D8" s="57" t="n">
-        <x:v>3.8209542739787503</x:v>
+        <x:v>3.8594933341042457</x:v>
       </x:c>
       <x:c r="E8" s="57" t="n">
         <x:v>4.269115113801183</x:v>
       </x:c>
       <x:c r="F8" s="58" t="n">
         <x:f>IF(E8="","",D8-E8)</x:f>
-        <x:v>-0.4481608398224326</x:v>
+        <x:v>-0.40962177969693725</x:v>
       </x:c>
       <x:c r="G8" s="58" t="n">
         <x:f>D8-'Summary'!$B$5</x:f>
-        <x:v>0.19095427397875042</x:v>
+        <x:v>0.22949333410424577</x:v>
       </x:c>
       <x:c r="H8" s="59" t="str">
         <x:f>IF(D8&gt;'Summary'!$B$7,"Above range",IF(D8&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
-        <x:v>Above range</x:v>
+        <x:v>Within range</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -997,22 +997,22 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D9" s="57" t="n">
-        <x:v>3.7871275818753105</x:v>
+        <x:v>3.7700675133562607</x:v>
       </x:c>
       <x:c r="E9" s="57" t="n">
         <x:v>4.235288421697744</x:v>
       </x:c>
       <x:c r="F9" s="58" t="n">
         <x:f>IF(E9="","",D9-E9)</x:f>
-        <x:v>-0.4481608398224335</x:v>
+        <x:v>-0.46522090834148333</x:v>
       </x:c>
       <x:c r="G9" s="58" t="n">
         <x:f>D9-'Summary'!$B$5</x:f>
-        <x:v>0.15712758187531062</x:v>
+        <x:v>0.14006751335626078</x:v>
       </x:c>
       <x:c r="H9" s="59" t="str">
         <x:f>IF(D9&gt;'Summary'!$B$7,"Above range",IF(D9&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
-        <x:v>Above range</x:v>
+        <x:v>Within range</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1026,18 +1026,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D10" s="57" t="n">
-        <x:v>5.379166666666666</x:v>
+        <x:v>5.410416666666666</x:v>
       </x:c>
       <x:c r="E10" s="57" t="n">
         <x:v>4.282500000000001</x:v>
       </x:c>
       <x:c r="F10" s="58" t="n">
         <x:f>IF(E10="","",D10-E10)</x:f>
-        <x:v>1.0966666666666658</x:v>
+        <x:v>1.1279166666666658</x:v>
       </x:c>
       <x:c r="G10" s="58" t="n">
         <x:f>D10-'Summary'!$B$5</x:f>
-        <x:v>1.7491666666666665</x:v>
+        <x:v>1.7804166666666665</x:v>
       </x:c>
       <x:c r="H10" s="59" t="str">
         <x:f>IF(D10&gt;'Summary'!$B$7,"Above range",IF(D10&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -1055,18 +1055,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D11" s="57" t="n">
-        <x:v>5.345339974563227</x:v>
+        <x:v>5.320990845918681</x:v>
       </x:c>
       <x:c r="E11" s="57" t="n">
         <x:v>4.24867330789656</x:v>
       </x:c>
       <x:c r="F11" s="58" t="n">
         <x:f>IF(E11="","",D11-E11)</x:f>
-        <x:v>1.0966666666666667</x:v>
+        <x:v>1.072317538022121</x:v>
       </x:c>
       <x:c r="G11" s="58" t="n">
         <x:f>D11-'Summary'!$B$5</x:f>
-        <x:v>1.7153399745632267</x:v>
+        <x:v>1.690990845918681</x:v>
       </x:c>
       <x:c r="H11" s="59" t="str">
         <x:f>IF(D11&gt;'Summary'!$B$7,"Above range",IF(D11&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -1084,18 +1084,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D12" s="57" t="n">
-        <x:v>4.104166666666666</x:v>
+        <x:v>4.135416666666666</x:v>
       </x:c>
       <x:c r="E12" s="57" t="n">
         <x:v>3.7925</x:v>
       </x:c>
       <x:c r="F12" s="58" t="n">
         <x:f>IF(E12="","",D12-E12)</x:f>
-        <x:v>0.3116666666666661</x:v>
+        <x:v>0.3429166666666661</x:v>
       </x:c>
       <x:c r="G12" s="58" t="n">
         <x:f>D12-'Summary'!$B$5</x:f>
-        <x:v>0.4741666666666662</x:v>
+        <x:v>0.5054166666666662</x:v>
       </x:c>
       <x:c r="H12" s="59" t="str">
         <x:f>IF(D12&gt;'Summary'!$B$7,"Above range",IF(D12&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -1113,18 +1113,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D13" s="62" t="n">
-        <x:v>4.070339974563226</x:v>
+        <x:v>4.0459908459186815</x:v>
       </x:c>
       <x:c r="E13" s="62" t="n">
         <x:v>3.75867330789656</x:v>
       </x:c>
       <x:c r="F13" s="63" t="n">
         <x:f>IF(E13="","",D13-E13)</x:f>
-        <x:v>0.3116666666666661</x:v>
+        <x:v>0.28731753802212134</x:v>
       </x:c>
       <x:c r="G13" s="63" t="n">
         <x:f>D13-'Summary'!$B$5</x:f>
-        <x:v>0.4403399745632264</x:v>
+        <x:v>0.41599084591868163</x:v>
       </x:c>
       <x:c r="H13" s="64" t="str">
         <x:f>IF(D13&gt;'Summary'!$B$7,"Above range",IF(D13&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -1190,10 +1190,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E2" s="24" t="n">
-        <x:v>0.3821016681731235</x:v>
+        <x:v>0.38490293626892447</x:v>
       </x:c>
       <x:c r="F2" s="24" t="n">
-        <x:v>-0.269107221787717</x:v>
+        <x:v>-0.2677065877398163</x:v>
       </x:c>
       <x:c r="G2" s="24" t="n">
         <x:v>2.4730007673131067</x:v>
@@ -1216,10 +1216,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E3" s="26" t="n">
-        <x:v>-0.8326031227715198</x:v>
+        <x:v>-0.8284719911318006</x:v>
       </x:c>
       <x:c r="F3" s="26" t="n">
-        <x:v>-0.1298814495718702</x:v>
+        <x:v>-0.12781588375201058</x:v>
       </x:c>
       <x:c r="G3" s="26" t="n">
         <x:v>1.2441062071424311</x:v>
@@ -1242,10 +1242,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E4" s="26" t="n">
-        <x:v>-1.1162925748105326</x:v>
+        <x:v>-1.1113073205408677</x:v>
       </x:c>
       <x:c r="F4" s="26" t="n">
-        <x:v>-0.21746600953620332</x:v>
+        <x:v>-0.21497338240137065</x:v>
       </x:c>
       <x:c r="G4" s="26" t="n">
         <x:v>0.8433772703718136</x:v>
@@ -1268,10 +1268,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E5" s="26" t="n">
-        <x:v>-0.5870868566785359</x:v>
+        <x:v>-0.582651516520317</x:v>
       </x:c>
       <x:c r="F5" s="26" t="n">
-        <x:v>-0.08034277791053557</x:v>
+        <x:v>-0.07812510783142612</x:v>
       </x:c>
       <x:c r="G5" s="26" t="n">
         <x:v>0.6646813974596116</x:v>
@@ -1294,10 +1294,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E6" s="26" t="n">
-        <x:v>-0.9018337442522486</x:v>
+        <x:v>-0.8970339398681917</x:v>
       </x:c>
       <x:c r="F6" s="26" t="n">
-        <x:v>-0.13723017681231836</x:v>
+        <x:v>-0.1348302746202899</x:v>
       </x:c>
       <x:c r="G6" s="26" t="n">
         <x:v>2.311508234309721</x:v>
@@ -1320,10 +1320,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E7" s="26" t="n">
-        <x:v>-1.1399096151533883</x:v>
+        <x:v>-1.1343208794182933</x:v>
       </x:c>
       <x:c r="F7" s="26" t="n">
-        <x:v>-0.1429496752027558</x:v>
+        <x:v>-0.1401553073352083</x:v>
       </x:c>
       <x:c r="G7" s="26" t="n">
         <x:v>0.38147643487036864</x:v>
@@ -1346,10 +1346,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E8" s="26" t="n">
-        <x:v>-0.5499810738444617</x:v>
+        <x:v>-0.5449600660021867</x:v>
       </x:c>
       <x:c r="F8" s="26" t="n">
-        <x:v>0.1109521430589202</x:v>
+        <x:v>0.11346264698005748</x:v>
       </x:c>
       <x:c r="G8" s="26" t="n">
         <x:v>2.2006126257134824</x:v>
@@ -1372,10 +1372,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E9" s="26" t="n">
-        <x:v>-0.4745849785112586</x:v>
+        <x:v>-0.46972019110341967</x:v>
       </x:c>
       <x:c r="F9" s="26" t="n">
-        <x:v>0.23494109456178083</x:v>
+        <x:v>0.2373734882657003</x:v>
       </x:c>
       <x:c r="G9" s="26" t="n">
         <x:v>2.348726332287194</x:v>
@@ -1398,10 +1398,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E10" s="26" t="n">
-        <x:v>-0.3331052144195261</x:v>
+        <x:v>-0.3274526432531333</x:v>
       </x:c>
       <x:c r="F10" s="26" t="n">
-        <x:v>0.07481014268004305</x:v>
+        <x:v>0.07763642826323947</x:v>
       </x:c>
       <x:c r="G10" s="26" t="n">
         <x:v>-0.5838783808387616</x:v>
@@ -1424,10 +1424,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E11" s="26" t="n">
-        <x:v>0.98945312280034</x:v>
+        <x:v>0.9943609624140632</x:v>
       </x:c>
       <x:c r="F11" s="26" t="n">
-        <x:v>0.5334493888278254</x:v>
+        <x:v>0.5359033086346868</x:v>
       </x:c>
       <x:c r="G11" s="26" t="n">
         <x:v>3.3120010781102565</x:v>
@@ -1450,10 +1450,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E12" s="26" t="n">
-        <x:v>0.9997098066219077</x:v>
+        <x:v>1.0049754867295633</x:v>
       </x:c>
       <x:c r="F12" s="26" t="n">
-        <x:v>0.8470291642922179</x:v>
+        <x:v>0.8496620043460454</x:v>
       </x:c>
       <x:c r="G12" s="26" t="n">
         <x:v>2.8816371357637953</x:v>
@@ -1476,10 +1476,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E13" s="26" t="n">
-        <x:v>0.47859827231595053</x:v>
+        <x:v>0.48440123364286736</x:v>
       </x:c>
       <x:c r="F13" s="26" t="n">
-        <x:v>0.7188351054736</x:v>
+        <x:v>0.7217365861370584</x:v>
       </x:c>
       <x:c r="G13" s="26" t="n">
         <x:v>0.7083096976844404</x:v>
@@ -1502,10 +1502,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E14" s="26" t="n">
-        <x:v>-0.7340946173657777</x:v>
+        <x:v>-0.7279379188368263</x:v>
       </x:c>
       <x:c r="F14" s="26" t="n">
-        <x:v>0.4236881519221628</x:v>
+        <x:v>0.4267665011866385</x:v>
       </x:c>
       <x:c r="G14" s="26" t="n">
         <x:v>1.2091953231133175</x:v>
@@ -1528,10 +1528,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E15" s="26" t="n">
-        <x:v>-0.4841006726035403</x:v>
+        <x:v>-0.4793870486294086</x:v>
       </x:c>
       <x:c r="F15" s="26" t="n">
-        <x:v>0.9278858242904965</x:v>
+        <x:v>0.9302426362775623</x:v>
       </x:c>
       <x:c r="G15" s="26" t="n">
         <x:v>1.9833615711902415</x:v>
@@ -1554,10 +1554,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E16" s="26" t="n">
-        <x:v>-0.26378976740916116</x:v>
+        <x:v>-0.25848979955973084</x:v>
       </x:c>
       <x:c r="F16" s="26" t="n">
-        <x:v>1.056122447784881</x:v>
+        <x:v>1.058772431709596</x:v>
       </x:c>
       <x:c r="G16" s="26" t="n">
         <x:v>0.8636563204683402</x:v>
@@ -1580,10 +1580,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E17" s="26" t="n">
-        <x:v>-0.23614697533535844</x:v>
+        <x:v>-0.2304877718417444</x:v>
       </x:c>
       <x:c r="F17" s="26" t="n">
-        <x:v>0.9199199231276465</x:v>
+        <x:v>0.9227495248744535</x:v>
       </x:c>
       <x:c r="G17" s="26" t="n">
         <x:v>-0.1607304136422616</x:v>
@@ -1606,10 +1606,10 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="E18" s="26" t="n">
-        <x:v>0.7334421511508613</x:v>
+        <x:v>0.7382208540145001</x:v>
       </x:c>
       <x:c r="F18" s="26" t="n">
-        <x:v>0.9387744256063996</x:v>
+        <x:v>0.941163777038219</x:v>
       </x:c>
       <x:c r="G18" s="26" t="n">
         <x:v>0.5279087843499429</x:v>
@@ -1632,10 +1632,10 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="E19" s="26" t="n">
-        <x:v>0.911804377260435</x:v>
+        <x:v>0.9160067257441682</x:v>
       </x:c>
       <x:c r="F19" s="26" t="n">
-        <x:v>1.313982466746617</x:v>
+        <x:v>1.3160836409884833</x:v>
       </x:c>
       <x:c r="G19" s="26" t="n">
         <x:v>1.6837063217905477</x:v>
@@ -1658,10 +1658,10 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="E20" s="26" t="n">
-        <x:v>1.0907355719263059</x:v>
+        <x:v>1.0954909589878707</x:v>
       </x:c>
       <x:c r="F20" s="26" t="n">
-        <x:v>1.3737327141425666</x:v>
+        <x:v>1.3761104076733488</x:v>
       </x:c>
       <x:c r="G20" s="26" t="n">
         <x:v>1.6341492077661843</x:v>
@@ -1684,10 +1684,10 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="E21" s="26" t="n">
-        <x:v>1.9771502632471236</x:v>
+        <x:v>1.9823448673733433</x:v>
       </x:c>
       <x:c r="F21" s="26" t="n">
-        <x:v>1.472265711977446</x:v>
+        <x:v>1.4748630140405563</x:v>
       </x:c>
       <x:c r="G21" s="26" t="n">
         <x:v>1.780489771680438</x:v>
@@ -1710,10 +1710,10 @@
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="E22" s="26" t="n">
-        <x:v>2.988700104156327</x:v>
+        <x:v>2.9932838907015817</x:v>
       </x:c>
       <x:c r="F22" s="26" t="n">
-        <x:v>1.710996031261</x:v>
+        <x:v>1.7132879245336274</x:v>
       </x:c>
       <x:c r="G22" s="26" t="n">
         <x:v>1.7272747602018097</x:v>
@@ -1736,10 +1736,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E23" s="26" t="n">
-        <x:v>2.4628435534217945</x:v>
+        <x:v>2.4679666840565213</x:v>
       </x:c>
       <x:c r="F23" s="26" t="n">
-        <x:v>1.7411351725916586</x:v>
+        <x:v>1.7436967379090222</x:v>
       </x:c>
       <x:c r="G23" s="26" t="n">
         <x:v>1.4654252215648507</x:v>
@@ -1762,10 +1762,10 @@
         <x:v>1.25</x:v>
       </x:c>
       <x:c r="E24" s="26" t="n">
-        <x:v>2.5243682198372355</x:v>
+        <x:v>2.5294895957557095</x:v>
       </x:c>
       <x:c r="F24" s="26" t="n">
-        <x:v>1.8932702644015555</x:v>
+        <x:v>1.8958309523607926</x:v>
       </x:c>
       <x:c r="G24" s="26" t="n">
         <x:v>2.6051431101121785</x:v>
@@ -1788,10 +1788,10 @@
         <x:v>1.25</x:v>
       </x:c>
       <x:c r="E25" s="26" t="n">
-        <x:v>3.0763680923650623</x:v>
+        <x:v>3.080480741831552</x:v>
       </x:c>
       <x:c r="F25" s="26" t="n">
-        <x:v>2.1786604521553508</x:v>
+        <x:v>2.1807167768885956</x:v>
       </x:c>
       <x:c r="G25" s="26" t="n">
         <x:v>3.7223201668443515</x:v>
@@ -1814,10 +1814,10 @@
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="E26" s="26" t="n">
-        <x:v>3.5044501001423702</x:v>
+        <x:v>3.5073977589056904</x:v>
       </x:c>
       <x:c r="F26" s="26" t="n">
-        <x:v>2.421458100058985</x:v>
+        <x:v>2.4229319294406446</x:v>
       </x:c>
       <x:c r="G26" s="26" t="n">
         <x:v>3.191565137274937</x:v>
@@ -1840,10 +1840,10 @@
         <x:v>1.75</x:v>
       </x:c>
       <x:c r="E27" s="26" t="n">
-        <x:v>4.059853739362089</x:v>
+        <x:v>4.0631155451813</x:v>
       </x:c>
       <x:c r="F27" s="26" t="n">
-        <x:v>2.6264616184932414</x:v>
+        <x:v>2.6280925214028463</x:v>
       </x:c>
       <x:c r="G27" s="26" t="n">
         <x:v>2.856178046918224</x:v>
@@ -1866,10 +1866,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="E28" s="26" t="n">
-        <x:v>4.119458979190385</x:v>
+        <x:v>4.123624943561804</x:v>
       </x:c>
       <x:c r="F28" s="26" t="n">
-        <x:v>2.83704791988533</x:v>
+        <x:v>2.8391309020710396</x:v>
       </x:c>
       <x:c r="G28" s="26" t="n">
         <x:v>2.5895288817549833</x:v>
@@ -1892,10 +1892,10 @@
         <x:v>2.25</x:v>
       </x:c>
       <x:c r="E29" s="26" t="n">
-        <x:v>3.6515046460325964</x:v>
+        <x:v>3.654830946880467</x:v>
       </x:c>
       <x:c r="F29" s="26" t="n">
-        <x:v>2.937190023228269</x:v>
+        <x:v>2.938853173652204</x:v>
       </x:c>
       <x:c r="G29" s="26" t="n">
         <x:v>1.6593051762157365</x:v>
@@ -1918,10 +1918,10 @@
         <x:v>2.5</x:v>
       </x:c>
       <x:c r="E30" s="26" t="n">
-        <x:v>2.874131003635641</x:v>
+        <x:v>2.87758167073873</x:v>
       </x:c>
       <x:c r="F30" s="26" t="n">
-        <x:v>2.9078590231844466</x:v>
+        <x:v>2.9095843567359916</x:v>
       </x:c>
       <x:c r="G30" s="26" t="n">
         <x:v>2.53864341878802</x:v>
@@ -1944,10 +1944,10 @@
         <x:v>2.5</x:v>
       </x:c>
       <x:c r="E31" s="26" t="n">
-        <x:v>3.238296321185564</x:v>
+        <x:v>3.241419820275634</x:v>
       </x:c>
       <x:c r="F31" s="26" t="n">
-        <x:v>3.227206100793783</x:v>
+        <x:v>3.2287678503388184</x:v>
       </x:c>
       <x:c r="G31" s="26" t="n">
         <x:v>3.5623191319959266</x:v>
@@ -1970,10 +1970,10 @@
         <x:v>2.25</x:v>
       </x:c>
       <x:c r="E32" s="26" t="n">
-        <x:v>3.24553377785381</x:v>
+        <x:v>3.24857808850713</x:v>
       </x:c>
       <x:c r="F32" s="26" t="n">
-        <x:v>3.1606999569765</x:v>
+        <x:v>3.1622221123031604</x:v>
       </x:c>
       <x:c r="G32" s="26" t="n">
         <x:v>3.902589940807384</x:v>
@@ -1996,10 +1996,10 @@
         <x:v>1.75</x:v>
       </x:c>
       <x:c r="E33" s="26" t="n">
-        <x:v>3.2448534530401165</x:v>
+        <x:v>3.247723802644356</x:v>
       </x:c>
       <x:c r="F33" s="26" t="n">
-        <x:v>3.0725231911023574</x:v>
+        <x:v>3.0739583659044776</x:v>
       </x:c>
       <x:c r="G33" s="26" t="n">
         <x:v>2.75932878910821</x:v>
@@ -2022,10 +2022,10 @@
         <x:v>1.75</x:v>
       </x:c>
       <x:c r="E34" s="26" t="n">
-        <x:v>3.249229134445158</x:v>
+        <x:v>3.252297102051638</x:v>
       </x:c>
       <x:c r="F34" s="26" t="n">
-        <x:v>2.6732481347274724</x:v>
+        <x:v>2.6747821185307123</x:v>
       </x:c>
       <x:c r="G34" s="26" t="n">
         <x:v>-1.1572899638753935</x:v>
@@ -2048,10 +2048,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E35" s="26" t="n">
-        <x:v>-7.42204423386461</x:v>
+        <x:v>-7.41868209286291</x:v>
       </x:c>
       <x:c r="F35" s="26" t="n">
-        <x:v>-2.9496719028354406</x:v>
+        <x:v>-2.9479908323345905</x:v>
       </x:c>
       <x:c r="G35" s="26" t="n">
         <x:v>-14.283053660277126</x:v>
@@ -2074,10 +2074,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E36" s="26" t="n">
-        <x:v>-2.335452714831879</x:v>
+        <x:v>-2.332598240414319</x:v>
       </x:c>
       <x:c r="F36" s="26" t="n">
-        <x:v>-0.8932536683666039</x:v>
+        <x:v>-0.8918264311578239</x:v>
       </x:c>
       <x:c r="G36" s="26" t="n">
         <x:v>19.638965967167202</x:v>
@@ -2100,10 +2100,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E37" s="26" t="n">
-        <x:v>-0.14989594210499968</x:v>
+        <x:v>-0.14702804370430966</x:v>
       </x:c>
       <x:c r="F37" s="26" t="n">
-        <x:v>0.42314436740906963</x:v>
+        <x:v>0.42457831660941464</x:v>
       </x:c>
       <x:c r="G37" s="26" t="n">
         <x:v>3.335564646194587</x:v>
@@ -2126,10 +2126,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E38" s="26" t="n">
-        <x:v>1.7152292424199764</x:v>
+        <x:v>1.7162918476874465</x:v>
       </x:c>
       <x:c r="F38" s="26" t="n">
-        <x:v>0.8955301722564287</x:v>
+        <x:v>0.8960614748901637</x:v>
       </x:c>
       <x:c r="G38" s="26" t="n">
         <x:v>5.37133346420406</x:v>
@@ -2152,10 +2152,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E39" s="26" t="n">
-        <x:v>5.046973960113488</x:v>
+        <x:v>5.045586071499688</x:v>
       </x:c>
       <x:c r="F39" s="26" t="n">
-        <x:v>1.3809963167664798</x:v>
+        <x:v>1.38030237245958</x:v>
       </x:c>
       <x:c r="G39" s="26" t="n">
         <x:v>6.703979730252985</x:v>
@@ -2178,10 +2178,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E40" s="26" t="n">
-        <x:v>6.750191968176389</x:v>
+        <x:v>6.74996734674795</x:v>
       </x:c>
       <x:c r="F40" s="26" t="n">
-        <x:v>2.0336362447298733</x:v>
+        <x:v>2.0335239340156535</x:v>
       </x:c>
       <x:c r="G40" s="26" t="n">
         <x:v>4.698405383976935</x:v>
@@ -2204,10 +2204,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E41" s="26" t="n">
-        <x:v>9.713306579330013</x:v>
+        <x:v>9.713291778112792</x:v>
       </x:c>
       <x:c r="F41" s="26" t="n">
-        <x:v>2.74313325126718</x:v>
+        <x:v>2.7431258506585703</x:v>
       </x:c>
       <x:c r="G41" s="26" t="n">
         <x:v>7.215051167427025</x:v>
@@ -2230,10 +2230,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E42" s="26" t="n">
-        <x:v>10.901330628521716</x:v>
+        <x:v>10.901871683198607</x:v>
       </x:c>
       <x:c r="F42" s="26" t="n">
-        <x:v>2.948983840081961</x:v>
+        <x:v>2.949254367420406</x:v>
       </x:c>
       <x:c r="G42" s="26" t="n">
         <x:v>3.3883401903792447</x:v>
@@ -2256,10 +2256,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E43" s="26" t="n">
-        <x:v>11.395479915607341</x:v>
+        <x:v>11.39809497156169</x:v>
       </x:c>
       <x:c r="F43" s="26" t="n">
-        <x:v>3.4851348404718157</x:v>
+        <x:v>3.486442368448991</x:v>
       </x:c>
       <x:c r="G43" s="26" t="n">
         <x:v>4.70552334267994</x:v>
@@ -2282,10 +2282,10 @@
         <x:v>2.5</x:v>
       </x:c>
       <x:c r="E44" s="26" t="n">
-        <x:v>11.248537740847466</x:v>
+        <x:v>11.251829881421084</x:v>
       </x:c>
       <x:c r="F44" s="26" t="n">
-        <x:v>3.7458792174314564</x:v>
+        <x:v>3.7475252877182665</x:v>
       </x:c>
       <x:c r="G44" s="26" t="n">
         <x:v>3.83478458676203</x:v>
@@ -2308,10 +2308,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E45" s="26" t="n">
-        <x:v>10.123793845314218</x:v>
+        <x:v>10.127860951471467</x:v>
       </x:c>
       <x:c r="F45" s="26" t="n">
-        <x:v>4.326783272555097</x:v>
+        <x:v>4.328816825633722</x:v>
       </x:c>
       <x:c r="G45" s="26" t="n">
         <x:v>4.11856904466292</x:v>
@@ -2334,10 +2334,10 @@
         <x:v>4.75</x:v>
       </x:c>
       <x:c r="E46" s="26" t="n">
-        <x:v>8.668830270727176</x:v>
+        <x:v>8.673434439310375</x:v>
       </x:c>
       <x:c r="F46" s="26" t="n">
-        <x:v>4.517366963722702</x:v>
+        <x:v>4.519669048014301</x:v>
       </x:c>
       <x:c r="G46" s="26" t="n">
         <x:v>4.865779144624146</x:v>
@@ -2360,10 +2360,10 @@
         <x:v>5.25</x:v>
       </x:c>
       <x:c r="E47" s="26" t="n">
-        <x:v>6.862849902713428</x:v>
+        <x:v>6.868500986055668</x:v>
       </x:c>
       <x:c r="F47" s="26" t="n">
-        <x:v>4.963107184915492</x:v>
+        <x:v>4.965932726586612</x:v>
       </x:c>
       <x:c r="G47" s="26" t="n">
         <x:v>4.169634460548068</x:v>
@@ -2386,10 +2386,10 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="E48" s="26" t="n">
-        <x:v>5.9689194507047</x:v>
+        <x:v>5.976601206932669</x:v>
       </x:c>
       <x:c r="F48" s="26" t="n">
-        <x:v>4.873540848877008</x:v>
+        <x:v>4.877381726990993</x:v>
       </x:c>
       <x:c r="G48" s="26" t="n">
         <x:v>6.112845928592585</x:v>
@@ -2412,10 +2412,10 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="E49" s="26" t="n">
-        <x:v>4.834567537088672</x:v>
+        <x:v>4.841622486590254</x:v>
       </x:c>
       <x:c r="F49" s="26" t="n">
-        <x:v>4.813339750383399</x:v>
+        <x:v>4.81686722513419</x:v>
       </x:c>
       <x:c r="G49" s="26" t="n">
         <x:v>4.6616563331953005</x:v>
@@ -2438,10 +2438,10 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="E50" s="26" t="n">
-        <x:v>4.682775934746497</x:v>
+        <x:v>4.685985663378069</x:v>
       </x:c>
       <x:c r="F50" s="26" t="n">
-        <x:v>4.477461729265974</x:v>
+        <x:v>4.47906659358176</x:v>
       </x:c>
       <x:c r="G50" s="26" t="n">
         <x:v>4.171291813443606</x:v>
@@ -2464,10 +2464,10 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="E51" s="26" t="n">
-        <x:v>4.406087567466002</x:v>
+        <x:v>4.409681751822772</x:v>
       </x:c>
       <x:c r="F51" s="26" t="n">
-        <x:v>4.717011220620588</x:v>
+        <x:v>4.7188083127989735</x:v>
       </x:c>
       <x:c r="G51" s="26" t="n">
         <x:v>5.278481201787318</x:v>
@@ -2490,10 +2490,10 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="E52" s="26" t="n">
-        <x:v>3.7965034494659005</x:v>
+        <x:v>3.799914006669143</x:v>
       </x:c>
       <x:c r="F52" s="26" t="n">
-        <x:v>4.3589976854492045</x:v>
+        <x:v>4.360702964050825</x:v>
       </x:c>
       <x:c r="G52" s="26" t="n">
         <x:v>4.687273990599743</x:v>
@@ -2516,10 +2516,10 @@
         <x:v>4.75</x:v>
       </x:c>
       <x:c r="E53" s="26" t="n">
-        <x:v>4.043941832142453</x:v>
+        <x:v>4.046029978711584</x:v>
       </x:c>
       <x:c r="F53" s="26" t="n">
-        <x:v>4.295586902226258</x:v>
+        <x:v>4.296630975510824</x:v>
       </x:c>
       <x:c r="G53" s="26" t="n">
         <x:v>4.239026806530559</x:v>
@@ -2542,10 +2542,10 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="E54" s="26" t="n">
-        <x:v>3.9051376874803783</x:v>
+        <x:v>3.906071783997163</x:v>
       </x:c>
       <x:c r="F54" s="26" t="n">
-        <x:v>4.160733793346079</x:v>
+        <x:v>4.1612008416044715</x:v>
       </x:c>
       <x:c r="G54" s="26" t="n">
         <x:v>3.2045020295779345</x:v>
@@ -2568,10 +2568,10 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="E55" s="26" t="n">
-        <x:v>3.7751900791639903</x:v>
+        <x:v>3.776447523581173</x:v>
       </x:c>
       <x:c r="F55" s="26" t="n">
-        <x:v>4.516896342558374</x:v>
+        <x:v>4.517525064766964</x:v>
       </x:c>
       <x:c r="G55" s="26" t="n">
         <x:v>4.648128271500598</x:v>
@@ -2594,10 +2594,10 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="E56" s="26" t="n">
-        <x:v>4.193458127485422</x:v>
+        <x:v>4.193984641190231</x:v>
       </x:c>
       <x:c r="F56" s="26" t="n">
-        <x:v>4.286957109968895</x:v>
+        <x:v>4.2872203668213</x:v>
       </x:c>
       <x:c r="G56" s="26" t="n">
         <x:v>5.839158232724845</x:v>
@@ -2620,10 +2620,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E57" s="26" t="n">
-        <x:v>4.045832903464467</x:v>
+        <x:v>4.046316682399642</x:v>
       </x:c>
       <x:c r="F57" s="26" t="n">
-        <x:v>4.093153300572105</x:v>
+        <x:v>4.0933951900396925</x:v>
       </x:c>
       <x:c r="G57" s="26" t="n">
         <x:v>3.7281694478500333</x:v>
@@ -2646,10 +2646,10 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="E58" s="26" t="n">
-        <x:v>4.769996798550084</x:v>
+        <x:v>4.8043430978133745</x:v>
       </x:c>
       <x:c r="F58" s="26" t="n">
-        <x:v>4.008487301069509</x:v>
+        <x:v>4.025660450701153</x:v>
       </x:c>
       <x:c r="G58" s="26" t="n">
         <x:v>3.984897781183367</x:v>
@@ -2672,10 +2672,10 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="E59" s="26" t="n">
-        <x:v>6.000635970135097</x:v>
+        <x:v>5.951937712846006</x:v>
       </x:c>
       <x:c r="F59" s="26" t="n">
-        <x:v>4.235288421697744</x:v>
+        <x:v>4.210939293053199</x:v>
       </x:c>
       <x:c r="G59" s="26" t="n">
         <x:v>4.24867330789656</x:v>
@@ -2692,22 +2692,22 @@
         <x:v>3.63</x:v>
       </x:c>
       <x:c r="C60" s="70" t="n">
-        <x:v>3.5</x:v>
+        <x:v>3.75</x:v>
       </x:c>
       <x:c r="D60" s="70" t="n">
-        <x:v>3.75</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E60" s="70" t="n">
-        <x:v>5.956002463524023</x:v>
+        <x:v>5.978880506132231</x:v>
       </x:c>
       <x:c r="F60" s="70" t="n">
-        <x:v>3.7871275818753105</x:v>
+        <x:v>3.7700675133562607</x:v>
       </x:c>
       <x:c r="G60" s="70" t="n">
-        <x:v>5.345339974563227</x:v>
+        <x:v>5.320990845918681</x:v>
       </x:c>
       <x:c r="H60" s="70" t="n">
-        <x:v>4.070339974563226</x:v>
+        <x:v>4.0459908459186815</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2804,25 +2804,25 @@
         <x:v>1.6391030289831354</x:v>
       </x:c>
       <x:c r="F2" s="52" t="n">
-        <x:v>0.3821016681731235</x:v>
+        <x:v>0.38490293626892447</x:v>
       </x:c>
       <x:c r="G2" s="52" t="n">
         <x:v>0.6454535839012445</x:v>
       </x:c>
       <x:c r="H2" s="52" t="n">
-        <x:v>-0.6115477769087674</x:v>
+        <x:v>-0.608746508812966</x:v>
       </x:c>
       <x:c r="I2" s="52" t="n">
         <x:v>0.8562181811582343</x:v>
       </x:c>
       <x:c r="J2" s="52" t="n">
-        <x:v>0.22771750075322844</x:v>
+        <x:v>0.22911813480112891</x:v>
       </x:c>
       <x:c r="K2" s="52" t="n">
         <x:v>0.35939345861728894</x:v>
       </x:c>
       <x:c r="L2" s="52" t="n">
-        <x:v>-0.269107221787717</x:v>
+        <x:v>-0.2677065877398163</x:v>
       </x:c>
       <x:c r="M2" s="52" t="n">
         <x:v>3.0836216666666667</x:v>
@@ -2854,25 +2854,25 @@
         <x:v>0.5624390864586113</x:v>
       </x:c>
       <x:c r="F3" s="57" t="n">
-        <x:v>-0.8326031227715198</x:v>
+        <x:v>-0.8284719911318006</x:v>
       </x:c>
       <x:c r="G3" s="57" t="n">
         <x:v>1.0319459767530574</x:v>
       </x:c>
       <x:c r="H3" s="57" t="n">
-        <x:v>-0.3630962324770737</x:v>
+        <x:v>-0.35896510083735444</x:v>
       </x:c>
       <x:c r="I3" s="57" t="n">
         <x:v>0.3328862098959723</x:v>
       </x:c>
       <x:c r="J3" s="57" t="n">
-        <x:v>-0.36463489471909327</x:v>
+        <x:v>-0.36256932889923366</x:v>
       </x:c>
       <x:c r="K3" s="57" t="n">
         <x:v>0.5676396550431954</x:v>
       </x:c>
       <x:c r="L3" s="57" t="n">
-        <x:v>-0.1298814495718702</x:v>
+        <x:v>-0.12781588375201058</x:v>
       </x:c>
       <x:c r="M3" s="57" t="n">
         <x:v>1.9204916666666667</x:v>
@@ -2904,25 +2904,25 @@
         <x:v>0.28609731986647224</x:v>
       </x:c>
       <x:c r="F4" s="57" t="n">
-        <x:v>-1.1162925748105326</x:v>
+        <x:v>-1.1113073205408677</x:v>
       </x:c>
       <x:c r="G4" s="57" t="n">
         <x:v>0.8141245422712649</x:v>
       </x:c>
       <x:c r="H4" s="57" t="n">
-        <x:v>-0.58826535240574</x:v>
+        <x:v>-0.5832800981360746</x:v>
       </x:c>
       <x:c r="I4" s="57" t="n">
         <x:v>0.21971532659990278</x:v>
       </x:c>
       <x:c r="J4" s="57" t="n">
-        <x:v>-0.4814796207385996</x:v>
+        <x:v>-0.4789869936037672</x:v>
       </x:c>
       <x:c r="K4" s="57" t="n">
         <x:v>0.4837289378022991</x:v>
       </x:c>
       <x:c r="L4" s="57" t="n">
-        <x:v>-0.21746600953620332</x:v>
+        <x:v>-0.21497338240137065</x:v>
       </x:c>
       <x:c r="M4" s="57" t="n">
         <x:v>1.5202033333333331</x:v>
@@ -2954,25 +2954,25 @@
         <x:v>0.770371489703134</x:v>
       </x:c>
       <x:c r="F5" s="57" t="n">
-        <x:v>-0.5870868566785359</x:v>
+        <x:v>-0.582651516520317</x:v>
       </x:c>
       <x:c r="G5" s="57" t="n">
         <x:v>1.0534394572272654</x:v>
       </x:c>
       <x:c r="H5" s="57" t="n">
-        <x:v>-0.30401888915440445</x:v>
+        <x:v>-0.29958354899618556</x:v>
       </x:c>
       <x:c r="I5" s="57" t="n">
         <x:v>0.45685241151823364</x:v>
       </x:c>
       <x:c r="J5" s="57" t="n">
-        <x:v>-0.22187676167260129</x:v>
+        <x:v>-0.21965909159349184</x:v>
       </x:c>
       <x:c r="K5" s="57" t="n">
         <x:v>0.5983863952802994</x:v>
       </x:c>
       <x:c r="L5" s="57" t="n">
-        <x:v>-0.08034277791053557</x:v>
+        <x:v>-0.07812510783142612</x:v>
       </x:c>
       <x:c r="M5" s="57" t="n">
         <x:v>1.3194616666666668</x:v>
@@ -3004,25 +3004,25 @@
         <x:v>0.3466821405545044</x:v>
       </x:c>
       <x:c r="F6" s="57" t="n">
-        <x:v>-0.9018337442522486</x:v>
+        <x:v>-0.8970339398681917</x:v>
       </x:c>
       <x:c r="G6" s="57" t="n">
         <x:v>0.8140555311821163</x:v>
       </x:c>
       <x:c r="H6" s="57" t="n">
-        <x:v>-0.43446035362463675</x:v>
+        <x:v>-0.42966054924057984</x:v>
       </x:c>
       <x:c r="I6" s="57" t="n">
         <x:v>0.2533410702772522</x:v>
       </x:c>
       <x:c r="J6" s="57" t="n">
-        <x:v>-0.3709168721261243</x:v>
+        <x:v>-0.36851696993409583</x:v>
       </x:c>
       <x:c r="K6" s="57" t="n">
         <x:v>0.48702776559105815</x:v>
       </x:c>
       <x:c r="L6" s="57" t="n">
-        <x:v>-0.13723017681231836</x:v>
+        <x:v>-0.1348302746202899</x:v>
       </x:c>
       <x:c r="M6" s="57" t="n">
         <x:v>2.912485</x:v>
@@ -3054,25 +3054,25 @@
         <x:v>0.24036929916632133</x:v>
       </x:c>
       <x:c r="F7" s="57" t="n">
-        <x:v>-1.1399096151533883</x:v>
+        <x:v>-1.1343208794182933</x:v>
       </x:c>
       <x:c r="G7" s="57" t="n">
         <x:v>0.9510462305808649</x:v>
       </x:c>
       <x:c r="H7" s="57" t="n">
-        <x:v>-0.42923268373884493</x:v>
+        <x:v>-0.42364394800374994</x:v>
       </x:c>
       <x:c r="I7" s="57" t="n">
         <x:v>0.19185131624982732</x:v>
       </x:c>
       <x:c r="J7" s="57" t="n">
-        <x:v>-0.4982881409100275</x:v>
+        <x:v>-0.49549377304248</x:v>
       </x:c>
       <x:c r="K7" s="57" t="n">
         <x:v>0.5471897819570991</x:v>
       </x:c>
       <x:c r="L7" s="57" t="n">
-        <x:v>-0.1429496752027558</x:v>
+        <x:v>-0.1401553073352083</x:v>
       </x:c>
       <x:c r="M7" s="57" t="n">
         <x:v>1.0457516666666669</x:v>
@@ -3104,25 +3104,25 @@
         <x:v>0.7056006483781756</x:v>
       </x:c>
       <x:c r="F8" s="57" t="n">
-        <x:v>-0.5499810738444617</x:v>
+        <x:v>-0.5449600660021867</x:v>
       </x:c>
       <x:c r="G8" s="57" t="n">
         <x:v>1.3608193416738104</x:v>
       </x:c>
       <x:c r="H8" s="57" t="n">
-        <x:v>0.10523761945117371</x:v>
+        <x:v>0.11025862729344826</x:v>
       </x:c>
       <x:c r="I8" s="57" t="n">
         <x:v>0.41113365752242115</x:v>
       </x:c>
       <x:c r="J8" s="57" t="n">
-        <x:v>-0.2166572035888975</x:v>
+        <x:v>-0.21414669966776</x:v>
       </x:c>
       <x:c r="K8" s="57" t="n">
         <x:v>0.7387430041702385</x:v>
       </x:c>
       <x:c r="L8" s="57" t="n">
-        <x:v>0.1109521430589202</x:v>
+        <x:v>0.11346264698005748</x:v>
       </x:c>
       <x:c r="M8" s="57" t="n">
         <x:v>2.8049583333333334</x:v>
@@ -3154,25 +3154,25 @@
         <x:v>0.6943601889423974</x:v>
       </x:c>
       <x:c r="F9" s="57" t="n">
-        <x:v>-0.4745849785112586</x:v>
+        <x:v>-0.46972019110341967</x:v>
       </x:c>
       <x:c r="G9" s="57" t="n">
         <x:v>1.5554940232438845</x:v>
       </x:c>
       <x:c r="H9" s="57" t="n">
-        <x:v>0.38654885579022835</x:v>
+        <x:v>0.39141364319806726</x:v>
       </x:c>
       <x:c r="I9" s="57" t="n">
         <x:v>0.38884676113786537</x:v>
       </x:c>
       <x:c r="J9" s="57" t="n">
-        <x:v>-0.19562582258896263</x:v>
+        <x:v>-0.19319342888504318</x:v>
       </x:c>
       <x:c r="K9" s="57" t="n">
         <x:v>0.8194136782886089</x:v>
       </x:c>
       <x:c r="L9" s="57" t="n">
-        <x:v>0.23494109456178083</x:v>
+        <x:v>0.2373734882657003</x:v>
       </x:c>
       <x:c r="M9" s="57" t="n">
         <x:v>2.9111966666666667</x:v>
@@ -3204,25 +3204,25 @@
         <x:v>1.106099767090232</x:v>
       </x:c>
       <x:c r="F10" s="57" t="n">
-        <x:v>-0.3331052144195261</x:v>
+        <x:v>-0.3274526432531333</x:v>
       </x:c>
       <x:c r="G10" s="57" t="n">
         <x:v>1.5021586002031777</x:v>
       </x:c>
       <x:c r="H10" s="57" t="n">
-        <x:v>0.06295361869341942</x:v>
+        <x:v>0.06860618985981226</x:v>
       </x:c>
       <x:c r="I10" s="57" t="n">
         <x:v>0.5963832168784493</x:v>
       </x:c>
       <x:c r="J10" s="57" t="n">
-        <x:v>-0.12321927387642972</x:v>
+        <x:v>-0.1203929882932333</x:v>
       </x:c>
       <x:c r="K10" s="57" t="n">
         <x:v>0.7944126334349222</x:v>
       </x:c>
       <x:c r="L10" s="57" t="n">
-        <x:v>0.07481014268004305</x:v>
+        <x:v>0.07763642826323947</x:v>
       </x:c>
       <x:c r="M10" s="57" t="n">
         <x:v>0.10989333333333329</x:v>
@@ -3254,25 +3254,25 @@
         <x:v>1.9871933660007672</x:v>
       </x:c>
       <x:c r="F11" s="57" t="n">
-        <x:v>0.98945312280034</x:v>
+        <x:v>0.9943609624140632</x:v>
       </x:c>
       <x:c r="G11" s="57" t="n">
         <x:v>1.9913056875227448</x:v>
       </x:c>
       <x:c r="H11" s="57" t="n">
-        <x:v>0.9935654443223176</x:v>
+        <x:v>0.9984732839360404</x:v>
       </x:c>
       <x:c r="I11" s="57" t="n">
         <x:v>1.0302633496670504</x:v>
       </x:c>
       <x:c r="J11" s="57" t="n">
-        <x:v>0.5313932280668366</x:v>
+        <x:v>0.5338471478736982</x:v>
       </x:c>
       <x:c r="K11" s="57" t="n">
         <x:v>1.0323195104280392</x:v>
       </x:c>
       <x:c r="L11" s="57" t="n">
-        <x:v>0.5334493888278254</x:v>
+        <x:v>0.5359033086346868</x:v>
       </x:c>
       <x:c r="M11" s="57" t="n">
         <x:v>3.789378333333333</x:v>
@@ -3304,25 +3304,25 @@
         <x:v>1.8065540296764424</x:v>
       </x:c>
       <x:c r="F12" s="57" t="n">
-        <x:v>0.9997098066219077</x:v>
+        <x:v>1.0049754867295633</x:v>
       </x:c>
       <x:c r="G12" s="57" t="n">
         <x:v>2.407569218305637</x:v>
       </x:c>
       <x:c r="H12" s="57" t="n">
-        <x:v>1.6007249952511025</x:v>
+        <x:v>1.6059906753587576</x:v>
       </x:c>
       <x:c r="I12" s="57" t="n">
         <x:v>0.9499436815048878</x:v>
       </x:c>
       <x:c r="J12" s="57" t="n">
-        <x:v>0.5465215699776205</x:v>
+        <x:v>0.5491544100314483</x:v>
       </x:c>
       <x:c r="K12" s="57" t="n">
         <x:v>1.2504512758194852</x:v>
       </x:c>
       <x:c r="L12" s="57" t="n">
-        <x:v>0.8470291642922179</x:v>
+        <x:v>0.8496620043460454</x:v>
       </x:c>
       <x:c r="M12" s="57" t="n">
         <x:v>3.264261666666667</x:v>
@@ -3354,25 +3354,25 @@
         <x:v>1.3925189394726523</x:v>
       </x:c>
       <x:c r="F13" s="57" t="n">
-        <x:v>0.47859827231595053</x:v>
+        <x:v>0.48440123364286736</x:v>
       </x:c>
       <x:c r="G13" s="57" t="n">
         <x:v>2.2615908781039025</x:v>
       </x:c>
       <x:c r="H13" s="57" t="n">
-        <x:v>1.3476702109471999</x:v>
+        <x:v>1.3534731722741167</x:v>
       </x:c>
       <x:c r="I13" s="57" t="n">
         <x:v>0.7412594697363262</x:v>
       </x:c>
       <x:c r="J13" s="57" t="n">
-        <x:v>0.28429913615797525</x:v>
+        <x:v>0.28720061682143366</x:v>
       </x:c>
       <x:c r="K13" s="57" t="n">
         <x:v>1.1757954390519512</x:v>
       </x:c>
       <x:c r="L13" s="57" t="n">
-        <x:v>0.7188351054736</x:v>
+        <x:v>0.7217365861370584</x:v>
       </x:c>
       <x:c r="M13" s="57" t="n">
         <x:v>1.142575</x:v>
@@ -3404,25 +3404,25 @@
         <x:v>0.16898337056339152</x:v>
       </x:c>
       <x:c r="F14" s="57" t="n">
-        <x:v>-0.7340946173657777</x:v>
+        <x:v>-0.7279379188368263</x:v>
       </x:c>
       <x:c r="G14" s="57" t="n">
         <x:v>1.650454291773495</x:v>
       </x:c>
       <x:c r="H14" s="57" t="n">
-        <x:v>0.7473763038443256</x:v>
+        <x:v>0.753533002373277</x:v>
       </x:c>
       <x:c r="I14" s="57" t="n">
         <x:v>0.13449168528169575</x:v>
       </x:c>
       <x:c r="J14" s="57" t="n">
-        <x:v>-0.3170473086828889</x:v>
+        <x:v>-0.3139689594184132</x:v>
       </x:c>
       <x:c r="K14" s="57" t="n">
         <x:v>0.8752271458867475</x:v>
       </x:c>
       <x:c r="L14" s="57" t="n">
-        <x:v>0.4236881519221628</x:v>
+        <x:v>0.4267665011866385</x:v>
       </x:c>
       <x:c r="M14" s="57" t="n">
         <x:v>1.637605</x:v>
@@ -3454,25 +3454,25 @@
         <x:v>0.3242805101119556</x:v>
       </x:c>
       <x:c r="F15" s="57" t="n">
-        <x:v>-0.4841006726035403</x:v>
+        <x:v>-0.4793870486294086</x:v>
       </x:c>
       <x:c r="G15" s="57" t="n">
         <x:v>2.5541528312964887</x:v>
       </x:c>
       <x:c r="H15" s="57" t="n">
-        <x:v>1.7457716485809929</x:v>
+        <x:v>1.7504852725551245</x:v>
       </x:c>
       <x:c r="I15" s="57" t="n">
         <x:v>0.21714025505597778</x:v>
       </x:c>
       <x:c r="J15" s="57" t="n">
-        <x:v>-0.18705033630177015</x:v>
+        <x:v>-0.18469352431470432</x:v>
       </x:c>
       <x:c r="K15" s="57" t="n">
         <x:v>1.3320764156482443</x:v>
       </x:c>
       <x:c r="L15" s="57" t="n">
-        <x:v>0.9278858242904965</x:v>
+        <x:v>0.9302426362775623</x:v>
       </x:c>
       <x:c r="M15" s="57" t="n">
         <x:v>2.367725</x:v>
@@ -3504,25 +3504,25 @@
         <x:v>0.4506965795291791</x:v>
       </x:c>
       <x:c r="F16" s="57" t="n">
-        <x:v>-0.26378976740916116</x:v>
+        <x:v>-0.25848979955973084</x:v>
       </x:c>
       <x:c r="G16" s="57" t="n">
         <x:v>2.7033979091747686</x:v>
       </x:c>
       <x:c r="H16" s="57" t="n">
-        <x:v>1.9889115622364284</x:v>
+        <x:v>1.9942115300858587</x:v>
       </x:c>
       <x:c r="I16" s="57" t="n">
         <x:v>0.2870149564312562</x:v>
       </x:c>
       <x:c r="J16" s="57" t="n">
-        <x:v>-0.07022821703791393</x:v>
+        <x:v>-0.06757823311319877</x:v>
       </x:c>
       <x:c r="K16" s="57" t="n">
         <x:v>1.413365621254051</x:v>
       </x:c>
       <x:c r="L16" s="57" t="n">
-        <x:v>1.056122447784881</x:v>
+        <x:v>1.058772431709596</x:v>
       </x:c>
       <x:c r="M16" s="57" t="n">
         <x:v>1.1997983333333333</x:v>
@@ -3554,25 +3554,25 @@
         <x:v>0.4976568481296586</x:v>
       </x:c>
       <x:c r="F17" s="57" t="n">
-        <x:v>-0.23614697533535844</x:v>
+        <x:v>-0.2304877718417444</x:v>
       </x:c>
       <x:c r="G17" s="57" t="n">
         <x:v>2.4369770030536433</x:v>
       </x:c>
       <x:c r="H17" s="57" t="n">
-        <x:v>1.7031731795886262</x:v>
+        <x:v>1.7088323830822403</x:v>
       </x:c>
       <x:c r="I17" s="57" t="n">
         <x:v>0.31716175739816266</x:v>
       </x:c>
       <x:c r="J17" s="57" t="n">
-        <x:v>-0.04974015433434588</x:v>
+        <x:v>-0.04691055258753886</x:v>
       </x:c>
       <x:c r="K17" s="57" t="n">
         <x:v>1.286821834860155</x:v>
       </x:c>
       <x:c r="L17" s="57" t="n">
-        <x:v>0.9199199231276465</x:v>
+        <x:v>0.9227495248744535</x:v>
       </x:c>
       <x:c r="M17" s="57" t="n">
         <x:v>0.18354833333333342</x:v>
@@ -3604,25 +3604,25 @@
         <x:v>1.195661313587188</x:v>
       </x:c>
       <x:c r="F18" s="57" t="n">
-        <x:v>0.7334421511508613</x:v>
+        <x:v>0.7382208540145001</x:v>
       </x:c>
       <x:c r="G18" s="57" t="n">
         <x:v>2.179768013649126</x:v>
       </x:c>
       <x:c r="H18" s="57" t="n">
-        <x:v>1.7175488512127992</x:v>
+        <x:v>1.722327554076438</x:v>
       </x:c>
       <x:c r="I18" s="57" t="n">
         <x:v>0.677830656793594</x:v>
       </x:c>
       <x:c r="J18" s="57" t="n">
-        <x:v>0.44672107557543067</x:v>
+        <x:v>0.44911042700725007</x:v>
       </x:c>
       <x:c r="K18" s="57" t="n">
         <x:v>1.169884006824563</x:v>
       </x:c>
       <x:c r="L18" s="57" t="n">
-        <x:v>0.9387744256063996</x:v>
+        <x:v>0.941163777038219</x:v>
       </x:c>
       <x:c r="M18" s="57" t="n">
         <x:v>0.7390016666666664</x:v>
@@ -3654,25 +3654,25 @@
         <x:v>1.096511509371929</x:v>
       </x:c>
       <x:c r="F19" s="57" t="n">
-        <x:v>0.911804377260435</x:v>
+        <x:v>0.9160067257441682</x:v>
       </x:c>
       <x:c r="G19" s="57" t="n">
         <x:v>2.4526720656047276</x:v>
       </x:c>
       <x:c r="H19" s="57" t="n">
-        <x:v>2.267964933493234</x:v>
+        <x:v>2.2721672819769667</x:v>
       </x:c>
       <x:c r="I19" s="57" t="n">
         <x:v>0.7282557546859645</x:v>
       </x:c>
       <x:c r="J19" s="57" t="n">
-        <x:v>0.6359021886302174</x:v>
+        <x:v>0.638003362872084</x:v>
       </x:c>
       <x:c r="K19" s="57" t="n">
         <x:v>1.4063360328023637</x:v>
       </x:c>
       <x:c r="L19" s="57" t="n">
-        <x:v>1.313982466746617</x:v>
+        <x:v>1.3160836409884833</x:v>
       </x:c>
       <x:c r="M19" s="57" t="n">
         <x:v>1.7575316666666663</x:v>
@@ -3704,25 +3704,25 @@
         <x:v>1.0740201233365823</x:v>
       </x:c>
       <x:c r="F20" s="57" t="n">
-        <x:v>1.0907355719263059</x:v>
+        <x:v>1.0954909589878707</x:v>
       </x:c>
       <x:c r="G20" s="57" t="n">
         <x:v>2.3574166463620756</x:v>
       </x:c>
       <x:c r="H20" s="57" t="n">
-        <x:v>2.3741320949517997</x:v>
+        <x:v>2.378887482013364</x:v>
       </x:c>
       <x:c r="I20" s="57" t="n">
         <x:v>0.7236767283349579</x:v>
       </x:c>
       <x:c r="J20" s="57" t="n">
-        <x:v>0.7320344526298197</x:v>
+        <x:v>0.7344121461606021</x:v>
       </x:c>
       <x:c r="K20" s="57" t="n">
         <x:v>1.3653749898477046</x:v>
       </x:c>
       <x:c r="L20" s="57" t="n">
-        <x:v>1.3737327141425666</x:v>
+        <x:v>1.3761104076733488</x:v>
       </x:c>
       <x:c r="M20" s="57" t="n">
         <x:v>1.60718</x:v>
@@ -3754,25 +3754,25 @@
         <x:v>2.0414350531678522</x:v>
       </x:c>
       <x:c r="F21" s="57" t="n">
-        <x:v>1.9771502632471236</x:v>
+        <x:v>1.9823448673733433</x:v>
       </x:c>
       <x:c r="G21" s="57" t="n">
         <x:v>2.612149547208954</x:v>
       </x:c>
       <x:c r="H21" s="57" t="n">
-        <x:v>2.5478647572882256</x:v>
+        <x:v>2.553059361414446</x:v>
       </x:c>
       <x:c r="I21" s="57" t="n">
         <x:v>1.2190508599172594</x:v>
       </x:c>
       <x:c r="J21" s="57" t="n">
-        <x:v>1.186908464956895</x:v>
+        <x:v>1.1895057670200049</x:v>
       </x:c>
       <x:c r="K21" s="57" t="n">
         <x:v>1.5044081069378104</x:v>
       </x:c>
       <x:c r="L21" s="57" t="n">
-        <x:v>1.472265711977446</x:v>
+        <x:v>1.4748630140405563</x:v>
       </x:c>
       <x:c r="M21" s="57" t="n">
         <x:v>1.7929750000000002</x:v>
@@ -3804,25 +3804,25 @@
         <x:v>3.0775275960822093</x:v>
       </x:c>
       <x:c r="F22" s="57" t="n">
-        <x:v>2.988700104156327</x:v>
+        <x:v>2.9932838907015817</x:v>
       </x:c>
       <x:c r="G22" s="57" t="n">
         <x:v>3.060819554447882</x:v>
       </x:c>
       <x:c r="H22" s="57" t="n">
-        <x:v>2.9719920625219998</x:v>
+        <x:v>2.9765758490672547</x:v>
       </x:c>
       <x:c r="I22" s="57" t="n">
         <x:v>1.7637637980411047</x:v>
       </x:c>
       <x:c r="J22" s="57" t="n">
-        <x:v>1.7193500520781635</x:v>
+        <x:v>1.721641945350791</x:v>
       </x:c>
       <x:c r="K22" s="57" t="n">
         <x:v>1.755409777223941</x:v>
       </x:c>
       <x:c r="L22" s="57" t="n">
-        <x:v>1.710996031261</x:v>
+        <x:v>1.7132879245336274</x:v>
       </x:c>
       <x:c r="M22" s="57" t="n">
         <x:v>1.7531600000000003</x:v>
@@ -3854,25 +3854,25 @@
         <x:v>2.6019664211416393</x:v>
       </x:c>
       <x:c r="F23" s="57" t="n">
-        <x:v>2.4628435534217945</x:v>
+        <x:v>2.4679666840565213</x:v>
       </x:c>
       <x:c r="G23" s="57" t="n">
         <x:v>2.921393212903162</x:v>
       </x:c>
       <x:c r="H23" s="57" t="n">
-        <x:v>2.782270345183317</x:v>
+        <x:v>2.7873934758180443</x:v>
       </x:c>
       <x:c r="I23" s="57" t="n">
         <x:v>1.6509832105708198</x:v>
       </x:c>
       <x:c r="J23" s="57" t="n">
-        <x:v>1.5814217767108973</x:v>
+        <x:v>1.5839833420282607</x:v>
       </x:c>
       <x:c r="K23" s="57" t="n">
         <x:v>1.810696606451581</x:v>
       </x:c>
       <x:c r="L23" s="57" t="n">
-        <x:v>1.7411351725916586</x:v>
+        <x:v>1.7436967379090222</x:v>
       </x:c>
       <x:c r="M23" s="57" t="n">
         <x:v>1.5152</x:v>
@@ -3904,25 +3904,25 @@
         <x:v>2.4651890838206754</x:v>
       </x:c>
       <x:c r="F24" s="57" t="n">
-        <x:v>2.5243682198372355</x:v>
+        <x:v>2.5294895957557095</x:v>
       </x:c>
       <x:c r="G24" s="57" t="n">
         <x:v>2.7773613927865513</x:v>
       </x:c>
       <x:c r="H24" s="57" t="n">
-        <x:v>2.836540528803111</x:v>
+        <x:v>2.841661904721585</x:v>
       </x:c>
       <x:c r="I24" s="57" t="n">
         <x:v>1.7075945419103378</x:v>
       </x:c>
       <x:c r="J24" s="57" t="n">
-        <x:v>1.7371841099186178</x:v>
+        <x:v>1.7397447978778549</x:v>
       </x:c>
       <x:c r="K24" s="57" t="n">
         <x:v>1.8636806963932757</x:v>
       </x:c>
       <x:c r="L24" s="57" t="n">
-        <x:v>1.8932702644015555</x:v>
+        <x:v>1.8958309523607926</x:v>
       </x:c>
       <x:c r="M24" s="57" t="n">
         <x:v>2.556171666666667</x:v>
@@ -3954,25 +3954,25 @@
         <x:v>2.749433518280822</x:v>
       </x:c>
       <x:c r="F25" s="57" t="n">
-        <x:v>3.0763680923650623</x:v>
+        <x:v>3.080480741831552</x:v>
       </x:c>
       <x:c r="G25" s="57" t="n">
         <x:v>2.877052996893128</x:v>
       </x:c>
       <x:c r="H25" s="57" t="n">
-        <x:v>3.203987570977368</x:v>
+        <x:v>3.208100220443858</x:v>
       </x:c>
       <x:c r="I25" s="57" t="n">
         <x:v>1.9513834258070775</x:v>
       </x:c>
       <x:c r="J25" s="57" t="n">
-        <x:v>2.1148507128491976</x:v>
+        <x:v>2.1169070375824424</x:v>
       </x:c>
       <x:c r="K25" s="57" t="n">
         <x:v>2.0151931651132307</x:v>
       </x:c>
       <x:c r="L25" s="57" t="n">
-        <x:v>2.1786604521553508</x:v>
+        <x:v>2.1807167768885956</x:v>
       </x:c>
       <x:c r="M25" s="57" t="n">
         <x:v>3.5432516666666665</x:v>
@@ -4004,25 +4004,25 @@
         <x:v>3.1283152204493136</x:v>
       </x:c>
       <x:c r="F26" s="57" t="n">
-        <x:v>3.5044501001423702</x:v>
+        <x:v>3.5073977589056904</x:v>
       </x:c>
       <x:c r="G26" s="57" t="n">
         <x:v>3.2634479870915802</x:v>
       </x:c>
       <x:c r="H26" s="57" t="n">
-        <x:v>3.639582866784637</x:v>
+        <x:v>3.6425305255479565</x:v>
       </x:c>
       <x:c r="I26" s="57" t="n">
         <x:v>2.1658242768913234</x:v>
       </x:c>
       <x:c r="J26" s="57" t="n">
-        <x:v>2.3538917167378517</x:v>
+        <x:v>2.3553655461195118</x:v>
       </x:c>
       <x:c r="K26" s="57" t="n">
         <x:v>2.2333906602124567</x:v>
       </x:c>
       <x:c r="L26" s="57" t="n">
-        <x:v>2.421458100058985</x:v>
+        <x:v>2.4229319294406446</x:v>
       </x:c>
       <x:c r="M26" s="57" t="n">
         <x:v>2.9916883333333333</x:v>
@@ -4054,25 +4054,25 @@
         <x:v>3.7517500568234894</x:v>
       </x:c>
       <x:c r="F27" s="57" t="n">
-        <x:v>4.059853739362089</x:v>
+        <x:v>4.0631155451813</x:v>
       </x:c>
       <x:c r="G27" s="57" t="n">
         <x:v>3.498152887781216</x:v>
       </x:c>
       <x:c r="H27" s="57" t="n">
-        <x:v>3.8062565703198157</x:v>
+        <x:v>3.809518376139026</x:v>
       </x:c>
       <x:c r="I27" s="57" t="n">
         <x:v>2.5992083617450783</x:v>
       </x:c>
       <x:c r="J27" s="57" t="n">
-        <x:v>2.7532602030143782</x:v>
+        <x:v>2.7548911059239836</x:v>
       </x:c>
       <x:c r="K27" s="57" t="n">
         <x:v>2.4724097772239415</x:v>
       </x:c>
       <x:c r="L27" s="57" t="n">
-        <x:v>2.6264616184932414</x:v>
+        <x:v>2.6280925214028463</x:v>
       </x:c>
       <x:c r="M27" s="57" t="n">
         <x:v>2.690248333333334</x:v>
@@ -4104,25 +4104,25 @@
         <x:v>3.964185632252838</x:v>
       </x:c>
       <x:c r="F28" s="57" t="n">
-        <x:v>4.119458979190385</x:v>
+        <x:v>4.123624943561804</x:v>
       </x:c>
       <x:c r="G28" s="57" t="n">
         <x:v>3.782155826166446</x:v>
       </x:c>
       <x:c r="H28" s="57" t="n">
-        <x:v>3.9374291731039923</x:v>
+        <x:v>3.9415951374754123</x:v>
       </x:c>
       <x:c r="I28" s="57" t="n">
         <x:v>2.8504261494597527</x:v>
       </x:c>
       <x:c r="J28" s="57" t="n">
-        <x:v>2.928062822928526</x:v>
+        <x:v>2.9301458051142357</x:v>
       </x:c>
       <x:c r="K28" s="57" t="n">
         <x:v>2.7594112464165566</x:v>
       </x:c>
       <x:c r="L28" s="57" t="n">
-        <x:v>2.83704791988533</x:v>
+        <x:v>2.8391309020710396</x:v>
       </x:c>
       <x:c r="M28" s="57" t="n">
         <x:v>2.49804</x:v>
@@ -4154,25 +4154,25 @@
         <x:v>3.4271986173467397</x:v>
       </x:c>
       <x:c r="F29" s="57" t="n">
-        <x:v>3.6515046460325964</x:v>
+        <x:v>3.654830946880467</x:v>
       </x:c>
       <x:c r="G29" s="57" t="n">
         <x:v>3.726740684437348</x:v>
       </x:c>
       <x:c r="H29" s="57" t="n">
-        <x:v>3.9510467131232048</x:v>
+        <x:v>3.9543730139710753</x:v>
       </x:c>
       <x:c r="I29" s="57" t="n">
         <x:v>2.6752659753400363</x:v>
       </x:c>
       <x:c r="J29" s="57" t="n">
-        <x:v>2.7874189896829646</x:v>
+        <x:v>2.7890821401069</x:v>
       </x:c>
       <x:c r="K29" s="57" t="n">
         <x:v>2.8250370088853405</x:v>
       </x:c>
       <x:c r="L29" s="57" t="n">
-        <x:v>2.937190023228269</x:v>
+        <x:v>2.938853173652204</x:v>
       </x:c>
       <x:c r="M29" s="57" t="n">
         <x:v>1.5338333333333332</x:v>
@@ -4204,25 +4204,25 @@
         <x:v>2.549798119287191</x:v>
       </x:c>
       <x:c r="F30" s="57" t="n">
-        <x:v>2.874131003635641</x:v>
+        <x:v>2.87758167073873</x:v>
       </x:c>
       <x:c r="G30" s="57" t="n">
         <x:v>3.2713851620204433</x:v>
       </x:c>
       <x:c r="H30" s="57" t="n">
-        <x:v>3.5957180463688934</x:v>
+        <x:v>3.599168713471983</x:v>
       </x:c>
       <x:c r="I30" s="57" t="n">
         <x:v>2.3848990596435957</x:v>
       </x:c>
       <x:c r="J30" s="57" t="n">
-        <x:v>2.5470655018178205</x:v>
+        <x:v>2.548790835369365</x:v>
       </x:c>
       <x:c r="K30" s="57" t="n">
         <x:v>2.7456925810102217</x:v>
       </x:c>
       <x:c r="L30" s="57" t="n">
-        <x:v>2.9078590231844466</x:v>
+        <x:v>2.9095843567359916</x:v>
       </x:c>
       <x:c r="M30" s="57" t="n">
         <x:v>2.36321</x:v>
@@ -4254,25 +4254,25 @@
         <x:v>2.6603931234790776</x:v>
       </x:c>
       <x:c r="F31" s="57" t="n">
-        <x:v>3.238296321185564</x:v>
+        <x:v>3.241419820275634</x:v>
       </x:c>
       <x:c r="G31" s="57" t="n">
         <x:v>3.473175670547747</x:v>
       </x:c>
       <x:c r="H31" s="57" t="n">
-        <x:v>4.051078868254233</x:v>
+        <x:v>4.0542023673443035</x:v>
       </x:c>
       <x:c r="I31" s="57" t="n">
         <x:v>2.5318632284062055</x:v>
       </x:c>
       <x:c r="J31" s="57" t="n">
-        <x:v>2.8208148272594484</x:v>
+        <x:v>2.8223765768044835</x:v>
       </x:c>
       <x:c r="K31" s="57" t="n">
         <x:v>2.93825450194054</x:v>
       </x:c>
       <x:c r="L31" s="57" t="n">
-        <x:v>3.227206100793783</x:v>
+        <x:v>3.2287678503388184</x:v>
       </x:c>
       <x:c r="M31" s="57" t="n">
         <x:v>3.261633333333333</x:v>
@@ -4304,25 +4304,25 @@
         <x:v>2.45951503119682</x:v>
       </x:c>
       <x:c r="F32" s="57" t="n">
-        <x:v>3.24553377785381</x:v>
+        <x:v>3.24857808850713</x:v>
       </x:c>
       <x:c r="G32" s="57" t="n">
         <x:v>3.1387145006293435</x:v>
       </x:c>
       <x:c r="H32" s="57" t="n">
-        <x:v>3.9247332472863334</x:v>
+        <x:v>3.9277775579396534</x:v>
       </x:c>
       <x:c r="I32" s="57" t="n">
         <x:v>2.4280908489317437</x:v>
       </x:c>
       <x:c r="J32" s="57" t="n">
-        <x:v>2.821100222260238</x:v>
+        <x:v>2.8226223775868986</x:v>
       </x:c>
       <x:c r="K32" s="57" t="n">
         <x:v>2.7676905836480055</x:v>
       </x:c>
       <x:c r="L32" s="57" t="n">
-        <x:v>3.1606999569765</x:v>
+        <x:v>3.1622221123031604</x:v>
       </x:c>
       <x:c r="M32" s="57" t="n">
         <x:v>3.4995483333333333</x:v>
@@ -4354,25 +4354,25 @@
         <x:v>2.4748630969778564</x:v>
       </x:c>
       <x:c r="F33" s="57" t="n">
-        <x:v>3.2448534530401165</x:v>
+        <x:v>3.247723802644356</x:v>
       </x:c>
       <x:c r="G33" s="57" t="n">
         <x:v>3.1850560261424548</x:v>
       </x:c>
       <x:c r="H33" s="57" t="n">
-        <x:v>3.9550463822047153</x:v>
+        <x:v>3.9579167318089548</x:v>
       </x:c>
       <x:c r="I33" s="57" t="n">
         <x:v>2.332431548488928</x:v>
       </x:c>
       <x:c r="J33" s="57" t="n">
-        <x:v>2.717426726520058</x:v>
+        <x:v>2.718861901322178</x:v>
       </x:c>
       <x:c r="K33" s="57" t="n">
         <x:v>2.687528013071227</x:v>
       </x:c>
       <x:c r="L33" s="57" t="n">
-        <x:v>3.0725231911023574</x:v>
+        <x:v>3.0739583659044776</x:v>
       </x:c>
       <x:c r="M33" s="57" t="n">
         <x:v>2.3645199999999997</x:v>
@@ -4404,25 +4404,25 @@
         <x:v>2.454388837574078</x:v>
       </x:c>
       <x:c r="F34" s="57" t="n">
-        <x:v>3.249229134445158</x:v>
+        <x:v>3.252297102051638</x:v>
       </x:c>
       <x:c r="G34" s="57" t="n">
         <x:v>2.9083226392505312</x:v>
       </x:c>
       <x:c r="H34" s="57" t="n">
-        <x:v>3.7031629361216116</x:v>
+        <x:v>3.7062309037280916</x:v>
       </x:c>
       <x:c r="I34" s="57" t="n">
         <x:v>2.0488610854537055</x:v>
       </x:c>
       <x:c r="J34" s="57" t="n">
-        <x:v>2.4462812338892457</x:v>
+        <x:v>2.4478152176924857</x:v>
       </x:c>
       <x:c r="K34" s="57" t="n">
         <x:v>2.275827986291932</x:v>
       </x:c>
       <x:c r="L34" s="57" t="n">
-        <x:v>2.6732481347274724</x:v>
+        <x:v>2.6747821185307123</x:v>
       </x:c>
       <x:c r="M34" s="57" t="n">
         <x:v>-1.5671883333333334</x:v>
@@ -4454,25 +4454,25 @@
         <x:v>-8.18386543035602</x:v>
       </x:c>
       <x:c r="F35" s="57" t="n">
-        <x:v>-7.42204423386461</x:v>
+        <x:v>-7.41868209286291</x:v>
       </x:c>
       <x:c r="G35" s="57" t="n">
         <x:v>-7.92116500216229</x:v>
       </x:c>
       <x:c r="H35" s="57" t="n">
-        <x:v>-7.159343805670881</x:v>
+        <x:v>-7.155981664669181</x:v>
       </x:c>
       <x:c r="I35" s="57" t="n">
         <x:v>-3.46193271517801</x:v>
       </x:c>
       <x:c r="J35" s="57" t="n">
-        <x:v>-3.081022116932305</x:v>
+        <x:v>-3.079341046431455</x:v>
       </x:c>
       <x:c r="K35" s="57" t="n">
         <x:v>-3.330582501081145</x:v>
       </x:c>
       <x:c r="L35" s="57" t="n">
-        <x:v>-2.9496719028354406</x:v>
+        <x:v>-2.9479908323345905</x:v>
       </x:c>
       <x:c r="M35" s="57" t="n">
         <x:v>-14.677245000000001</x:v>
@@ -4504,25 +4504,25 @@
         <x:v>-3.166678321678319</x:v>
       </x:c>
       <x:c r="F36" s="57" t="n">
-        <x:v>-2.335452714831879</x:v>
+        <x:v>-2.332598240414319</x:v>
       </x:c>
       <x:c r="G36" s="57" t="n">
         <x:v>-2.677732943579648</x:v>
       </x:c>
       <x:c r="H36" s="57" t="n">
-        <x:v>-1.8465073367332079</x:v>
+        <x:v>-1.8436528623156478</x:v>
       </x:c>
       <x:c r="I36" s="57" t="n">
         <x:v>-1.5533391608391596</x:v>
       </x:c>
       <x:c r="J36" s="57" t="n">
-        <x:v>-1.1377263574159395</x:v>
+        <x:v>-1.1362991202071595</x:v>
       </x:c>
       <x:c r="K36" s="57" t="n">
         <x:v>-1.308866471789824</x:v>
       </x:c>
       <x:c r="L36" s="57" t="n">
-        <x:v>-0.8932536683666039</x:v>
+        <x:v>-0.8918264311578239</x:v>
       </x:c>
       <x:c r="M36" s="57" t="n">
         <x:v>19.211155</x:v>
@@ -4554,25 +4554,25 @@
         <x:v>-0.9613380731403294</x:v>
       </x:c>
       <x:c r="F37" s="57" t="n">
-        <x:v>-0.14989594210499968</x:v>
+        <x:v>-0.14702804370430966</x:v>
       </x:c>
       <x:c r="G37" s="57" t="n">
         <x:v>-0.05848672955052381</x:v>
       </x:c>
       <x:c r="H37" s="57" t="n">
-        <x:v>0.7529554014848059</x:v>
+        <x:v>0.7558232998854959</x:v>
       </x:c>
       <x:c r="I37" s="57" t="n">
         <x:v>-0.434002369903498</x:v>
       </x:c>
       <x:c r="J37" s="57" t="n">
-        <x:v>-0.02828130438583317</x:v>
+        <x:v>-0.026847355185488163</x:v>
       </x:c>
       <x:c r="K37" s="57" t="n">
         <x:v>0.017423301891404765</x:v>
       </x:c>
       <x:c r="L37" s="57" t="n">
-        <x:v>0.42314436740906963</x:v>
+        <x:v>0.42457831660941464</x:v>
       </x:c>
       <x:c r="M37" s="57" t="n">
         <x:v>2.917726666666667</x:v>
@@ -4604,25 +4604,25 @@
         <x:v>0.7672036478529263</x:v>
       </x:c>
       <x:c r="F38" s="57" t="n">
-        <x:v>1.7152292424199764</x:v>
+        <x:v>1.7162918476874465</x:v>
       </x:c>
       <x:c r="G38" s="57" t="n">
         <x:v>0.7530347499458072</x:v>
       </x:c>
       <x:c r="H38" s="57" t="n">
-        <x:v>1.7010603445128574</x:v>
+        <x:v>1.7021229497803274</x:v>
       </x:c>
       <x:c r="I38" s="57" t="n">
         <x:v>0.4286018239264631</x:v>
       </x:c>
       <x:c r="J38" s="57" t="n">
-        <x:v>0.9026146212099883</x:v>
+        <x:v>0.9031459238437233</x:v>
       </x:c>
       <x:c r="K38" s="57" t="n">
         <x:v>0.4215173749729036</x:v>
       </x:c>
       <x:c r="L38" s="57" t="n">
-        <x:v>0.8955301722564287</x:v>
+        <x:v>0.8960614748901637</x:v>
       </x:c>
       <x:c r="M38" s="57" t="n">
         <x:v>4.8900049999999995</x:v>
@@ -4654,25 +4654,25 @@
         <x:v>4.025780561510787</x:v>
       </x:c>
       <x:c r="F39" s="57" t="n">
-        <x:v>5.046973960113488</x:v>
+        <x:v>5.045586071499688</x:v>
       </x:c>
       <x:c r="G39" s="57" t="n">
         <x:v>1.66079923493026</x:v>
       </x:c>
       <x:c r="H39" s="57" t="n">
-        <x:v>2.6819926335329596</x:v>
+        <x:v>2.68060474491916</x:v>
       </x:c>
       <x:c r="I39" s="57" t="n">
         <x:v>2.0528902807553937</x:v>
       </x:c>
       <x:c r="J39" s="57" t="n">
-        <x:v>2.563486980056744</x:v>
+        <x:v>2.562793035749844</x:v>
       </x:c>
       <x:c r="K39" s="57" t="n">
         <x:v>0.8703996174651301</x:v>
       </x:c>
       <x:c r="L39" s="57" t="n">
-        <x:v>1.3809963167664798</x:v>
+        <x:v>1.38030237245958</x:v>
       </x:c>
       <x:c r="M39" s="57" t="n">
         <x:v>6.1924</x:v>
@@ -4704,25 +4704,25 @@
         <x:v>5.776885057471289</x:v>
       </x:c>
       <x:c r="F40" s="57" t="n">
-        <x:v>6.750191968176389</x:v>
+        <x:v>6.74996734674795</x:v>
       </x:c>
       <x:c r="G40" s="57" t="n">
         <x:v>3.0239655787546464</x:v>
       </x:c>
       <x:c r="H40" s="57" t="n">
-        <x:v>3.9972724894597462</x:v>
+        <x:v>3.9970478680313066</x:v>
       </x:c>
       <x:c r="I40" s="57" t="n">
         <x:v>2.9234425287356447</x:v>
       </x:c>
       <x:c r="J40" s="57" t="n">
-        <x:v>3.4100959840881946</x:v>
+        <x:v>3.4099836733739752</x:v>
       </x:c>
       <x:c r="K40" s="57" t="n">
         <x:v>1.5469827893773231</x:v>
       </x:c>
       <x:c r="L40" s="57" t="n">
-        <x:v>2.0336362447298733</x:v>
+        <x:v>2.0335239340156535</x:v>
       </x:c>
       <x:c r="M40" s="57" t="n">
         <x:v>4.207865</x:v>
@@ -4754,25 +4754,25 @@
         <x:v>8.482455333162513</x:v>
       </x:c>
       <x:c r="F41" s="57" t="n">
-        <x:v>9.713306579330013</x:v>
+        <x:v>9.713291778112792</x:v>
       </x:c>
       <x:c r="G41" s="57" t="n">
         <x:v>4.1654152563668605</x:v>
       </x:c>
       <x:c r="H41" s="57" t="n">
-        <x:v>5.396266502534361</x:v>
+        <x:v>5.396251701317141</x:v>
       </x:c>
       <x:c r="I41" s="57" t="n">
         <x:v>4.286227666581256</x:v>
       </x:c>
       <x:c r="J41" s="57" t="n">
-        <x:v>4.901653289665006</x:v>
+        <x:v>4.901645889056396</x:v>
       </x:c>
       <x:c r="K41" s="57" t="n">
         <x:v>2.12770762818343</x:v>
       </x:c>
       <x:c r="L41" s="57" t="n">
-        <x:v>2.74313325126718</x:v>
+        <x:v>2.7431258506585703</x:v>
       </x:c>
       <x:c r="M41" s="57" t="n">
         <x:v>6.595715</x:v>
@@ -4804,25 +4804,25 @@
         <x:v>9.866069834001152</x:v>
       </x:c>
       <x:c r="F42" s="57" t="n">
-        <x:v>10.901330628521716</x:v>
+        <x:v>10.901871683198607</x:v>
       </x:c>
       <x:c r="G42" s="57" t="n">
         <x:v>4.782706885643359</x:v>
       </x:c>
       <x:c r="H42" s="57" t="n">
-        <x:v>5.817967680163922</x:v>
+        <x:v>5.818508734840812</x:v>
       </x:c>
       <x:c r="I42" s="57" t="n">
         <x:v>4.973034917000576</x:v>
       </x:c>
       <x:c r="J42" s="57" t="n">
-        <x:v>5.490665314260858</x:v>
+        <x:v>5.4909358415993035</x:v>
       </x:c>
       <x:c r="K42" s="57" t="n">
         <x:v>2.4313534428216794</x:v>
       </x:c>
       <x:c r="L42" s="57" t="n">
-        <x:v>2.948983840081961</x:v>
+        <x:v>2.949254367420406</x:v>
       </x:c>
       <x:c r="M42" s="57" t="n">
         <x:v>2.862593333333333</x:v>
@@ -4854,25 +4854,25 @@
         <x:v>10.627900244028694</x:v>
       </x:c>
       <x:c r="F43" s="57" t="n">
-        <x:v>11.395479915607341</x:v>
+        <x:v>11.39809497156169</x:v>
       </x:c>
       <x:c r="G43" s="57" t="n">
         <x:v>6.082690009364985</x:v>
       </x:c>
       <x:c r="H43" s="57" t="n">
-        <x:v>6.850269680943631</x:v>
+        <x:v>6.852884736897982</x:v>
       </x:c>
       <x:c r="I43" s="57" t="n">
         <x:v>5.373950122014347</x:v>
       </x:c>
       <x:c r="J43" s="57" t="n">
-        <x:v>5.75773995780367</x:v>
+        <x:v>5.759047485780845</x:v>
       </x:c>
       <x:c r="K43" s="57" t="n">
         <x:v>3.1013450046824924</x:v>
       </x:c>
       <x:c r="L43" s="57" t="n">
-        <x:v>3.4851348404718157</x:v>
+        <x:v>3.486442368448991</x:v>
       </x:c>
       <x:c r="M43" s="57" t="n">
         <x:v>4.3067416666666665</x:v>
@@ -4904,25 +4904,25 @@
         <x:v>10.433937151368685</x:v>
       </x:c>
       <x:c r="F44" s="57" t="n">
-        <x:v>11.248537740847466</x:v>
+        <x:v>11.251829881421084</x:v>
       </x:c>
       <x:c r="G44" s="57" t="n">
         <x:v>5.907157845384132</x:v>
       </x:c>
       <x:c r="H44" s="57" t="n">
-        <x:v>6.721758434862913</x:v>
+        <x:v>6.725050575436533</x:v>
       </x:c>
       <x:c r="I44" s="57" t="n">
         <x:v>5.601968575684342</x:v>
       </x:c>
       <x:c r="J44" s="57" t="n">
-        <x:v>6.009268870423733</x:v>
+        <x:v>6.010914940710542</x:v>
       </x:c>
       <x:c r="K44" s="57" t="n">
         <x:v>3.338578922692066</x:v>
       </x:c>
       <x:c r="L44" s="57" t="n">
-        <x:v>3.7458792174314564</x:v>
+        <x:v>3.7475252877182665</x:v>
       </x:c>
       <x:c r="M44" s="57" t="n">
         <x:v>3.4109949999999998</x:v>
@@ -4954,25 +4954,25 @@
         <x:v>9.374315967612707</x:v>
       </x:c>
       <x:c r="F45" s="57" t="n">
-        <x:v>10.123793845314218</x:v>
+        <x:v>10.127860951471467</x:v>
       </x:c>
       <x:c r="G45" s="57" t="n">
         <x:v>5.714088667408684</x:v>
       </x:c>
       <x:c r="H45" s="57" t="n">
-        <x:v>6.4635665451101945</x:v>
+        <x:v>6.467633651267445</x:v>
       </x:c>
       <x:c r="I45" s="57" t="n">
         <x:v>5.7821579838063535</x:v>
       </x:c>
       <x:c r="J45" s="57" t="n">
-        <x:v>6.156896922657109</x:v>
+        <x:v>6.158930475735733</x:v>
       </x:c>
       <x:c r="K45" s="57" t="n">
         <x:v>3.9520443337043423</x:v>
       </x:c>
       <x:c r="L45" s="57" t="n">
-        <x:v>4.326783272555097</x:v>
+        <x:v>4.328816825633722</x:v>
       </x:c>
       <x:c r="M45" s="57" t="n">
         <x:v>3.724875</x:v>
@@ -5004,25 +5004,25 @@
         <x:v>7.963604297629344</x:v>
       </x:c>
       <x:c r="F46" s="57" t="n">
-        <x:v>8.668830270727176</x:v>
+        <x:v>8.673434439310375</x:v>
       </x:c>
       <x:c r="G46" s="57" t="n">
         <x:v>4.67617462101424</x:v>
       </x:c>
       <x:c r="H46" s="57" t="n">
-        <x:v>5.38140059411207</x:v>
+        <x:v>5.386004762695269</x:v>
       </x:c>
       <x:c r="I46" s="57" t="n">
         <x:v>5.808468815481339</x:v>
       </x:c>
       <x:c r="J46" s="57" t="n">
-        <x:v>6.161081802030254</x:v>
+        <x:v>6.163383886321854</x:v>
       </x:c>
       <x:c r="K46" s="57" t="n">
         <x:v>4.1647539771737865</x:v>
       </x:c>
       <x:c r="L46" s="57" t="n">
-        <x:v>4.517366963722702</x:v>
+        <x:v>4.519669048014301</x:v>
       </x:c>
       <x:c r="M46" s="57" t="n">
         <x:v>4.492346666666666</x:v>
@@ -5054,25 +5054,25 @@
         <x:v>6.277340498135288</x:v>
       </x:c>
       <x:c r="F47" s="57" t="n">
-        <x:v>6.862849902713428</x:v>
+        <x:v>6.868500986055668</x:v>
       </x:c>
       <x:c r="G47" s="57" t="n">
         <x:v>4.824038298586177</x:v>
       </x:c>
       <x:c r="H47" s="57" t="n">
-        <x:v>5.409547703164317</x:v>
+        <x:v>5.415198786506557</x:v>
       </x:c>
       <x:c r="I47" s="57" t="n">
         <x:v>5.397003582400977</x:v>
       </x:c>
       <x:c r="J47" s="57" t="n">
-        <x:v>5.689758284690047</x:v>
+        <x:v>5.692583826361167</x:v>
       </x:c>
       <x:c r="K47" s="57" t="n">
         <x:v>4.670352482626422</x:v>
       </x:c>
       <x:c r="L47" s="57" t="n">
-        <x:v>4.963107184915492</x:v>
+        <x:v>4.965932726586612</x:v>
       </x:c>
       <x:c r="M47" s="57" t="n">
         <x:v>3.8530333333333333</x:v>
@@ -5104,25 +5104,25 @@
         <x:v>5.44315416089675</x:v>
       </x:c>
       <x:c r="F48" s="57" t="n">
-        <x:v>5.9689194507047</x:v>
+        <x:v>5.976601206932669</x:v>
       </x:c>
       <x:c r="G48" s="57" t="n">
         <x:v>4.231316407946066</x:v>
       </x:c>
       <x:c r="H48" s="57" t="n">
-        <x:v>4.757081697754016</x:v>
+        <x:v>4.764763453981986</x:v>
       </x:c>
       <x:c r="I48" s="57" t="n">
         <x:v>5.216577080448375</x:v>
       </x:c>
       <x:c r="J48" s="57" t="n">
-        <x:v>5.47945972535235</x:v>
+        <x:v>5.4833006034663345</x:v>
       </x:c>
       <x:c r="K48" s="57" t="n">
         <x:v>4.610658203973033</x:v>
       </x:c>
       <x:c r="L48" s="57" t="n">
-        <x:v>4.873540848877008</x:v>
+        <x:v>4.877381726990993</x:v>
       </x:c>
       <x:c r="M48" s="57" t="n">
         <x:v>5.82183</x:v>
@@ -5154,25 +5154,25 @@
         <x:v>4.405518277822901</x:v>
       </x:c>
       <x:c r="F49" s="57" t="n">
-        <x:v>4.834567537088672</x:v>
+        <x:v>4.841622486590254</x:v>
       </x:c>
       <x:c r="G49" s="57" t="n">
         <x:v>3.937630241501027</x:v>
       </x:c>
       <x:c r="H49" s="57" t="n">
-        <x:v>4.366679500766798</x:v>
+        <x:v>4.37373445026838</x:v>
       </x:c>
       <x:c r="I49" s="57" t="n">
         <x:v>4.832759138911451</x:v>
       </x:c>
       <x:c r="J49" s="57" t="n">
-        <x:v>5.047283768544336</x:v>
+        <x:v>5.0508112432951275</x:v>
       </x:c>
       <x:c r="K49" s="57" t="n">
         <x:v>4.598815120750514</x:v>
       </x:c>
       <x:c r="L49" s="57" t="n">
-        <x:v>4.813339750383399</x:v>
+        <x:v>4.81686722513419</x:v>
       </x:c>
       <x:c r="M49" s="57" t="n">
         <x:v>4.41943</x:v>
@@ -5204,25 +5204,25 @@
         <x:v>4.2998603055397195</x:v>
       </x:c>
       <x:c r="F50" s="57" t="n">
-        <x:v>4.682775934746497</x:v>
+        <x:v>4.685985663378069</x:v>
       </x:c>
       <x:c r="G50" s="57" t="n">
         <x:v>3.24200782932517</x:v>
       </x:c>
       <x:c r="H50" s="57" t="n">
-        <x:v>3.624923458531947</x:v>
+        <x:v>3.62813318716352</x:v>
       </x:c>
       <x:c r="I50" s="57" t="n">
         <x:v>4.814930152769859</x:v>
       </x:c>
       <x:c r="J50" s="57" t="n">
-        <x:v>5.006387967373248</x:v>
+        <x:v>5.007992831689035</x:v>
       </x:c>
       <x:c r="K50" s="57" t="n">
         <x:v>4.286003914662585</x:v>
       </x:c>
       <x:c r="L50" s="57" t="n">
-        <x:v>4.477461729265974</x:v>
+        <x:v>4.47906659358176</x:v>
       </x:c>
       <x:c r="M50" s="57" t="n">
         <x:v>3.9601783333333334</x:v>
@@ -5254,25 +5254,25 @@
         <x:v>4.160222467204729</x:v>
       </x:c>
       <x:c r="F51" s="57" t="n">
-        <x:v>4.406087567466002</x:v>
+        <x:v>4.409681751822772</x:v>
       </x:c>
       <x:c r="G51" s="57" t="n">
         <x:v>3.8581573409799033</x:v>
       </x:c>
       <x:c r="H51" s="57" t="n">
-        <x:v>4.104022441241176</x:v>
+        <x:v>4.107616625597946</x:v>
       </x:c>
       <x:c r="I51" s="57" t="n">
         <x:v>4.745111233602365</x:v>
       </x:c>
       <x:c r="J51" s="57" t="n">
-        <x:v>4.868043783733</x:v>
+        <x:v>4.869840875911386</x:v>
       </x:c>
       <x:c r="K51" s="57" t="n">
         <x:v>4.594078670489951</x:v>
       </x:c>
       <x:c r="L51" s="57" t="n">
-        <x:v>4.717011220620588</x:v>
+        <x:v>4.7188083127989735</x:v>
       </x:c>
       <x:c r="M51" s="57" t="n">
         <x:v>5.13713</x:v>
@@ -5304,25 +5304,25 @@
         <x:v>3.718167769981595</x:v>
       </x:c>
       <x:c r="F52" s="57" t="n">
-        <x:v>3.7965034494659005</x:v>
+        <x:v>3.799914006669143</x:v>
       </x:c>
       <x:c r="G52" s="57" t="n">
         <x:v>3.3096596914141028</x:v>
       </x:c>
       <x:c r="H52" s="57" t="n">
-        <x:v>3.387995370898409</x:v>
+        <x:v>3.3914059281016504</x:v>
       </x:c>
       <x:c r="I52" s="57" t="n">
         <x:v>4.524083884990798</x:v>
       </x:c>
       <x:c r="J52" s="57" t="n">
-        <x:v>4.56325172473295</x:v>
+        <x:v>4.564957003334571</x:v>
       </x:c>
       <x:c r="K52" s="57" t="n">
         <x:v>4.319829845707051</x:v>
       </x:c>
       <x:c r="L52" s="57" t="n">
-        <x:v>4.3589976854492045</x:v>
+        <x:v>4.360702964050825</x:v>
       </x:c>
       <x:c r="M52" s="57" t="n">
         <x:v>4.630941666666667</x:v>
@@ -5354,25 +5354,25 @@
         <x:v>4.134055814259625</x:v>
       </x:c>
       <x:c r="F53" s="57" t="n">
-        <x:v>4.043941832142453</x:v>
+        <x:v>4.046029978711584</x:v>
       </x:c>
       <x:c r="G53" s="57" t="n">
         <x:v>3.417954453236356</x:v>
       </x:c>
       <x:c r="H53" s="57" t="n">
-        <x:v>3.327840471119184</x:v>
+        <x:v>3.3299286176883145</x:v>
       </x:c>
       <x:c r="I53" s="57" t="n">
         <x:v>4.6986945737964785</x:v>
       </x:c>
       <x:c r="J53" s="57" t="n">
-        <x:v>4.653637582737893</x:v>
+        <x:v>4.654681656022458</x:v>
       </x:c>
       <x:c r="K53" s="57" t="n">
         <x:v>4.340643893284844</x:v>
       </x:c>
       <x:c r="L53" s="57" t="n">
-        <x:v>4.295586902226258</x:v>
+        <x:v>4.296630975510824</x:v>
       </x:c>
       <x:c r="M53" s="57" t="n">
         <x:v>4.269638333333333</x:v>
@@ -5404,25 +5404,25 @@
         <x:v>4.113069416581042</x:v>
       </x:c>
       <x:c r="F54" s="57" t="n">
-        <x:v>3.9051376874803783</x:v>
+        <x:v>3.906071783997163</x:v>
       </x:c>
       <x:c r="G54" s="57" t="n">
         <x:v>3.8793993157928237</x:v>
       </x:c>
       <x:c r="H54" s="57" t="n">
-        <x:v>3.6714675866921596</x:v>
+        <x:v>3.672401683208945</x:v>
       </x:c>
       <x:c r="I54" s="57" t="n">
         <x:v>4.38153470829052</x:v>
       </x:c>
       <x:c r="J54" s="57" t="n">
-        <x:v>4.277568843740188</x:v>
+        <x:v>4.278035891998581</x:v>
       </x:c>
       <x:c r="K54" s="57" t="n">
         <x:v>4.264699657896411</x:v>
       </x:c>
       <x:c r="L54" s="57" t="n">
-        <x:v>4.160733793346079</x:v>
+        <x:v>4.1612008416044715</x:v>
       </x:c>
       <x:c r="M54" s="57" t="n">
         <x:v>3.295634999999999</x:v>
@@ -5454,25 +5454,25 @@
         <x:v>3.8706435835311903</x:v>
       </x:c>
       <x:c r="F55" s="57" t="n">
-        <x:v>3.7751900791639903</x:v>
+        <x:v>3.776447523581173</x:v>
       </x:c>
       <x:c r="G55" s="57" t="n">
         <x:v>4.799246189483946</x:v>
       </x:c>
       <x:c r="H55" s="57" t="n">
-        <x:v>4.703792685116746</x:v>
+        <x:v>4.705050129533929</x:v>
       </x:c>
       <x:c r="I55" s="57" t="n">
         <x:v>4.100321791765595</x:v>
       </x:c>
       <x:c r="J55" s="57" t="n">
-        <x:v>4.052595039581995</x:v>
+        <x:v>4.053223761790587</x:v>
       </x:c>
       <x:c r="K55" s="57" t="n">
         <x:v>4.5646230947419735</x:v>
       </x:c>
       <x:c r="L55" s="57" t="n">
-        <x:v>4.516896342558374</x:v>
+        <x:v>4.517525064766964</x:v>
       </x:c>
       <x:c r="M55" s="57" t="n">
         <x:v>4.684355</x:v>
@@ -5504,25 +5504,25 @@
         <x:v>4.141109658678292</x:v>
       </x:c>
       <x:c r="F56" s="57" t="n">
-        <x:v>4.193458127485422</x:v>
+        <x:v>4.193984641190231</x:v>
       </x:c>
       <x:c r="G56" s="57" t="n">
         <x:v>4.191565751130659</x:v>
       </x:c>
       <x:c r="H56" s="57" t="n">
-        <x:v>4.243914219937789</x:v>
+        <x:v>4.244440733642599</x:v>
       </x:c>
       <x:c r="I56" s="57" t="n">
         <x:v>4.235554829339145</x:v>
       </x:c>
       <x:c r="J56" s="57" t="n">
-        <x:v>4.261729063742711</x:v>
+        <x:v>4.261992320595116</x:v>
       </x:c>
       <x:c r="K56" s="57" t="n">
         <x:v>4.260782875565329</x:v>
       </x:c>
       <x:c r="L56" s="57" t="n">
-        <x:v>4.286957109968895</x:v>
+        <x:v>4.2872203668213</x:v>
       </x:c>
       <x:c r="M56" s="57" t="n">
         <x:v>5.804595</x:v>
@@ -5554,25 +5554,25 @@
         <x:v>4.157394393077939</x:v>
       </x:c>
       <x:c r="F57" s="57" t="n">
-        <x:v>4.045832903464467</x:v>
+        <x:v>4.046316682399642</x:v>
       </x:c>
       <x:c r="G57" s="57" t="n">
         <x:v>4.004534757424349</x:v>
       </x:c>
       <x:c r="H57" s="57" t="n">
-        <x:v>3.892973267810877</x:v>
+        <x:v>3.893457046746052</x:v>
       </x:c>
       <x:c r="I57" s="57" t="n">
         <x:v>4.2253638632056365</x:v>
       </x:c>
       <x:c r="J57" s="57" t="n">
-        <x:v>4.1695831183989</x:v>
+        <x:v>4.169825007866487</x:v>
       </x:c>
       <x:c r="K57" s="57" t="n">
         <x:v>4.148934045378841</x:v>
       </x:c>
       <x:c r="L57" s="57" t="n">
-        <x:v>4.093153300572105</x:v>
+        <x:v>4.0933951900396925</x:v>
       </x:c>
       <x:c r="M57" s="57" t="n">
         <x:v>3.766335</x:v>
@@ -5604,25 +5604,25 @@
         <x:v>4.795983516090297</x:v>
       </x:c>
       <x:c r="F58" s="57" t="n">
-        <x:v>4.769996798550084</x:v>
+        <x:v>4.8043430978133745</x:v>
       </x:c>
       <x:c r="G58" s="57" t="n">
         <x:v>4.146294653012562</x:v>
       </x:c>
       <x:c r="H58" s="57" t="n">
-        <x:v>4.12030793547235</x:v>
+        <x:v>4.15465423473564</x:v>
       </x:c>
       <x:c r="I58" s="57" t="n">
         <x:v>4.346325091378482</x:v>
       </x:c>
       <x:c r="J58" s="57" t="n">
-        <x:v>4.333331732608375</x:v>
+        <x:v>4.3505048822400205</x:v>
       </x:c>
       <x:c r="K58" s="57" t="n">
         <x:v>4.0214806598396144</x:v>
       </x:c>
       <x:c r="L58" s="57" t="n">
-        <x:v>4.008487301069509</x:v>
+        <x:v>4.025660450701153</x:v>
       </x:c>
       <x:c r="M58" s="57" t="n">
         <x:v>4.06473</x:v>
@@ -5651,28 +5651,28 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="E59" s="57" t="n">
-        <x:v>6.068289354341977</x:v>
+        <x:v>6.026622687675309</x:v>
       </x:c>
       <x:c r="F59" s="57" t="n">
-        <x:v>6.000635970135097</x:v>
+        <x:v>5.951937712846006</x:v>
       </x:c>
       <x:c r="G59" s="57" t="n">
-        <x:v>4.898230227602368</x:v>
+        <x:v>4.856563560935701</x:v>
       </x:c>
       <x:c r="H59" s="57" t="n">
-        <x:v>4.830576843395488</x:v>
+        <x:v>4.781878586106398</x:v>
       </x:c>
       <x:c r="I59" s="57" t="n">
-        <x:v>4.854144677170988</x:v>
+        <x:v>4.8333113438376545</x:v>
       </x:c>
       <x:c r="J59" s="57" t="n">
-        <x:v>4.820317985067549</x:v>
+        <x:v>4.795968856423003</x:v>
       </x:c>
       <x:c r="K59" s="57" t="n">
-        <x:v>4.269115113801184</x:v>
+        <x:v>4.248281780467851</x:v>
       </x:c>
       <x:c r="L59" s="57" t="n">
-        <x:v>4.235288421697744</x:v>
+        <x:v>4.210939293053199</x:v>
       </x:c>
       <x:c r="M59" s="57" t="n">
         <x:v>4.2825</x:v>
@@ -5695,46 +5695,46 @@
         <x:v>3.63</x:v>
       </x:c>
       <x:c r="C60" s="62" t="n">
-        <x:v>3.5</x:v>
+        <x:v>3.75</x:v>
       </x:c>
       <x:c r="D60" s="62" t="n">
-        <x:v>3.75</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E60" s="62" t="n">
-        <x:v>6.023655847730904</x:v>
+        <x:v>6.157732147628201</x:v>
       </x:c>
       <x:c r="F60" s="62" t="n">
-        <x:v>5.956002463524023</x:v>
+        <x:v>5.978880506132231</x:v>
       </x:c>
       <x:c r="G60" s="62" t="n">
-        <x:v>4.008575214624168</x:v>
+        <x:v>4.0856533348751585</x:v>
       </x:c>
       <x:c r="H60" s="62" t="n">
-        <x:v>3.9409218304172877</x:v>
+        <x:v>3.9068016933791885</x:v>
       </x:c>
       <x:c r="I60" s="62" t="n">
-        <x:v>4.828494590532118</x:v>
+        <x:v>4.895532740480768</x:v>
       </x:c>
       <x:c r="J60" s="62" t="n">
-        <x:v>4.794667898428678</x:v>
+        <x:v>4.806106919732782</x:v>
       </x:c>
       <x:c r="K60" s="62" t="n">
-        <x:v>3.8209542739787503</x:v>
+        <x:v>3.8594933341042457</x:v>
       </x:c>
       <x:c r="L60" s="62" t="n">
-        <x:v>3.7871275818753105</x:v>
+        <x:v>3.7700675133562607</x:v>
       </x:c>
       <x:c r="M60" s="62" t="n">
-        <x:v>5.379166666666666</x:v>
+        <x:v>5.410416666666666</x:v>
       </x:c>
       <x:c r="N60" s="62" t="n">
-        <x:v>5.345339974563227</x:v>
+        <x:v>5.320990845918681</x:v>
       </x:c>
       <x:c r="O60" s="62" t="n">
-        <x:v>4.104166666666666</x:v>
+        <x:v>4.135416666666666</x:v>
       </x:c>
       <x:c r="P60" s="82" t="n">
-        <x:v>4.070339974563226</x:v>
+        <x:v>4.0459908459186815</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5832,7 +5832,7 @@
         <x:v>r_star_sep</x:v>
       </x:c>
       <x:c r="D5" s="93" t="n">
-        <x:v>1.125</x:v>
+        <x:v>1.1875</x:v>
       </x:c>
       <x:c r="E5" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -5849,7 +5849,7 @@
         <x:v>r_star_hlw</x:v>
       </x:c>
       <x:c r="D6" s="93" t="n">
-        <x:v>1.05734661579312</x:v>
+        <x:v>1.00864835850403</x:v>
       </x:c>
       <x:c r="E6" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -5866,7 +5866,7 @@
         <x:v>pce</x:v>
       </x:c>
       <x:c r="D7" s="93" t="n">
-        <x:v>3.768335221498953</x:v>
+        <x:v>3.806334007929824</x:v>
       </x:c>
       <x:c r="E7" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -5900,7 +5900,7 @@
         <x:v>unemp_gap</x:v>
       </x:c>
       <x:c r="D9" s="93" t="n">
-        <x:v>0.492306030964949</x:v>
+        <x:v>0.5214622714669304</x:v>
       </x:c>
       <x:c r="E9" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -5985,7 +5985,7 @@
         <x:v>r_star_sep</x:v>
       </x:c>
       <x:c r="D14" s="93" t="n">
-        <x:v>1.125</x:v>
+        <x:v>1.1875</x:v>
       </x:c>
       <x:c r="E14" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -6002,7 +6002,7 @@
         <x:v>r_star_hlw</x:v>
       </x:c>
       <x:c r="D15" s="95" t="n">
-        <x:v>1.05734661579312</x:v>
+        <x:v>1.00864835850403</x:v>
       </x:c>
       <x:c r="E15" s="96" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -6042,13 +6042,13 @@
         <x:v>Latest Monetary Rules Report</x:v>
       </x:c>
       <x:c r="B2" s="99" t="n">
-        <x:v>46231.5</x:v>
+        <x:v>46280.5</x:v>
       </x:c>
       <x:c r="C2" s="99" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46281.5</x:v>
       </x:c>
       <x:c r="D2" s="54" t="str">
-        <x:v>https://fedagenda.substack.com/p/monetary-rules-report-31f</x:v>
+        <x:v>https://fedagenda.substack.com/p/monetary-rules-report-eef</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -6059,7 +6059,7 @@
         <x:v>46234.5</x:v>
       </x:c>
       <x:c r="C3" s="100" t="n">
-        <x:v>46260.5</x:v>
+        <x:v>46281.5</x:v>
       </x:c>
       <x:c r="D3" s="64" t="str">
         <x:v>https://fedagenda.substack.com/p/monetary-neutrality-report-9d2</x:v>

</xml_diff>

<commit_message>
Publish dashboard release 2026-09-issue-16
</commit_message>
<xml_diff>
--- a/data/monetary-rules-dashboard-data.xlsx
+++ b/data/monetary-rules-dashboard-data.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rac880583f4c84640"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Rules" sheetId="2" r:id="R4733a24713e3453f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Series" sheetId="3" r:id="R39fb2bba594e494b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Data Vintages" sheetId="4" r:id="R08ff6aacfaf04e18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="5" r:id="Radee14c6b0da4541"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="6" r:id="Rc509c566859f4ccb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3cdaa21a21c94473"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Rules" sheetId="2" r:id="R214a057b354a4f3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Series" sheetId="3" r:id="R31a467447d2c4ac6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Data Vintages" sheetId="4" r:id="Read295f13e484276"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="5" r:id="Re190b1deed114eeb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="6" r:id="R3300d22afde2489a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -630,7 +630,7 @@
         <x:v>Effective FFR</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
-        <x:v>3.63</x:v>
+        <x:v>3.88</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -664,7 +664,7 @@
       </x:c>
       <x:c r="B9" s="26" t="n">
         <x:f>MEDIAN('Current Rules'!D2:D13)</x:f>
-        <x:v>4.470761793199724</x:v>
+        <x:v>4.335780528653885</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -673,7 +673,7 @@
       </x:c>
       <x:c r="B10" s="26" t="n">
         <x:f>MAX('Current Rules'!D2:D13)</x:f>
-        <x:v>6.157732147628201</x:v>
+        <x:v>5.660416666666666</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -731,7 +731,7 @@
         <x:v>Dashboard generated at</x:v>
       </x:c>
       <x:c r="B17" s="30" t="n">
-        <x:v>46282.10877106481</x:v>
+        <x:v>46302.629387141205</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -794,18 +794,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D2" s="52" t="n">
-        <x:v>6.157732147628201</x:v>
+        <x:v>5.617807089444845</x:v>
       </x:c>
       <x:c r="E2" s="52" t="n">
         <x:v>6.011806193233087</x:v>
       </x:c>
       <x:c r="F2" s="53" t="n">
         <x:f>IF(E2="","",D2-E2)</x:f>
-        <x:v>0.14592595439511413</x:v>
+        <x:v>-0.393999103788242</x:v>
       </x:c>
       <x:c r="G2" s="53" t="n">
         <x:f>D2-'Summary'!$B$5</x:f>
-        <x:v>2.5277321476282015</x:v>
+        <x:v>1.7378070894448454</x:v>
       </x:c>
       <x:c r="H2" s="54" t="str">
         <x:f>IF(D2&gt;'Summary'!$B$7,"Above range",IF(D2&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -823,18 +823,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D3" s="57" t="n">
-        <x:v>5.978880506132231</x:v>
+        <x:v>5.438955447948875</x:v>
       </x:c>
       <x:c r="E3" s="57" t="n">
         <x:v>5.944152809026209</x:v>
       </x:c>
       <x:c r="F3" s="58" t="n">
         <x:f>IF(E3="","",D3-E3)</x:f>
-        <x:v>0.03472769710602286</x:v>
+        <x:v>-0.5051973610773333</x:v>
       </x:c>
       <x:c r="G3" s="58" t="n">
         <x:f>D3-'Summary'!$B$5</x:f>
-        <x:v>2.3488805061322315</x:v>
+        <x:v>1.5589554479488754</x:v>
       </x:c>
       <x:c r="H3" s="59" t="str">
         <x:f>IF(D3&gt;'Summary'!$B$7,"Above range",IF(D3&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -863,7 +863,7 @@
       </x:c>
       <x:c r="G4" s="58" t="n">
         <x:f>D4-'Summary'!$B$5</x:f>
-        <x:v>0.4556533348751586</x:v>
+        <x:v>0.20565333487515858</x:v>
       </x:c>
       <x:c r="H4" s="59" t="str">
         <x:f>IF(D4&gt;'Summary'!$B$7,"Above range",IF(D4&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -892,7 +892,7 @@
       </x:c>
       <x:c r="G5" s="58" t="n">
         <x:f>D5-'Summary'!$B$5</x:f>
-        <x:v>0.2768016933791886</x:v>
+        <x:v>0.026801693379188585</x:v>
       </x:c>
       <x:c r="H5" s="59" t="str">
         <x:f>IF(D5&gt;'Summary'!$B$7,"Above range",IF(D5&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -910,18 +910,18 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D6" s="57" t="n">
-        <x:v>4.895532740480768</x:v>
+        <x:v>4.625570211389089</x:v>
       </x:c>
       <x:c r="E6" s="57" t="n">
         <x:v>4.825903096616543</x:v>
       </x:c>
       <x:c r="F6" s="58" t="n">
         <x:f>IF(E6="","",D6-E6)</x:f>
-        <x:v>0.06962964386422499</x:v>
+        <x:v>-0.20033288522745352</x:v>
       </x:c>
       <x:c r="G6" s="58" t="n">
         <x:f>D6-'Summary'!$B$5</x:f>
-        <x:v>1.2655327404807677</x:v>
+        <x:v>0.7455702113890892</x:v>
       </x:c>
       <x:c r="H6" s="59" t="str">
         <x:f>IF(D6&gt;'Summary'!$B$7,"Above range",IF(D6&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -939,18 +939,18 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D7" s="57" t="n">
-        <x:v>4.806106919732782</x:v>
+        <x:v>4.536144390641104</x:v>
       </x:c>
       <x:c r="E7" s="57" t="n">
         <x:v>4.792076404513105</x:v>
       </x:c>
       <x:c r="F7" s="58" t="n">
         <x:f>IF(E7="","",D7-E7)</x:f>
-        <x:v>0.014030515219677575</x:v>
+        <x:v>-0.25593201387200093</x:v>
       </x:c>
       <x:c r="G7" s="58" t="n">
         <x:f>D7-'Summary'!$B$5</x:f>
-        <x:v>1.1761069197327823</x:v>
+        <x:v>0.6561443906411037</x:v>
       </x:c>
       <x:c r="H7" s="59" t="str">
         <x:f>IF(D7&gt;'Summary'!$B$7,"Above range",IF(D7&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -979,7 +979,7 @@
       </x:c>
       <x:c r="G8" s="58" t="n">
         <x:f>D8-'Summary'!$B$5</x:f>
-        <x:v>0.22949333410424577</x:v>
+        <x:v>-0.020506665895754228</x:v>
       </x:c>
       <x:c r="H8" s="59" t="str">
         <x:f>IF(D8&gt;'Summary'!$B$7,"Above range",IF(D8&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -1008,7 +1008,7 @@
       </x:c>
       <x:c r="G9" s="58" t="n">
         <x:f>D9-'Summary'!$B$5</x:f>
-        <x:v>0.14006751335626078</x:v>
+        <x:v>-0.10993248664373922</x:v>
       </x:c>
       <x:c r="H9" s="59" t="str">
         <x:f>IF(D9&gt;'Summary'!$B$7,"Above range",IF(D9&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -1026,14 +1026,14 @@
         <x:v>SEP</x:v>
       </x:c>
       <x:c r="D10" s="57" t="n">
-        <x:v>5.410416666666666</x:v>
+        <x:v>5.660416666666666</x:v>
       </x:c>
       <x:c r="E10" s="57" t="n">
         <x:v>4.282500000000001</x:v>
       </x:c>
       <x:c r="F10" s="58" t="n">
         <x:f>IF(E10="","",D10-E10)</x:f>
-        <x:v>1.1279166666666658</x:v>
+        <x:v>1.3779166666666658</x:v>
       </x:c>
       <x:c r="G10" s="58" t="n">
         <x:f>D10-'Summary'!$B$5</x:f>
@@ -1055,14 +1055,14 @@
         <x:v>HLW</x:v>
       </x:c>
       <x:c r="D11" s="57" t="n">
-        <x:v>5.320990845918681</x:v>
+        <x:v>5.570990845918681</x:v>
       </x:c>
       <x:c r="E11" s="57" t="n">
         <x:v>4.24867330789656</x:v>
       </x:c>
       <x:c r="F11" s="58" t="n">
         <x:f>IF(E11="","",D11-E11)</x:f>
-        <x:v>1.072317538022121</x:v>
+        <x:v>1.322317538022121</x:v>
       </x:c>
       <x:c r="G11" s="58" t="n">
         <x:f>D11-'Summary'!$B$5</x:f>
@@ -1095,7 +1095,7 @@
       </x:c>
       <x:c r="G12" s="58" t="n">
         <x:f>D12-'Summary'!$B$5</x:f>
-        <x:v>0.5054166666666662</x:v>
+        <x:v>0.2554166666666662</x:v>
       </x:c>
       <x:c r="H12" s="59" t="str">
         <x:f>IF(D12&gt;'Summary'!$B$7,"Above range",IF(D12&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -1124,7 +1124,7 @@
       </x:c>
       <x:c r="G13" s="63" t="n">
         <x:f>D13-'Summary'!$B$5</x:f>
-        <x:v>0.41599084591868163</x:v>
+        <x:v>0.16599084591868163</x:v>
       </x:c>
       <x:c r="H13" s="64" t="str">
         <x:f>IF(D13&gt;'Summary'!$B$7,"Above range",IF(D13&lt;'Summary'!$B$6,"Below range","Within range"))</x:f>
@@ -2126,7 +2126,7 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E38" s="26" t="n">
-        <x:v>1.7162918476874465</x:v>
+        <x:v>1.6315582558448565</x:v>
       </x:c>
       <x:c r="F38" s="26" t="n">
         <x:v>0.8960614748901637</x:v>
@@ -2152,7 +2152,7 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E39" s="26" t="n">
-        <x:v>5.045586071499688</x:v>
+        <x:v>4.918683738227261</x:v>
       </x:c>
       <x:c r="F39" s="26" t="n">
         <x:v>1.38030237245958</x:v>
@@ -2178,7 +2178,7 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E40" s="26" t="n">
-        <x:v>6.74996734674795</x:v>
+        <x:v>6.62834765866664</x:v>
       </x:c>
       <x:c r="F40" s="26" t="n">
         <x:v>2.0335239340156535</x:v>
@@ -2204,7 +2204,7 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E41" s="26" t="n">
-        <x:v>9.713291778112792</x:v>
+        <x:v>9.605100564378207</x:v>
       </x:c>
       <x:c r="F41" s="26" t="n">
         <x:v>2.7431258506585703</x:v>
@@ -2230,7 +2230,7 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E42" s="26" t="n">
-        <x:v>10.901871683198607</x:v>
+        <x:v>10.862274377082683</x:v>
       </x:c>
       <x:c r="F42" s="26" t="n">
         <x:v>2.949254367420406</x:v>
@@ -2256,7 +2256,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E43" s="26" t="n">
-        <x:v>11.39809497156169</x:v>
+        <x:v>11.356575722204411</x:v>
       </x:c>
       <x:c r="F43" s="26" t="n">
         <x:v>3.486442368448991</x:v>
@@ -2282,7 +2282,7 @@
         <x:v>2.5</x:v>
       </x:c>
       <x:c r="E44" s="26" t="n">
-        <x:v>11.251829881421084</x:v>
+        <x:v>11.340379694245764</x:v>
       </x:c>
       <x:c r="F44" s="26" t="n">
         <x:v>3.7475252877182665</x:v>
@@ -2308,7 +2308,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E45" s="26" t="n">
-        <x:v>10.127860951471467</x:v>
+        <x:v>10.221519420164947</x:v>
       </x:c>
       <x:c r="F45" s="26" t="n">
         <x:v>4.328816825633722</x:v>
@@ -2334,7 +2334,7 @@
         <x:v>4.75</x:v>
       </x:c>
       <x:c r="E46" s="26" t="n">
-        <x:v>8.673434439310375</x:v>
+        <x:v>8.729722042066653</x:v>
       </x:c>
       <x:c r="F46" s="26" t="n">
         <x:v>4.519669048014301</x:v>
@@ -2360,7 +2360,7 @@
         <x:v>5.25</x:v>
       </x:c>
       <x:c r="E47" s="26" t="n">
-        <x:v>6.868500986055668</x:v>
+        <x:v>6.972183292174249</x:v>
       </x:c>
       <x:c r="F47" s="26" t="n">
         <x:v>4.965932726586612</x:v>
@@ -2386,7 +2386,7 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="E48" s="26" t="n">
-        <x:v>5.976601206932669</x:v>
+        <x:v>5.977745039651977</x:v>
       </x:c>
       <x:c r="F48" s="26" t="n">
         <x:v>4.877381726990993</x:v>
@@ -2412,7 +2412,7 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="E49" s="26" t="n">
-        <x:v>4.841622486590254</x:v>
+        <x:v>4.989272405779983</x:v>
       </x:c>
       <x:c r="F49" s="26" t="n">
         <x:v>4.81686722513419</x:v>
@@ -2438,7 +2438,7 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="E50" s="26" t="n">
-        <x:v>4.685985663378069</x:v>
+        <x:v>4.773368380492905</x:v>
       </x:c>
       <x:c r="F50" s="26" t="n">
         <x:v>4.47906659358176</x:v>
@@ -2464,7 +2464,7 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="E51" s="26" t="n">
-        <x:v>4.409681751822772</x:v>
+        <x:v>4.445030650762808</x:v>
       </x:c>
       <x:c r="F51" s="26" t="n">
         <x:v>4.7188083127989735</x:v>
@@ -2490,7 +2490,7 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="E52" s="26" t="n">
-        <x:v>3.799914006669143</x:v>
+        <x:v>3.8118544481617294</x:v>
       </x:c>
       <x:c r="F52" s="26" t="n">
         <x:v>4.360702964050825</x:v>
@@ -2516,7 +2516,7 @@
         <x:v>4.75</x:v>
       </x:c>
       <x:c r="E53" s="26" t="n">
-        <x:v>4.046029978711584</x:v>
+        <x:v>3.923062753941574</x:v>
       </x:c>
       <x:c r="F53" s="26" t="n">
         <x:v>4.296630975510824</x:v>
@@ -2542,7 +2542,7 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="E54" s="26" t="n">
-        <x:v>3.906071783997163</x:v>
+        <x:v>3.7991908178837432</x:v>
       </x:c>
       <x:c r="F54" s="26" t="n">
         <x:v>4.1612008416044715</x:v>
@@ -2568,7 +2568,7 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="E55" s="26" t="n">
-        <x:v>3.776447523581173</x:v>
+        <x:v>3.8160029237354633</x:v>
       </x:c>
       <x:c r="F55" s="26" t="n">
         <x:v>4.517525064766964</x:v>
@@ -2594,7 +2594,7 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="E56" s="26" t="n">
-        <x:v>4.193984641190231</x:v>
+        <x:v>4.157016748643552</x:v>
       </x:c>
       <x:c r="F56" s="26" t="n">
         <x:v>4.2872203668213</x:v>
@@ -2620,7 +2620,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E57" s="26" t="n">
-        <x:v>4.046316682399642</x:v>
+        <x:v>3.9125381772546204</x:v>
       </x:c>
       <x:c r="F57" s="26" t="n">
         <x:v>4.0933951900396925</x:v>
@@ -2646,7 +2646,7 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="E58" s="26" t="n">
-        <x:v>4.8043430978133745</x:v>
+        <x:v>4.606507067143191</x:v>
       </x:c>
       <x:c r="F58" s="26" t="n">
         <x:v>4.025660450701153</x:v>
@@ -2672,7 +2672,7 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="E59" s="26" t="n">
-        <x:v>5.951937712846006</x:v>
+        <x:v>5.5611555691172</x:v>
       </x:c>
       <x:c r="F59" s="26" t="n">
         <x:v>4.210939293053199</x:v>
@@ -2689,7 +2689,7 @@
         <x:v>46249.5</x:v>
       </x:c>
       <x:c r="B60" s="70" t="n">
-        <x:v>3.63</x:v>
+        <x:v>3.88</x:v>
       </x:c>
       <x:c r="C60" s="70" t="n">
         <x:v>3.75</x:v>
@@ -2698,13 +2698,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E60" s="70" t="n">
-        <x:v>5.978880506132231</x:v>
+        <x:v>5.438955447948875</x:v>
       </x:c>
       <x:c r="F60" s="70" t="n">
         <x:v>3.7700675133562607</x:v>
       </x:c>
       <x:c r="G60" s="70" t="n">
-        <x:v>5.320990845918681</x:v>
+        <x:v>5.570990845918681</x:v>
       </x:c>
       <x:c r="H60" s="70" t="n">
         <x:v>4.0459908459186815</x:v>
@@ -4601,10 +4601,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E38" s="57" t="n">
-        <x:v>0.7672036478529263</x:v>
+        <x:v>0.6824700560103363</x:v>
       </x:c>
       <x:c r="F38" s="57" t="n">
-        <x:v>1.7162918476874465</x:v>
+        <x:v>1.6315582558448565</x:v>
       </x:c>
       <x:c r="G38" s="57" t="n">
         <x:v>0.7530347499458072</x:v>
@@ -4613,10 +4613,10 @@
         <x:v>1.7021229497803274</x:v>
       </x:c>
       <x:c r="I38" s="57" t="n">
-        <x:v>0.4286018239264631</x:v>
+        <x:v>0.3862350280051681</x:v>
       </x:c>
       <x:c r="J38" s="57" t="n">
-        <x:v>0.9031459238437233</x:v>
+        <x:v>0.8607791279224283</x:v>
       </x:c>
       <x:c r="K38" s="57" t="n">
         <x:v>0.4215173749729036</x:v>
@@ -4651,10 +4651,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E39" s="57" t="n">
-        <x:v>4.025780561510787</x:v>
+        <x:v>3.8988782282383614</x:v>
       </x:c>
       <x:c r="F39" s="57" t="n">
-        <x:v>5.045586071499688</x:v>
+        <x:v>4.918683738227261</x:v>
       </x:c>
       <x:c r="G39" s="57" t="n">
         <x:v>1.66079923493026</x:v>
@@ -4663,10 +4663,10 @@
         <x:v>2.68060474491916</x:v>
       </x:c>
       <x:c r="I39" s="57" t="n">
-        <x:v>2.0528902807553937</x:v>
+        <x:v>1.9894391141191807</x:v>
       </x:c>
       <x:c r="J39" s="57" t="n">
-        <x:v>2.562793035749844</x:v>
+        <x:v>2.4993418691136307</x:v>
       </x:c>
       <x:c r="K39" s="57" t="n">
         <x:v>0.8703996174651301</x:v>
@@ -4701,10 +4701,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E40" s="57" t="n">
-        <x:v>5.776885057471289</x:v>
+        <x:v>5.655265369389981</x:v>
       </x:c>
       <x:c r="F40" s="57" t="n">
-        <x:v>6.74996734674795</x:v>
+        <x:v>6.62834765866664</x:v>
       </x:c>
       <x:c r="G40" s="57" t="n">
         <x:v>3.0239655787546464</x:v>
@@ -4713,10 +4713,10 @@
         <x:v>3.9970478680313066</x:v>
       </x:c>
       <x:c r="I40" s="57" t="n">
-        <x:v>2.9234425287356447</x:v>
+        <x:v>2.8626326846949905</x:v>
       </x:c>
       <x:c r="J40" s="57" t="n">
-        <x:v>3.4099836733739752</x:v>
+        <x:v>3.34917382933332</x:v>
       </x:c>
       <x:c r="K40" s="57" t="n">
         <x:v>1.5469827893773231</x:v>
@@ -4751,10 +4751,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E41" s="57" t="n">
-        <x:v>8.482455333162513</x:v>
+        <x:v>8.374264119427925</x:v>
       </x:c>
       <x:c r="F41" s="57" t="n">
-        <x:v>9.713291778112792</x:v>
+        <x:v>9.605100564378207</x:v>
       </x:c>
       <x:c r="G41" s="57" t="n">
         <x:v>4.1654152563668605</x:v>
@@ -4763,10 +4763,10 @@
         <x:v>5.396251701317141</x:v>
       </x:c>
       <x:c r="I41" s="57" t="n">
-        <x:v>4.286227666581256</x:v>
+        <x:v>4.232132059713963</x:v>
       </x:c>
       <x:c r="J41" s="57" t="n">
-        <x:v>4.901645889056396</x:v>
+        <x:v>4.847550282189103</x:v>
       </x:c>
       <x:c r="K41" s="57" t="n">
         <x:v>2.12770762818343</x:v>
@@ -4801,10 +4801,10 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="E42" s="57" t="n">
-        <x:v>9.866069834001152</x:v>
+        <x:v>9.82647252788523</x:v>
       </x:c>
       <x:c r="F42" s="57" t="n">
-        <x:v>10.901871683198607</x:v>
+        <x:v>10.862274377082683</x:v>
       </x:c>
       <x:c r="G42" s="57" t="n">
         <x:v>4.782706885643359</x:v>
@@ -4813,10 +4813,10 @@
         <x:v>5.818508734840812</x:v>
       </x:c>
       <x:c r="I42" s="57" t="n">
-        <x:v>4.973034917000576</x:v>
+        <x:v>4.953236263942615</x:v>
       </x:c>
       <x:c r="J42" s="57" t="n">
-        <x:v>5.4909358415993035</x:v>
+        <x:v>5.471137188541341</x:v>
       </x:c>
       <x:c r="K42" s="57" t="n">
         <x:v>2.4313534428216794</x:v>
@@ -4851,10 +4851,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E43" s="57" t="n">
-        <x:v>10.627900244028694</x:v>
+        <x:v>10.586380994671414</x:v>
       </x:c>
       <x:c r="F43" s="57" t="n">
-        <x:v>11.39809497156169</x:v>
+        <x:v>11.356575722204411</x:v>
       </x:c>
       <x:c r="G43" s="57" t="n">
         <x:v>6.082690009364985</x:v>
@@ -4863,10 +4863,10 @@
         <x:v>6.852884736897982</x:v>
       </x:c>
       <x:c r="I43" s="57" t="n">
-        <x:v>5.373950122014347</x:v>
+        <x:v>5.3531904973357065</x:v>
       </x:c>
       <x:c r="J43" s="57" t="n">
-        <x:v>5.759047485780845</x:v>
+        <x:v>5.738287861102205</x:v>
       </x:c>
       <x:c r="K43" s="57" t="n">
         <x:v>3.1013450046824924</x:v>
@@ -4901,10 +4901,10 @@
         <x:v>2.5</x:v>
       </x:c>
       <x:c r="E44" s="57" t="n">
-        <x:v>10.433937151368685</x:v>
+        <x:v>10.522486964193364</x:v>
       </x:c>
       <x:c r="F44" s="57" t="n">
-        <x:v>11.251829881421084</x:v>
+        <x:v>11.340379694245764</x:v>
       </x:c>
       <x:c r="G44" s="57" t="n">
         <x:v>5.907157845384132</x:v>
@@ -4913,10 +4913,10 @@
         <x:v>6.725050575436533</x:v>
       </x:c>
       <x:c r="I44" s="57" t="n">
-        <x:v>5.601968575684342</x:v>
+        <x:v>5.646243482096682</x:v>
       </x:c>
       <x:c r="J44" s="57" t="n">
-        <x:v>6.010914940710542</x:v>
+        <x:v>6.0551898471228816</x:v>
       </x:c>
       <x:c r="K44" s="57" t="n">
         <x:v>3.338578922692066</x:v>
@@ -4951,10 +4951,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E45" s="57" t="n">
-        <x:v>9.374315967612707</x:v>
+        <x:v>9.467974436306188</x:v>
       </x:c>
       <x:c r="F45" s="57" t="n">
-        <x:v>10.127860951471467</x:v>
+        <x:v>10.221519420164947</x:v>
       </x:c>
       <x:c r="G45" s="57" t="n">
         <x:v>5.714088667408684</x:v>
@@ -4963,10 +4963,10 @@
         <x:v>6.467633651267445</x:v>
       </x:c>
       <x:c r="I45" s="57" t="n">
-        <x:v>5.7821579838063535</x:v>
+        <x:v>5.8289872181530935</x:v>
       </x:c>
       <x:c r="J45" s="57" t="n">
-        <x:v>6.158930475735733</x:v>
+        <x:v>6.205759710082473</x:v>
       </x:c>
       <x:c r="K45" s="57" t="n">
         <x:v>3.9520443337043423</x:v>
@@ -5001,10 +5001,10 @@
         <x:v>4.75</x:v>
       </x:c>
       <x:c r="E46" s="57" t="n">
-        <x:v>7.963604297629344</x:v>
+        <x:v>8.019891900385623</x:v>
       </x:c>
       <x:c r="F46" s="57" t="n">
-        <x:v>8.673434439310375</x:v>
+        <x:v>8.729722042066653</x:v>
       </x:c>
       <x:c r="G46" s="57" t="n">
         <x:v>4.67617462101424</x:v>
@@ -5013,10 +5013,10 @@
         <x:v>5.386004762695269</x:v>
       </x:c>
       <x:c r="I46" s="57" t="n">
-        <x:v>5.808468815481339</x:v>
+        <x:v>5.836612616859478</x:v>
       </x:c>
       <x:c r="J46" s="57" t="n">
-        <x:v>6.163383886321854</x:v>
+        <x:v>6.191527687699993</x:v>
       </x:c>
       <x:c r="K46" s="57" t="n">
         <x:v>4.1647539771737865</x:v>
@@ -5051,10 +5051,10 @@
         <x:v>5.25</x:v>
       </x:c>
       <x:c r="E47" s="57" t="n">
-        <x:v>6.277340498135288</x:v>
+        <x:v>6.381022804253869</x:v>
       </x:c>
       <x:c r="F47" s="57" t="n">
-        <x:v>6.868500986055668</x:v>
+        <x:v>6.972183292174249</x:v>
       </x:c>
       <x:c r="G47" s="57" t="n">
         <x:v>4.824038298586177</x:v>
@@ -5063,10 +5063,10 @@
         <x:v>5.415198786506557</x:v>
       </x:c>
       <x:c r="I47" s="57" t="n">
-        <x:v>5.397003582400977</x:v>
+        <x:v>5.448844735460268</x:v>
       </x:c>
       <x:c r="J47" s="57" t="n">
-        <x:v>5.692583826361167</x:v>
+        <x:v>5.744424979420458</x:v>
       </x:c>
       <x:c r="K47" s="57" t="n">
         <x:v>4.670352482626422</x:v>
@@ -5101,10 +5101,10 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="E48" s="57" t="n">
-        <x:v>5.44315416089675</x:v>
+        <x:v>5.444297993616058</x:v>
       </x:c>
       <x:c r="F48" s="57" t="n">
-        <x:v>5.976601206932669</x:v>
+        <x:v>5.977745039651977</x:v>
       </x:c>
       <x:c r="G48" s="57" t="n">
         <x:v>4.231316407946066</x:v>
@@ -5113,10 +5113,10 @@
         <x:v>4.764763453981986</x:v>
       </x:c>
       <x:c r="I48" s="57" t="n">
-        <x:v>5.216577080448375</x:v>
+        <x:v>5.217148996808029</x:v>
       </x:c>
       <x:c r="J48" s="57" t="n">
-        <x:v>5.4833006034663345</x:v>
+        <x:v>5.483872519825988</x:v>
       </x:c>
       <x:c r="K48" s="57" t="n">
         <x:v>4.610658203973033</x:v>
@@ -5151,10 +5151,10 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="E49" s="57" t="n">
-        <x:v>4.405518277822901</x:v>
+        <x:v>4.55316819701263</x:v>
       </x:c>
       <x:c r="F49" s="57" t="n">
-        <x:v>4.841622486590254</x:v>
+        <x:v>4.989272405779983</x:v>
       </x:c>
       <x:c r="G49" s="57" t="n">
         <x:v>3.937630241501027</x:v>
@@ -5163,10 +5163,10 @@
         <x:v>4.37373445026838</x:v>
       </x:c>
       <x:c r="I49" s="57" t="n">
-        <x:v>4.832759138911451</x:v>
+        <x:v>4.906584098506315</x:v>
       </x:c>
       <x:c r="J49" s="57" t="n">
-        <x:v>5.0508112432951275</x:v>
+        <x:v>5.124636202889992</x:v>
       </x:c>
       <x:c r="K49" s="57" t="n">
         <x:v>4.598815120750514</x:v>
@@ -5201,10 +5201,10 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="E50" s="57" t="n">
-        <x:v>4.2998603055397195</x:v>
+        <x:v>4.387243022654555</x:v>
       </x:c>
       <x:c r="F50" s="57" t="n">
-        <x:v>4.685985663378069</x:v>
+        <x:v>4.773368380492905</x:v>
       </x:c>
       <x:c r="G50" s="57" t="n">
         <x:v>3.24200782932517</x:v>
@@ -5213,10 +5213,10 @@
         <x:v>3.62813318716352</x:v>
       </x:c>
       <x:c r="I50" s="57" t="n">
-        <x:v>4.814930152769859</x:v>
+        <x:v>4.858621511327278</x:v>
       </x:c>
       <x:c r="J50" s="57" t="n">
-        <x:v>5.007992831689035</x:v>
+        <x:v>5.051684190246453</x:v>
       </x:c>
       <x:c r="K50" s="57" t="n">
         <x:v>4.286003914662585</x:v>
@@ -5251,10 +5251,10 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="E51" s="57" t="n">
-        <x:v>4.160222467204729</x:v>
+        <x:v>4.195571366144765</x:v>
       </x:c>
       <x:c r="F51" s="57" t="n">
-        <x:v>4.409681751822772</x:v>
+        <x:v>4.445030650762808</x:v>
       </x:c>
       <x:c r="G51" s="57" t="n">
         <x:v>3.8581573409799033</x:v>
@@ -5263,10 +5263,10 @@
         <x:v>4.107616625597946</x:v>
       </x:c>
       <x:c r="I51" s="57" t="n">
-        <x:v>4.745111233602365</x:v>
+        <x:v>4.762785683072383</x:v>
       </x:c>
       <x:c r="J51" s="57" t="n">
-        <x:v>4.869840875911386</x:v>
+        <x:v>4.887515325381404</x:v>
       </x:c>
       <x:c r="K51" s="57" t="n">
         <x:v>4.594078670489951</x:v>
@@ -5301,10 +5301,10 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="E52" s="57" t="n">
-        <x:v>3.718167769981595</x:v>
+        <x:v>3.7301082114741817</x:v>
       </x:c>
       <x:c r="F52" s="57" t="n">
-        <x:v>3.799914006669143</x:v>
+        <x:v>3.8118544481617294</x:v>
       </x:c>
       <x:c r="G52" s="57" t="n">
         <x:v>3.3096596914141028</x:v>
@@ -5313,10 +5313,10 @@
         <x:v>3.3914059281016504</x:v>
       </x:c>
       <x:c r="I52" s="57" t="n">
-        <x:v>4.524083884990798</x:v>
+        <x:v>4.530054105737091</x:v>
       </x:c>
       <x:c r="J52" s="57" t="n">
-        <x:v>4.564957003334571</x:v>
+        <x:v>4.570927224080865</x:v>
       </x:c>
       <x:c r="K52" s="57" t="n">
         <x:v>4.319829845707051</x:v>
@@ -5351,10 +5351,10 @@
         <x:v>4.75</x:v>
       </x:c>
       <x:c r="E53" s="57" t="n">
-        <x:v>4.134055814259625</x:v>
+        <x:v>4.011088589489615</x:v>
       </x:c>
       <x:c r="F53" s="57" t="n">
-        <x:v>4.046029978711584</x:v>
+        <x:v>3.923062753941574</x:v>
       </x:c>
       <x:c r="G53" s="57" t="n">
         <x:v>3.417954453236356</x:v>
@@ -5363,10 +5363,10 @@
         <x:v>3.3299286176883145</x:v>
       </x:c>
       <x:c r="I53" s="57" t="n">
-        <x:v>4.6986945737964785</x:v>
+        <x:v>4.6372109614114745</x:v>
       </x:c>
       <x:c r="J53" s="57" t="n">
-        <x:v>4.654681656022458</x:v>
+        <x:v>4.593198043637454</x:v>
       </x:c>
       <x:c r="K53" s="57" t="n">
         <x:v>4.340643893284844</x:v>
@@ -5401,10 +5401,10 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="E54" s="57" t="n">
-        <x:v>4.113069416581042</x:v>
+        <x:v>4.006188450467622</x:v>
       </x:c>
       <x:c r="F54" s="57" t="n">
-        <x:v>3.906071783997163</x:v>
+        <x:v>3.7991908178837432</x:v>
       </x:c>
       <x:c r="G54" s="57" t="n">
         <x:v>3.8793993157928237</x:v>
@@ -5413,10 +5413,10 @@
         <x:v>3.672401683208945</x:v>
       </x:c>
       <x:c r="I54" s="57" t="n">
-        <x:v>4.38153470829052</x:v>
+        <x:v>4.32809422523381</x:v>
       </x:c>
       <x:c r="J54" s="57" t="n">
-        <x:v>4.278035891998581</x:v>
+        <x:v>4.224595408941871</x:v>
       </x:c>
       <x:c r="K54" s="57" t="n">
         <x:v>4.264699657896411</x:v>
@@ -5451,10 +5451,10 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="E55" s="57" t="n">
-        <x:v>3.8706435835311903</x:v>
+        <x:v>3.910198983685481</x:v>
       </x:c>
       <x:c r="F55" s="57" t="n">
-        <x:v>3.776447523581173</x:v>
+        <x:v>3.8160029237354633</x:v>
       </x:c>
       <x:c r="G55" s="57" t="n">
         <x:v>4.799246189483946</x:v>
@@ -5463,10 +5463,10 @@
         <x:v>4.705050129533929</x:v>
       </x:c>
       <x:c r="I55" s="57" t="n">
-        <x:v>4.100321791765595</x:v>
+        <x:v>4.1200994918427405</x:v>
       </x:c>
       <x:c r="J55" s="57" t="n">
-        <x:v>4.053223761790587</x:v>
+        <x:v>4.073001461867731</x:v>
       </x:c>
       <x:c r="K55" s="57" t="n">
         <x:v>4.5646230947419735</x:v>
@@ -5501,10 +5501,10 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="E56" s="57" t="n">
-        <x:v>4.141109658678292</x:v>
+        <x:v>4.104141766131613</x:v>
       </x:c>
       <x:c r="F56" s="57" t="n">
-        <x:v>4.193984641190231</x:v>
+        <x:v>4.157016748643552</x:v>
       </x:c>
       <x:c r="G56" s="57" t="n">
         <x:v>4.191565751130659</x:v>
@@ -5513,10 +5513,10 @@
         <x:v>4.244440733642599</x:v>
       </x:c>
       <x:c r="I56" s="57" t="n">
-        <x:v>4.235554829339145</x:v>
+        <x:v>4.217070883065807</x:v>
       </x:c>
       <x:c r="J56" s="57" t="n">
-        <x:v>4.261992320595116</x:v>
+        <x:v>4.243508374321776</x:v>
       </x:c>
       <x:c r="K56" s="57" t="n">
         <x:v>4.260782875565329</x:v>
@@ -5551,10 +5551,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E57" s="57" t="n">
-        <x:v>4.157394393077939</x:v>
+        <x:v>4.023615887932917</x:v>
       </x:c>
       <x:c r="F57" s="57" t="n">
-        <x:v>4.046316682399642</x:v>
+        <x:v>3.9125381772546204</x:v>
       </x:c>
       <x:c r="G57" s="57" t="n">
         <x:v>4.004534757424349</x:v>
@@ -5563,10 +5563,10 @@
         <x:v>3.893457046746052</x:v>
       </x:c>
       <x:c r="I57" s="57" t="n">
-        <x:v>4.2253638632056365</x:v>
+        <x:v>4.1584746106331245</x:v>
       </x:c>
       <x:c r="J57" s="57" t="n">
-        <x:v>4.169825007866487</x:v>
+        <x:v>4.102935755293977</x:v>
       </x:c>
       <x:c r="K57" s="57" t="n">
         <x:v>4.148934045378841</x:v>
@@ -5601,10 +5601,10 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="E58" s="57" t="n">
-        <x:v>4.795983516090297</x:v>
+        <x:v>4.598147485420114</x:v>
       </x:c>
       <x:c r="F58" s="57" t="n">
-        <x:v>4.8043430978133745</x:v>
+        <x:v>4.606507067143191</x:v>
       </x:c>
       <x:c r="G58" s="57" t="n">
         <x:v>4.146294653012562</x:v>
@@ -5613,10 +5613,10 @@
         <x:v>4.15465423473564</x:v>
       </x:c>
       <x:c r="I58" s="57" t="n">
-        <x:v>4.346325091378482</x:v>
+        <x:v>4.24740707604339</x:v>
       </x:c>
       <x:c r="J58" s="57" t="n">
-        <x:v>4.3505048822400205</x:v>
+        <x:v>4.251586866904929</x:v>
       </x:c>
       <x:c r="K58" s="57" t="n">
         <x:v>4.0214806598396144</x:v>
@@ -5651,10 +5651,10 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="E59" s="57" t="n">
-        <x:v>6.026622687675309</x:v>
+        <x:v>5.635840543946503</x:v>
       </x:c>
       <x:c r="F59" s="57" t="n">
-        <x:v>5.951937712846006</x:v>
+        <x:v>5.5611555691172</x:v>
       </x:c>
       <x:c r="G59" s="57" t="n">
         <x:v>4.856563560935701</x:v>
@@ -5663,10 +5663,10 @@
         <x:v>4.781878586106398</x:v>
       </x:c>
       <x:c r="I59" s="57" t="n">
-        <x:v>4.8333113438376545</x:v>
+        <x:v>4.637920271973251</x:v>
       </x:c>
       <x:c r="J59" s="57" t="n">
-        <x:v>4.795968856423003</x:v>
+        <x:v>4.6005777845586</x:v>
       </x:c>
       <x:c r="K59" s="57" t="n">
         <x:v>4.248281780467851</x:v>
@@ -5692,7 +5692,7 @@
         <x:v>46249.5</x:v>
       </x:c>
       <x:c r="B60" s="62" t="n">
-        <x:v>3.63</x:v>
+        <x:v>3.88</x:v>
       </x:c>
       <x:c r="C60" s="62" t="n">
         <x:v>3.75</x:v>
@@ -5701,10 +5701,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E60" s="62" t="n">
-        <x:v>6.157732147628201</x:v>
+        <x:v>5.617807089444845</x:v>
       </x:c>
       <x:c r="F60" s="62" t="n">
-        <x:v>5.978880506132231</x:v>
+        <x:v>5.438955447948875</x:v>
       </x:c>
       <x:c r="G60" s="62" t="n">
         <x:v>4.0856533348751585</x:v>
@@ -5713,10 +5713,10 @@
         <x:v>3.9068016933791885</x:v>
       </x:c>
       <x:c r="I60" s="62" t="n">
-        <x:v>4.895532740480768</x:v>
+        <x:v>4.625570211389089</x:v>
       </x:c>
       <x:c r="J60" s="62" t="n">
-        <x:v>4.806106919732782</x:v>
+        <x:v>4.536144390641104</x:v>
       </x:c>
       <x:c r="K60" s="62" t="n">
         <x:v>3.8594933341042457</x:v>
@@ -5725,10 +5725,10 @@
         <x:v>3.7700675133562607</x:v>
       </x:c>
       <x:c r="M60" s="62" t="n">
-        <x:v>5.410416666666666</x:v>
+        <x:v>5.660416666666666</x:v>
       </x:c>
       <x:c r="N60" s="62" t="n">
-        <x:v>5.320990845918681</x:v>
+        <x:v>5.570990845918681</x:v>
       </x:c>
       <x:c r="O60" s="62" t="n">
         <x:v>4.135416666666666</x:v>
@@ -5781,7 +5781,7 @@
         <x:v>effr</x:v>
       </x:c>
       <x:c r="D2" s="91" t="n">
-        <x:v>3.63</x:v>
+        <x:v>3.88</x:v>
       </x:c>
       <x:c r="E2" s="92" t="str">
         <x:v>Federal Reserve Bank of New York Effective FFR — https://www.newyorkfed.org/markets/reference-rates/effr</x:v>
@@ -5866,7 +5866,7 @@
         <x:v>pce</x:v>
       </x:c>
       <x:c r="D7" s="93" t="n">
-        <x:v>3.806334007929824</x:v>
+        <x:v>3.44638396914092</x:v>
       </x:c>
       <x:c r="E7" s="94" t="str">
         <x:v>Federal Reserve Bank of Atlanta Taylor Rule Utility — https://www.atlantafed.org/research-and-data/data/taylor-rule</x:v>
@@ -5951,7 +5951,7 @@
         <x:v>ngdp</x:v>
       </x:c>
       <x:c r="D12" s="93" t="n">
-        <x:v>8</x:v>
+        <x:v>8.5</x:v>
       </x:c>
       <x:c r="E12" s="94" t="str">
         <x:v>Bureau of Economic Analysis Nominal GDP — https://www.bea.gov/data/gdp/gross-domestic-product</x:v>
@@ -6045,7 +6045,7 @@
         <x:v>46280.5</x:v>
       </x:c>
       <x:c r="C2" s="99" t="n">
-        <x:v>46281.5</x:v>
+        <x:v>46302.5</x:v>
       </x:c>
       <x:c r="D2" s="54" t="str">
         <x:v>https://fedagenda.substack.com/p/monetary-rules-report-eef</x:v>
@@ -6059,7 +6059,7 @@
         <x:v>46234.5</x:v>
       </x:c>
       <x:c r="C3" s="100" t="n">
-        <x:v>46281.5</x:v>
+        <x:v>46302.5</x:v>
       </x:c>
       <x:c r="D3" s="64" t="str">
         <x:v>https://fedagenda.substack.com/p/monetary-neutrality-report-9d2</x:v>

</xml_diff>